<commit_message>
Auto commit - 09151757
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$91</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$115</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="728">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-11  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="872">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-15  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -2233,6 +2233,447 @@
   </si>
   <si>
     <t>2026-09-11 16:30:00</t>
+  </si>
+  <si>
+    <t>14541115091301</t>
+  </si>
+  <si>
+    <t>淡水海天店</t>
+  </si>
+  <si>
+    <t>新北市淡水區</t>
+  </si>
+  <si>
+    <t>2026-09-13 09:09:37</t>
+  </si>
+  <si>
+    <t>門市反應SC CCD掃描器(F460B)刷讀條碼無反應刷不出來有亮燈，門市不願協助操作校正請客服直接派工....需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04541</t>
+  </si>
+  <si>
+    <t>2026-09-13 09:10:51</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:12:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:42:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 13:00:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119005353
+換上8119014187</t>
+  </si>
+  <si>
+    <t>E2259115091401</t>
+  </si>
+  <si>
+    <t>三重興華店</t>
+  </si>
+  <si>
+    <t>2026-09-14 08:16:21</t>
+  </si>
+  <si>
+    <t>門市反應TM2(TCX800)半夜更後就無法開機無電源反應，請門市將電源插頭拔插休息仍無電源，與門市確認附近無其他插座可更換測試....需請台芝到店協助(大夜更新過後 機台就不開機了，能否換一台阿  這台超常故障)PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)與門市確認今日尚未清帳09/14有交易</t>
+  </si>
+  <si>
+    <t>THILF02259</t>
+  </si>
+  <si>
+    <t>2026-09-14 09:11:36</t>
+  </si>
+  <si>
+    <t>2026-09-14 11:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 12:08:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 13:11:00</t>
+  </si>
+  <si>
+    <t>變壓器鬆脫.  差好後即可正常開機</t>
+  </si>
+  <si>
+    <t>12482115091401</t>
+  </si>
+  <si>
+    <t>蘆竹光明店</t>
+  </si>
+  <si>
+    <t>2026-09-14 09:21:36</t>
+  </si>
+  <si>
+    <t>2026/09/14 09:23 啟動緊急叫修:門市反應SC(SHUTTLE7S)開啟HISHOP、e網、訂貨3.0都會出現【捷徑HISHOP.lnk參照的磁碟機或網路連線無法使用。請確定插入的磁碟正確，而且網路資源可以使用，然後重試。】，重啟SC仍異常。因開啟[訂貨3.0][HiShop][E網]出現捷徑異常訊息，請更換第二顆硬碟不備份還原，並攜帶主機隨行檢測...請台芝到店協助 PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 與門市確認帳務做到09/13，與通訊嘉芳確認缺少tm1、2電子存根聯</t>
+  </si>
+  <si>
+    <t>THILF02482</t>
+  </si>
+  <si>
+    <t>2026-09-14 09:24:43</t>
+  </si>
+  <si>
+    <t>2026-09-14 11:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 12:48:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:24:00</t>
+  </si>
+  <si>
+    <t>更換第二顆硬碟不備份還原
+SATA線*2</t>
+  </si>
+  <si>
+    <t>新莊福慧店</t>
+  </si>
+  <si>
+    <t>THILF04552</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:27:07</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:20:00</t>
+  </si>
+  <si>
+    <t>D195</t>
+  </si>
+  <si>
+    <t>三重車路頭</t>
+  </si>
+  <si>
+    <t>THILF0D195</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:48:07</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:33:00</t>
+  </si>
+  <si>
+    <t>新莊頭前店</t>
+  </si>
+  <si>
+    <t>THILF04144</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:48:24</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:50:00</t>
+  </si>
+  <si>
+    <t>新莊化成店</t>
+  </si>
+  <si>
+    <t>THILF02362</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:06:02</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:10:00</t>
+  </si>
+  <si>
+    <t>PMQ3
+店章故障無法蓋章</t>
+  </si>
+  <si>
+    <t>三重永福店</t>
+  </si>
+  <si>
+    <t>THILF02349</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:12:44</t>
+  </si>
+  <si>
+    <t>2026-09-14 14:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:02:00</t>
+  </si>
+  <si>
+    <t>北縣黎明店</t>
+  </si>
+  <si>
+    <t>THILF03137</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:35:39</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:30:00</t>
+  </si>
+  <si>
+    <t>三重福仁店</t>
+  </si>
+  <si>
+    <t>THILF03957</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:43:04</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:12:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:35:00</t>
+  </si>
+  <si>
+    <t>三重薔薇店</t>
+  </si>
+  <si>
+    <t>THILF04388</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:15:28</t>
+  </si>
+  <si>
+    <t>2026-09-14 15:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:06:00</t>
+  </si>
+  <si>
+    <t>新莊輔園店</t>
+  </si>
+  <si>
+    <t>THILF03851</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:22:41</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:20:00</t>
+  </si>
+  <si>
+    <t>E3751115091401</t>
+  </si>
+  <si>
+    <t>淡水真理大</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:31:57</t>
+  </si>
+  <si>
+    <t>HL28</t>
+  </si>
+  <si>
+    <t>HL-立式掃描器</t>
+  </si>
+  <si>
+    <t>掃瞄無反應或感應不良</t>
+  </si>
+  <si>
+    <t>門市TM2立式掃描器(MS7580)掃描條碼有嗶聲有亮燈，但吃不進去TM，確認游標有停在輸入顯示的地方，使用CCD掃描器掃商品確認可正常刷讀且TM有顯示，門市TM重啟亦無法排除......還請台芝到店協助(1.機台2 清帳後 跳出刷卡機結帳失敗畫面 .已經拔掉刷卡機重新連線 依樣跳失敗(消費者可正常結帳)2.機台2 座式掃秒機 有聲音但是無法刷讀商品)</t>
+  </si>
+  <si>
+    <t>THILF03751</t>
+  </si>
+  <si>
+    <t>2026-09-14 16:54:56</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 20:54:00</t>
+  </si>
+  <si>
+    <t>更換掃描器
+換下8118001359
+換上8118001356</t>
+  </si>
+  <si>
+    <t>13749115091401</t>
+  </si>
+  <si>
+    <t>龜山長庚科大</t>
+  </si>
+  <si>
+    <t>2026-09-14 19:08:09</t>
+  </si>
+  <si>
+    <t>門市反應tm1(TCX800)經常觸控不良、都要點很多下或是點了之後要隔5~10秒才會有反應，確認無張貼文宣或商品壓到，且門市每天都會擦螢幕，此情況已有一段時間，先前有協助門市進行觸控校正，門市告知也沒有改善，要求直接請工程師到店查看......還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF03749</t>
+  </si>
+  <si>
+    <t>2026-09-14 19:12:36</t>
+  </si>
+  <si>
+    <t>2026-09-15 13:55:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 14:25:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 23:12:00</t>
+  </si>
+  <si>
+    <t>觸控螢幕矯正後，可正常使用</t>
+  </si>
+  <si>
+    <t>12746115091501</t>
+  </si>
+  <si>
+    <t>板橋板嘉店</t>
+  </si>
+  <si>
+    <t>2026-09-15 09:38:43</t>
+  </si>
+  <si>
+    <t>門市反應TM1(TCX800)昨晚突然黑屏無法開機，下方電源無亮燈，已有重新拔插線路仍異常，與門市確認線路皆無脫落，ping80不通無法vnc...請台芝到店協助 已與門市確認9/15有銷售PS若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)</t>
+  </si>
+  <si>
+    <t>THILF02746</t>
+  </si>
+  <si>
+    <t>2026-09-15 09:40:56</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:28:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 13:40:00</t>
+  </si>
+  <si>
+    <t>更換TCx800
+換上：8185000106
+換下：8185002265</t>
+  </si>
+  <si>
+    <t>中和和大店</t>
+  </si>
+  <si>
+    <t>THILF02911</t>
+  </si>
+  <si>
+    <t>2026-09-15 10:17:06</t>
+  </si>
+  <si>
+    <t>2026-09-15 09:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 10:02:00</t>
+  </si>
+  <si>
+    <t>中和景德店</t>
+  </si>
+  <si>
+    <t>THILF04536</t>
+  </si>
+  <si>
+    <t>2026-09-15 10:40:59</t>
+  </si>
+  <si>
+    <t>2026-09-15 10:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 10:36:00</t>
+  </si>
+  <si>
+    <t>中和和竹店</t>
+  </si>
+  <si>
+    <t>THILF03883</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:51:18</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:25:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 12:27:30</t>
+  </si>
+  <si>
+    <t>2026-09-15 12:20:00</t>
+  </si>
+  <si>
+    <t>新莊莊美店</t>
+  </si>
+  <si>
+    <t>THILF04341</t>
+  </si>
+  <si>
+    <t>2026-09-15 14:43:22</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 14:43:26</t>
+  </si>
+  <si>
+    <t>mmk主機8137002238
+補上一顆螺帽</t>
+  </si>
+  <si>
+    <t>龜山庚勤樓</t>
+  </si>
+  <si>
+    <t>THILF05465</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:01:51</t>
+  </si>
+  <si>
+    <t>2026-09-15 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:32:04</t>
+  </si>
+  <si>
+    <t>2026-09-15 12:42:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 12:57:00</t>
+  </si>
+  <si>
+    <t>龜山明德樓</t>
+  </si>
+  <si>
+    <t>THILF05251</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:39:05</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-15 15:40:00</t>
   </si>
 </sst>
 </file>
@@ -2646,7 +3087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK91"/>
+  <dimension ref="A1:AK115"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -10442,7 +10883,7 @@
       <c r="M91" s="8"/>
       <c r="N91" s="7"/>
       <c r="O91" s="8"/>
-      <c r="P91" s="8"/>
+      <c r="P91" s="9"/>
       <c r="Q91" s="7" t="s">
         <v>724</v>
       </c>
@@ -10475,7 +10916,7 @@
       <c r="AB91" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC91" s="8" t="s">
+      <c r="AC91" s="9" t="s">
         <v>67</v>
       </c>
       <c r="AD91" s="7" t="s">
@@ -10488,6 +10929,1996 @@
       <c r="AI91" s="7"/>
       <c r="AJ91" s="7"/>
       <c r="AK91" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="92" spans="1:37">
+      <c r="A92" s="3">
+        <v>90</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C92" s="3">
+        <v>2026091959</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>728</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F92" s="3">
+        <v>4541</v>
+      </c>
+      <c r="G92" s="3" t="s">
+        <v>729</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="I92" s="3" t="s">
+        <v>731</v>
+      </c>
+      <c r="J92" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K92" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L92" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="M92" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="N92" s="3">
+        <v>2901</v>
+      </c>
+      <c r="O92" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P92" s="10" t="s">
+        <v>732</v>
+      </c>
+      <c r="Q92" s="3" t="s">
+        <v>733</v>
+      </c>
+      <c r="R92" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S92" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T92" s="3">
+        <v>1</v>
+      </c>
+      <c r="U92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V92" s="3" t="s">
+        <v>734</v>
+      </c>
+      <c r="W92" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="X92" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="Y92" s="3" t="s">
+        <v>737</v>
+      </c>
+      <c r="Z92" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA92" s="3"/>
+      <c r="AB92" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC92" s="10" t="s">
+        <v>738</v>
+      </c>
+      <c r="AD92" s="3"/>
+      <c r="AE92" s="3"/>
+      <c r="AF92" s="3"/>
+      <c r="AG92" s="3"/>
+      <c r="AH92" s="3"/>
+      <c r="AI92" s="3"/>
+      <c r="AJ92" s="3"/>
+      <c r="AK92" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="93" spans="1:37">
+      <c r="A93" s="7">
+        <v>91</v>
+      </c>
+      <c r="B93" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C93" s="7">
+        <v>2026091973</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>739</v>
+      </c>
+      <c r="E93" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F93" s="7">
+        <v>2259</v>
+      </c>
+      <c r="G93" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="H93" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I93" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="J93" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="K93" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L93" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M93" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N93" s="7">
+        <v>2306</v>
+      </c>
+      <c r="O93" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="P93" s="9" t="s">
+        <v>742</v>
+      </c>
+      <c r="Q93" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="R93" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S93" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T93" s="7">
+        <v>1</v>
+      </c>
+      <c r="U93" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V93" s="7" t="s">
+        <v>744</v>
+      </c>
+      <c r="W93" s="7" t="s">
+        <v>745</v>
+      </c>
+      <c r="X93" s="7" t="s">
+        <v>746</v>
+      </c>
+      <c r="Y93" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="Z93" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA93" s="7"/>
+      <c r="AB93" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC93" s="9" t="s">
+        <v>748</v>
+      </c>
+      <c r="AD93" s="7"/>
+      <c r="AE93" s="7"/>
+      <c r="AF93" s="7"/>
+      <c r="AG93" s="7"/>
+      <c r="AH93" s="7"/>
+      <c r="AI93" s="7"/>
+      <c r="AJ93" s="7"/>
+      <c r="AK93" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="94" spans="1:37">
+      <c r="A94" s="3">
+        <v>92</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C94" s="3">
+        <v>2026091981</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>749</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F94" s="3">
+        <v>2482</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="H94" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I94" s="3" t="s">
+        <v>751</v>
+      </c>
+      <c r="J94" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K94" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L94" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M94" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N94" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O94" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="P94" s="10" t="s">
+        <v>752</v>
+      </c>
+      <c r="Q94" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="R94" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S94" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T94" s="3">
+        <v>1</v>
+      </c>
+      <c r="U94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V94" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="W94" s="3" t="s">
+        <v>755</v>
+      </c>
+      <c r="X94" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="Y94" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="Z94" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="AA94" s="3"/>
+      <c r="AB94" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC94" s="10" t="s">
+        <v>758</v>
+      </c>
+      <c r="AD94" s="3"/>
+      <c r="AE94" s="3"/>
+      <c r="AF94" s="3"/>
+      <c r="AG94" s="3"/>
+      <c r="AH94" s="3"/>
+      <c r="AI94" s="3"/>
+      <c r="AJ94" s="3"/>
+      <c r="AK94" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="95" spans="1:37">
+      <c r="A95" s="7">
+        <v>93</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C95" s="7">
+        <v>2026092034</v>
+      </c>
+      <c r="D95" s="7"/>
+      <c r="E95" s="7"/>
+      <c r="F95" s="7">
+        <v>4552</v>
+      </c>
+      <c r="G95" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="H95" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I95" s="7"/>
+      <c r="J95" s="7"/>
+      <c r="K95" s="7"/>
+      <c r="L95" s="7"/>
+      <c r="M95" s="8"/>
+      <c r="N95" s="7"/>
+      <c r="O95" s="8"/>
+      <c r="P95" s="9"/>
+      <c r="Q95" s="7" t="s">
+        <v>760</v>
+      </c>
+      <c r="R95" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S95" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T95" s="7">
+        <v>1</v>
+      </c>
+      <c r="U95" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V95" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="W95" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="X95" s="7" t="s">
+        <v>763</v>
+      </c>
+      <c r="Y95" s="7"/>
+      <c r="Z95" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA95" s="7"/>
+      <c r="AB95" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC95" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD95" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE95" s="7"/>
+      <c r="AF95" s="7"/>
+      <c r="AG95" s="7"/>
+      <c r="AH95" s="7"/>
+      <c r="AI95" s="7"/>
+      <c r="AJ95" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK95" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="96" spans="1:37">
+      <c r="A96" s="3">
+        <v>94</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C96" s="3">
+        <v>2026092036</v>
+      </c>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="G96" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="H96" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I96" s="3"/>
+      <c r="J96" s="3"/>
+      <c r="K96" s="3"/>
+      <c r="L96" s="3"/>
+      <c r="M96" s="4"/>
+      <c r="N96" s="3"/>
+      <c r="O96" s="4"/>
+      <c r="P96" s="10"/>
+      <c r="Q96" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="R96" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S96" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T96" s="3">
+        <v>1</v>
+      </c>
+      <c r="U96" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V96" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="W96" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="X96" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="Y96" s="3"/>
+      <c r="Z96" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA96" s="3"/>
+      <c r="AB96" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC96" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD96" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE96" s="3"/>
+      <c r="AF96" s="3"/>
+      <c r="AG96" s="3"/>
+      <c r="AH96" s="3"/>
+      <c r="AI96" s="3"/>
+      <c r="AJ96" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK96" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:37">
+      <c r="A97" s="7">
+        <v>95</v>
+      </c>
+      <c r="B97" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C97" s="7">
+        <v>2026092037</v>
+      </c>
+      <c r="D97" s="7"/>
+      <c r="E97" s="7"/>
+      <c r="F97" s="7">
+        <v>4144</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>770</v>
+      </c>
+      <c r="H97" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I97" s="7"/>
+      <c r="J97" s="7"/>
+      <c r="K97" s="7"/>
+      <c r="L97" s="7"/>
+      <c r="M97" s="8"/>
+      <c r="N97" s="7"/>
+      <c r="O97" s="8"/>
+      <c r="P97" s="9"/>
+      <c r="Q97" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="R97" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S97" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T97" s="7">
+        <v>1</v>
+      </c>
+      <c r="U97" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V97" s="7" t="s">
+        <v>772</v>
+      </c>
+      <c r="W97" s="7" t="s">
+        <v>773</v>
+      </c>
+      <c r="X97" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="Y97" s="7"/>
+      <c r="Z97" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA97" s="7"/>
+      <c r="AB97" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC97" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD97" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE97" s="7"/>
+      <c r="AF97" s="7"/>
+      <c r="AG97" s="7"/>
+      <c r="AH97" s="7"/>
+      <c r="AI97" s="7"/>
+      <c r="AJ97" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK97" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="98" spans="1:37">
+      <c r="A98" s="3">
+        <v>96</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C98" s="3">
+        <v>2026092046</v>
+      </c>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3">
+        <v>2362</v>
+      </c>
+      <c r="G98" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I98" s="3"/>
+      <c r="J98" s="3"/>
+      <c r="K98" s="3"/>
+      <c r="L98" s="3"/>
+      <c r="M98" s="4"/>
+      <c r="N98" s="3"/>
+      <c r="O98" s="4"/>
+      <c r="P98" s="10"/>
+      <c r="Q98" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="R98" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S98" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T98" s="3">
+        <v>1</v>
+      </c>
+      <c r="U98" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V98" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="W98" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="X98" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="Y98" s="3"/>
+      <c r="Z98" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA98" s="3"/>
+      <c r="AB98" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC98" s="10" t="s">
+        <v>779</v>
+      </c>
+      <c r="AD98" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE98" s="3"/>
+      <c r="AF98" s="3"/>
+      <c r="AG98" s="3"/>
+      <c r="AH98" s="3"/>
+      <c r="AI98" s="3"/>
+      <c r="AJ98" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK98" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="99" spans="1:37">
+      <c r="A99" s="7">
+        <v>97</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C99" s="7">
+        <v>2026092047</v>
+      </c>
+      <c r="D99" s="7"/>
+      <c r="E99" s="7"/>
+      <c r="F99" s="7">
+        <v>2349</v>
+      </c>
+      <c r="G99" s="7" t="s">
+        <v>780</v>
+      </c>
+      <c r="H99" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I99" s="7"/>
+      <c r="J99" s="7"/>
+      <c r="K99" s="7"/>
+      <c r="L99" s="7"/>
+      <c r="M99" s="8"/>
+      <c r="N99" s="7"/>
+      <c r="O99" s="8"/>
+      <c r="P99" s="9"/>
+      <c r="Q99" s="7" t="s">
+        <v>781</v>
+      </c>
+      <c r="R99" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S99" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T99" s="7">
+        <v>1</v>
+      </c>
+      <c r="U99" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V99" s="7" t="s">
+        <v>782</v>
+      </c>
+      <c r="W99" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="X99" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="Y99" s="7"/>
+      <c r="Z99" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA99" s="7"/>
+      <c r="AB99" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC99" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD99" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE99" s="7"/>
+      <c r="AF99" s="7"/>
+      <c r="AG99" s="7"/>
+      <c r="AH99" s="7"/>
+      <c r="AI99" s="7"/>
+      <c r="AJ99" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK99" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" spans="1:37">
+      <c r="A100" s="3">
+        <v>98</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C100" s="3">
+        <v>2026092054</v>
+      </c>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3">
+        <v>3137</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="H100" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="I100" s="3"/>
+      <c r="J100" s="3"/>
+      <c r="K100" s="3"/>
+      <c r="L100" s="3"/>
+      <c r="M100" s="4"/>
+      <c r="N100" s="3"/>
+      <c r="O100" s="4"/>
+      <c r="P100" s="10"/>
+      <c r="Q100" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="R100" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S100" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T100" s="3">
+        <v>1</v>
+      </c>
+      <c r="U100" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V100" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="W100" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="X100" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="Y100" s="3"/>
+      <c r="Z100" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA100" s="3"/>
+      <c r="AB100" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC100" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD100" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE100" s="3"/>
+      <c r="AF100" s="3"/>
+      <c r="AG100" s="3"/>
+      <c r="AH100" s="3"/>
+      <c r="AI100" s="3"/>
+      <c r="AJ100" s="3"/>
+      <c r="AK100" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="101" spans="1:37">
+      <c r="A101" s="7">
+        <v>99</v>
+      </c>
+      <c r="B101" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C101" s="7">
+        <v>2026092060</v>
+      </c>
+      <c r="D101" s="7"/>
+      <c r="E101" s="7"/>
+      <c r="F101" s="7">
+        <v>3957</v>
+      </c>
+      <c r="G101" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="H101" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I101" s="7"/>
+      <c r="J101" s="7"/>
+      <c r="K101" s="7"/>
+      <c r="L101" s="7"/>
+      <c r="M101" s="8"/>
+      <c r="N101" s="7"/>
+      <c r="O101" s="8"/>
+      <c r="P101" s="9"/>
+      <c r="Q101" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="R101" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S101" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T101" s="7">
+        <v>1</v>
+      </c>
+      <c r="U101" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V101" s="7" t="s">
+        <v>791</v>
+      </c>
+      <c r="W101" s="7" t="s">
+        <v>792</v>
+      </c>
+      <c r="X101" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="Y101" s="7"/>
+      <c r="Z101" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA101" s="7"/>
+      <c r="AB101" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC101" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD101" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE101" s="7"/>
+      <c r="AF101" s="7"/>
+      <c r="AG101" s="7"/>
+      <c r="AH101" s="7"/>
+      <c r="AI101" s="7"/>
+      <c r="AJ101" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK101" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="102" spans="1:37">
+      <c r="A102" s="3">
+        <v>100</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C102" s="3">
+        <v>2026092068</v>
+      </c>
+      <c r="D102" s="3"/>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3">
+        <v>4388</v>
+      </c>
+      <c r="G102" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I102" s="3"/>
+      <c r="J102" s="3"/>
+      <c r="K102" s="3"/>
+      <c r="L102" s="3"/>
+      <c r="M102" s="4"/>
+      <c r="N102" s="3"/>
+      <c r="O102" s="4"/>
+      <c r="P102" s="10"/>
+      <c r="Q102" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="R102" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S102" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T102" s="3">
+        <v>1</v>
+      </c>
+      <c r="U102" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V102" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="W102" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="X102" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="Y102" s="3"/>
+      <c r="Z102" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA102" s="3"/>
+      <c r="AB102" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC102" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD102" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE102" s="3"/>
+      <c r="AF102" s="3"/>
+      <c r="AG102" s="3"/>
+      <c r="AH102" s="3"/>
+      <c r="AI102" s="3"/>
+      <c r="AJ102" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK102" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="103" spans="1:37">
+      <c r="A103" s="7">
+        <v>101</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C103" s="7">
+        <v>2026092071</v>
+      </c>
+      <c r="D103" s="7"/>
+      <c r="E103" s="7"/>
+      <c r="F103" s="7">
+        <v>3851</v>
+      </c>
+      <c r="G103" s="7" t="s">
+        <v>799</v>
+      </c>
+      <c r="H103" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I103" s="7"/>
+      <c r="J103" s="7"/>
+      <c r="K103" s="7"/>
+      <c r="L103" s="7"/>
+      <c r="M103" s="8"/>
+      <c r="N103" s="7"/>
+      <c r="O103" s="8"/>
+      <c r="P103" s="9"/>
+      <c r="Q103" s="7" t="s">
+        <v>800</v>
+      </c>
+      <c r="R103" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S103" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T103" s="7">
+        <v>1</v>
+      </c>
+      <c r="U103" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V103" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="W103" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="X103" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="Y103" s="7"/>
+      <c r="Z103" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA103" s="7"/>
+      <c r="AB103" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC103" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD103" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE103" s="7"/>
+      <c r="AF103" s="7"/>
+      <c r="AG103" s="7"/>
+      <c r="AH103" s="7"/>
+      <c r="AI103" s="7"/>
+      <c r="AJ103" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK103" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="104" spans="1:37">
+      <c r="A104" s="3">
+        <v>102</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C104" s="3">
+        <v>2026092075</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>804</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F104" s="3">
+        <v>3751</v>
+      </c>
+      <c r="G104" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="I104" s="3" t="s">
+        <v>806</v>
+      </c>
+      <c r="J104" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K104" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L104" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="M104" s="4" t="s">
+        <v>808</v>
+      </c>
+      <c r="N104" s="3">
+        <v>2803</v>
+      </c>
+      <c r="O104" s="4" t="s">
+        <v>809</v>
+      </c>
+      <c r="P104" s="10" t="s">
+        <v>810</v>
+      </c>
+      <c r="Q104" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="R104" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S104" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T104" s="3">
+        <v>1</v>
+      </c>
+      <c r="U104" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V104" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="W104" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="X104" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="Y104" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="Z104" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA104" s="3"/>
+      <c r="AB104" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC104" s="10" t="s">
+        <v>816</v>
+      </c>
+      <c r="AD104" s="3"/>
+      <c r="AE104" s="3"/>
+      <c r="AF104" s="3"/>
+      <c r="AG104" s="3"/>
+      <c r="AH104" s="3"/>
+      <c r="AI104" s="3"/>
+      <c r="AJ104" s="3"/>
+      <c r="AK104" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="105" spans="1:37">
+      <c r="A105" s="7">
+        <v>103</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C105" s="7">
+        <v>2026092082</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>817</v>
+      </c>
+      <c r="E105" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F105" s="7">
+        <v>3749</v>
+      </c>
+      <c r="G105" s="7" t="s">
+        <v>818</v>
+      </c>
+      <c r="H105" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I105" s="7" t="s">
+        <v>819</v>
+      </c>
+      <c r="J105" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="K105" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="L105" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M105" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N105" s="7">
+        <v>2307</v>
+      </c>
+      <c r="O105" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="P105" s="9" t="s">
+        <v>820</v>
+      </c>
+      <c r="Q105" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="R105" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S105" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T105" s="7">
+        <v>1</v>
+      </c>
+      <c r="U105" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V105" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="W105" s="7" t="s">
+        <v>823</v>
+      </c>
+      <c r="X105" s="7" t="s">
+        <v>824</v>
+      </c>
+      <c r="Y105" s="7" t="s">
+        <v>825</v>
+      </c>
+      <c r="Z105" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA105" s="7"/>
+      <c r="AB105" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC105" s="9" t="s">
+        <v>826</v>
+      </c>
+      <c r="AD105" s="7"/>
+      <c r="AE105" s="7"/>
+      <c r="AF105" s="7"/>
+      <c r="AG105" s="7"/>
+      <c r="AH105" s="7"/>
+      <c r="AI105" s="7"/>
+      <c r="AJ105" s="7"/>
+      <c r="AK105" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="106" spans="1:37">
+      <c r="A106" s="3">
+        <v>104</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C106" s="3">
+        <v>2026092109</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F106" s="3">
+        <v>2746</v>
+      </c>
+      <c r="G106" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I106" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="J106" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K106" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L106" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M106" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N106" s="3">
+        <v>2306</v>
+      </c>
+      <c r="O106" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="P106" s="10" t="s">
+        <v>830</v>
+      </c>
+      <c r="Q106" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="R106" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S106" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T106" s="3">
+        <v>1</v>
+      </c>
+      <c r="U106" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V106" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="W106" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="X106" s="3" t="s">
+        <v>834</v>
+      </c>
+      <c r="Y106" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="Z106" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA106" s="3"/>
+      <c r="AB106" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC106" s="10" t="s">
+        <v>836</v>
+      </c>
+      <c r="AD106" s="3"/>
+      <c r="AE106" s="3"/>
+      <c r="AF106" s="3"/>
+      <c r="AG106" s="3"/>
+      <c r="AH106" s="3"/>
+      <c r="AI106" s="3"/>
+      <c r="AJ106" s="3"/>
+      <c r="AK106" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="107" spans="1:37">
+      <c r="A107" s="7">
+        <v>105</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C107" s="7">
+        <v>2026092125</v>
+      </c>
+      <c r="D107" s="7"/>
+      <c r="E107" s="7"/>
+      <c r="F107" s="7">
+        <v>2911</v>
+      </c>
+      <c r="G107" s="7" t="s">
+        <v>837</v>
+      </c>
+      <c r="H107" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I107" s="7"/>
+      <c r="J107" s="7"/>
+      <c r="K107" s="7"/>
+      <c r="L107" s="7"/>
+      <c r="M107" s="8"/>
+      <c r="N107" s="7"/>
+      <c r="O107" s="8"/>
+      <c r="P107" s="9"/>
+      <c r="Q107" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="R107" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S107" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T107" s="7">
+        <v>1</v>
+      </c>
+      <c r="U107" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V107" s="7" t="s">
+        <v>839</v>
+      </c>
+      <c r="W107" s="7" t="s">
+        <v>840</v>
+      </c>
+      <c r="X107" s="7" t="s">
+        <v>841</v>
+      </c>
+      <c r="Y107" s="7"/>
+      <c r="Z107" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA107" s="7"/>
+      <c r="AB107" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC107" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD107" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE107" s="7"/>
+      <c r="AF107" s="7"/>
+      <c r="AG107" s="7"/>
+      <c r="AH107" s="7"/>
+      <c r="AI107" s="7"/>
+      <c r="AJ107" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK107" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="108" spans="1:37">
+      <c r="A108" s="3">
+        <v>106</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C108" s="3">
+        <v>2026092131</v>
+      </c>
+      <c r="D108" s="3"/>
+      <c r="E108" s="3"/>
+      <c r="F108" s="3">
+        <v>4536</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>842</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I108" s="3"/>
+      <c r="J108" s="3"/>
+      <c r="K108" s="3"/>
+      <c r="L108" s="3"/>
+      <c r="M108" s="4"/>
+      <c r="N108" s="3"/>
+      <c r="O108" s="4"/>
+      <c r="P108" s="10"/>
+      <c r="Q108" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="R108" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S108" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T108" s="3">
+        <v>1</v>
+      </c>
+      <c r="U108" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V108" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="W108" s="3" t="s">
+        <v>845</v>
+      </c>
+      <c r="X108" s="3" t="s">
+        <v>846</v>
+      </c>
+      <c r="Y108" s="3"/>
+      <c r="Z108" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA108" s="3"/>
+      <c r="AB108" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC108" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD108" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE108" s="3"/>
+      <c r="AF108" s="3"/>
+      <c r="AG108" s="3"/>
+      <c r="AH108" s="3"/>
+      <c r="AI108" s="3"/>
+      <c r="AJ108" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK108" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="109" spans="1:37">
+      <c r="A109" s="7">
+        <v>107</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C109" s="7">
+        <v>2026092158</v>
+      </c>
+      <c r="D109" s="7"/>
+      <c r="E109" s="7"/>
+      <c r="F109" s="7">
+        <v>3883</v>
+      </c>
+      <c r="G109" s="7" t="s">
+        <v>847</v>
+      </c>
+      <c r="H109" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I109" s="7"/>
+      <c r="J109" s="7"/>
+      <c r="K109" s="7"/>
+      <c r="L109" s="7"/>
+      <c r="M109" s="8"/>
+      <c r="N109" s="7"/>
+      <c r="O109" s="8"/>
+      <c r="P109" s="9"/>
+      <c r="Q109" s="7" t="s">
+        <v>848</v>
+      </c>
+      <c r="R109" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S109" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T109" s="7">
+        <v>1</v>
+      </c>
+      <c r="U109" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V109" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="W109" s="7" t="s">
+        <v>850</v>
+      </c>
+      <c r="X109" s="7" t="s">
+        <v>813</v>
+      </c>
+      <c r="Y109" s="7"/>
+      <c r="Z109" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA109" s="7"/>
+      <c r="AB109" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC109" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD109" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE109" s="7"/>
+      <c r="AF109" s="7"/>
+      <c r="AG109" s="7"/>
+      <c r="AH109" s="7"/>
+      <c r="AI109" s="7"/>
+      <c r="AJ109" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK109" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="110" spans="1:37">
+      <c r="A110" s="3">
+        <v>108</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C110" s="3">
+        <v>2026092160</v>
+      </c>
+      <c r="D110" s="3"/>
+      <c r="E110" s="3"/>
+      <c r="F110" s="3">
+        <v>3751</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="H110" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="I110" s="3"/>
+      <c r="J110" s="3"/>
+      <c r="K110" s="3"/>
+      <c r="L110" s="3"/>
+      <c r="M110" s="4"/>
+      <c r="N110" s="3"/>
+      <c r="O110" s="4"/>
+      <c r="P110" s="10"/>
+      <c r="Q110" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="R110" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S110" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T110" s="3">
+        <v>1</v>
+      </c>
+      <c r="U110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V110" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="W110" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="X110" s="3" t="s">
+        <v>852</v>
+      </c>
+      <c r="Y110" s="3"/>
+      <c r="Z110" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA110" s="3"/>
+      <c r="AB110" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC110" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD110" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE110" s="3"/>
+      <c r="AF110" s="3"/>
+      <c r="AG110" s="3"/>
+      <c r="AH110" s="3"/>
+      <c r="AI110" s="3"/>
+      <c r="AJ110" s="3"/>
+      <c r="AK110" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="111" spans="1:37">
+      <c r="A111" s="7">
+        <v>109</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C111" s="7">
+        <v>2026092181</v>
+      </c>
+      <c r="D111" s="7"/>
+      <c r="E111" s="7"/>
+      <c r="F111" s="7">
+        <v>4341</v>
+      </c>
+      <c r="G111" s="7" t="s">
+        <v>853</v>
+      </c>
+      <c r="H111" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I111" s="7"/>
+      <c r="J111" s="7"/>
+      <c r="K111" s="7"/>
+      <c r="L111" s="7"/>
+      <c r="M111" s="8"/>
+      <c r="N111" s="7"/>
+      <c r="O111" s="8"/>
+      <c r="P111" s="9"/>
+      <c r="Q111" s="7" t="s">
+        <v>854</v>
+      </c>
+      <c r="R111" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S111" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T111" s="7">
+        <v>1</v>
+      </c>
+      <c r="U111" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V111" s="7" t="s">
+        <v>855</v>
+      </c>
+      <c r="W111" s="7" t="s">
+        <v>856</v>
+      </c>
+      <c r="X111" s="7" t="s">
+        <v>857</v>
+      </c>
+      <c r="Y111" s="7"/>
+      <c r="Z111" s="7">
+        <v>3.5</v>
+      </c>
+      <c r="AA111" s="7"/>
+      <c r="AB111" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC111" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="AD111" s="7"/>
+      <c r="AE111" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF111" s="7"/>
+      <c r="AG111" s="7"/>
+      <c r="AH111" s="7"/>
+      <c r="AI111" s="7"/>
+      <c r="AJ111" s="7"/>
+      <c r="AK111" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="112" spans="1:37">
+      <c r="A112" s="3">
+        <v>110</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C112" s="3">
+        <v>2026092182</v>
+      </c>
+      <c r="D112" s="3"/>
+      <c r="E112" s="3"/>
+      <c r="F112" s="3">
+        <v>4341</v>
+      </c>
+      <c r="G112" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I112" s="3"/>
+      <c r="J112" s="3"/>
+      <c r="K112" s="3"/>
+      <c r="L112" s="3"/>
+      <c r="M112" s="4"/>
+      <c r="N112" s="3"/>
+      <c r="O112" s="4"/>
+      <c r="P112" s="10"/>
+      <c r="Q112" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="R112" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S112" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T112" s="3">
+        <v>1</v>
+      </c>
+      <c r="U112" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V112" s="3" t="s">
+        <v>858</v>
+      </c>
+      <c r="W112" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="X112" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="Y112" s="3"/>
+      <c r="Z112" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="AA112" s="3"/>
+      <c r="AB112" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC112" s="10" t="s">
+        <v>859</v>
+      </c>
+      <c r="AD112" s="3"/>
+      <c r="AE112" s="3"/>
+      <c r="AF112" s="3"/>
+      <c r="AG112" s="3"/>
+      <c r="AH112" s="3"/>
+      <c r="AI112" s="3"/>
+      <c r="AJ112" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK112" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="113" spans="1:37">
+      <c r="A113" s="7">
+        <v>111</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C113" s="7">
+        <v>2026092187</v>
+      </c>
+      <c r="D113" s="7"/>
+      <c r="E113" s="7"/>
+      <c r="F113" s="7">
+        <v>5465</v>
+      </c>
+      <c r="G113" s="7" t="s">
+        <v>860</v>
+      </c>
+      <c r="H113" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I113" s="7"/>
+      <c r="J113" s="7"/>
+      <c r="K113" s="7"/>
+      <c r="L113" s="7"/>
+      <c r="M113" s="8"/>
+      <c r="N113" s="7"/>
+      <c r="O113" s="8"/>
+      <c r="P113" s="9"/>
+      <c r="Q113" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="R113" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S113" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T113" s="7">
+        <v>1</v>
+      </c>
+      <c r="U113" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V113" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="W113" s="7" t="s">
+        <v>857</v>
+      </c>
+      <c r="X113" s="7" t="s">
+        <v>863</v>
+      </c>
+      <c r="Y113" s="7"/>
+      <c r="Z113" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA113" s="7"/>
+      <c r="AB113" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC113" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD113" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE113" s="7"/>
+      <c r="AF113" s="7"/>
+      <c r="AG113" s="7"/>
+      <c r="AH113" s="7"/>
+      <c r="AI113" s="7"/>
+      <c r="AJ113" s="7"/>
+      <c r="AK113" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="114" spans="1:37">
+      <c r="A114" s="3">
+        <v>112</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C114" s="3">
+        <v>2026092195</v>
+      </c>
+      <c r="D114" s="3"/>
+      <c r="E114" s="3"/>
+      <c r="F114" s="3">
+        <v>2746</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I114" s="3"/>
+      <c r="J114" s="3"/>
+      <c r="K114" s="3"/>
+      <c r="L114" s="3"/>
+      <c r="M114" s="4"/>
+      <c r="N114" s="3"/>
+      <c r="O114" s="4"/>
+      <c r="P114" s="10"/>
+      <c r="Q114" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="R114" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S114" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T114" s="3">
+        <v>1</v>
+      </c>
+      <c r="U114" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V114" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="W114" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="X114" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="Y114" s="3"/>
+      <c r="Z114" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA114" s="3"/>
+      <c r="AB114" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC114" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD114" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE114" s="3"/>
+      <c r="AF114" s="3"/>
+      <c r="AG114" s="3"/>
+      <c r="AH114" s="3"/>
+      <c r="AI114" s="3"/>
+      <c r="AJ114" s="3"/>
+      <c r="AK114" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="115" spans="1:37">
+      <c r="A115" s="7">
+        <v>113</v>
+      </c>
+      <c r="B115" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C115" s="7">
+        <v>2026092203</v>
+      </c>
+      <c r="D115" s="7"/>
+      <c r="E115" s="7"/>
+      <c r="F115" s="7">
+        <v>5251</v>
+      </c>
+      <c r="G115" s="7" t="s">
+        <v>867</v>
+      </c>
+      <c r="H115" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I115" s="7"/>
+      <c r="J115" s="7"/>
+      <c r="K115" s="7"/>
+      <c r="L115" s="7"/>
+      <c r="M115" s="8"/>
+      <c r="N115" s="7"/>
+      <c r="O115" s="8"/>
+      <c r="P115" s="8"/>
+      <c r="Q115" s="7" t="s">
+        <v>868</v>
+      </c>
+      <c r="R115" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S115" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T115" s="7">
+        <v>1</v>
+      </c>
+      <c r="U115" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V115" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="W115" s="7" t="s">
+        <v>870</v>
+      </c>
+      <c r="X115" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="Y115" s="7"/>
+      <c r="Z115" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA115" s="7"/>
+      <c r="AB115" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC115" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD115" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE115" s="7"/>
+      <c r="AF115" s="7"/>
+      <c r="AG115" s="7"/>
+      <c r="AH115" s="7"/>
+      <c r="AI115" s="7"/>
+      <c r="AJ115" s="7"/>
+      <c r="AK115" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09171456
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$115</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$127</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="872">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-15  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="951">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-17  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -2600,6 +2600,39 @@
     <t>2026-09-15 10:36:00</t>
   </si>
   <si>
+    <t>15428115091501</t>
+  </si>
+  <si>
+    <t>三重野球魂</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:34:59</t>
+  </si>
+  <si>
+    <t>當機</t>
+  </si>
+  <si>
+    <t>門市反應TM1(TCX800)早上清帳後就只要一交易就會黑屏關機，確認下方電源無亮燈，已有請門市將轉接器及電源線插頭重新拔插仍無法排除，VNC請門市開機後一刷讀商品就馬上關機無法排除...請台芝到店協助 已與門市確認9/16無銷售PS若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)</t>
+  </si>
+  <si>
+    <t>THILF05428</t>
+  </si>
+  <si>
+    <t>2026-09-15 11:37:44</t>
+  </si>
+  <si>
+    <t>2026-09-16 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:37:00</t>
+  </si>
+  <si>
+    <t>TM1. 一二顆硬碟不備份還原。</t>
+  </si>
+  <si>
     <t>中和和竹店</t>
   </si>
   <si>
@@ -2674,6 +2707,210 @@
   </si>
   <si>
     <t>2026-09-15 15:40:00</t>
+  </si>
+  <si>
+    <t>E3785115091601</t>
+  </si>
+  <si>
+    <t>北縣莊榮店</t>
+  </si>
+  <si>
+    <t>2026-09-16 13:18:08</t>
+  </si>
+  <si>
+    <t>門市反應MMK4代機風扇聲音很大聲，已請門市關機拔插休息後開機聲音更大聲....需請台芝到店協助(風扇大聲吵雜要壞了)</t>
+  </si>
+  <si>
+    <t>THILF03785</t>
+  </si>
+  <si>
+    <t>2026-09-16 13:41:32</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 17:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 17:41:00</t>
+  </si>
+  <si>
+    <t>更換風扇</t>
+  </si>
+  <si>
+    <t>淡水阿給店</t>
+  </si>
+  <si>
+    <t>THILF05671</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:18:36</t>
+  </si>
+  <si>
+    <t>2026-09-16 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:17:00</t>
+  </si>
+  <si>
+    <t>新開門市裝機完工</t>
+  </si>
+  <si>
+    <t>三重重新三</t>
+  </si>
+  <si>
+    <t>THILF03741</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:27:48</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:02:00</t>
+  </si>
+  <si>
+    <t>三重重安店</t>
+  </si>
+  <si>
+    <t>THILF02302</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:02:09</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 14:55:00</t>
+  </si>
+  <si>
+    <t>14977115091601</t>
+  </si>
+  <si>
+    <t>三重初戀店</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:18:17</t>
+  </si>
+  <si>
+    <t>門市反應TM1多卡機(QP3000E)無電源反應，已確認後方線路無鬆脫..請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04977</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:19:38</t>
+  </si>
+  <si>
+    <t>2026-09-17 11:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 11:38:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 19:19:00</t>
+  </si>
+  <si>
+    <t>換下8183001843 換上8183000513</t>
+  </si>
+  <si>
+    <t>三重中央南</t>
+  </si>
+  <si>
+    <t>THILF04083</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:26:43</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:03:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:23:00</t>
+  </si>
+  <si>
+    <t>北投地熱谷</t>
+  </si>
+  <si>
+    <t>台北市北投區</t>
+  </si>
+  <si>
+    <t>THILF04313</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:03:34</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 15:58:00</t>
+  </si>
+  <si>
+    <t>三重文化北</t>
+  </si>
+  <si>
+    <t>THILF04312</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:08:00</t>
+  </si>
+  <si>
+    <t>三重圖書館</t>
+  </si>
+  <si>
+    <t>THILF02209</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:34:40</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:32:00</t>
+  </si>
+  <si>
+    <t>15251115091701</t>
+  </si>
+  <si>
+    <t>2026-09-17 12:29:15</t>
+  </si>
+  <si>
+    <t>門市TM2(UPOS211K)觸控不良，數字鍵需點選很多次才會有反應，已有確認螢幕沒有保護貼或廣告文宣，並有擦拭過螢幕後進行觸控校正仍無法排除...還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-17 12:31:10</t>
+  </si>
+  <si>
+    <t>2026-09-17 14:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 14:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 16:31:00</t>
+  </si>
+  <si>
+    <t>現場無異狀，測試各式觸控皆為正常</t>
+  </si>
+  <si>
+    <t>新莊瓏山林</t>
+  </si>
+  <si>
+    <t>THILF05389</t>
+  </si>
+  <si>
+    <t>2026-09-17 14:46:07</t>
+  </si>
+  <si>
+    <t>2026-09-17 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 14:50:00</t>
   </si>
 </sst>
 </file>
@@ -3087,7 +3324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK115"/>
+  <dimension ref="A1:AK127"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -12386,32 +12623,52 @@
         <v>107</v>
       </c>
       <c r="B109" s="7" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C109" s="7">
-        <v>2026092158</v>
-      </c>
-      <c r="D109" s="7"/>
-      <c r="E109" s="7"/>
+        <v>2026092150</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>847</v>
+      </c>
+      <c r="E109" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F109" s="7">
-        <v>3883</v>
+        <v>5428</v>
       </c>
       <c r="G109" s="7" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="H109" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I109" s="7"/>
-      <c r="J109" s="7"/>
-      <c r="K109" s="7"/>
-      <c r="L109" s="7"/>
-      <c r="M109" s="8"/>
-      <c r="N109" s="7"/>
-      <c r="O109" s="8"/>
-      <c r="P109" s="9"/>
+        <v>42</v>
+      </c>
+      <c r="I109" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="J109" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K109" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L109" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M109" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N109" s="7">
+        <v>2301</v>
+      </c>
+      <c r="O109" s="8" t="s">
+        <v>850</v>
+      </c>
+      <c r="P109" s="9" t="s">
+        <v>851</v>
+      </c>
       <c r="Q109" s="7" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="R109" s="7" t="s">
         <v>51</v>
@@ -12426,36 +12683,34 @@
         <v>53</v>
       </c>
       <c r="V109" s="7" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
       <c r="W109" s="7" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="X109" s="7" t="s">
-        <v>813</v>
-      </c>
-      <c r="Y109" s="7"/>
+        <v>855</v>
+      </c>
+      <c r="Y109" s="7" t="s">
+        <v>856</v>
+      </c>
       <c r="Z109" s="7">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="AA109" s="7"/>
       <c r="AB109" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC109" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD109" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>857</v>
+      </c>
+      <c r="AD109" s="7"/>
       <c r="AE109" s="7"/>
       <c r="AF109" s="7"/>
       <c r="AG109" s="7"/>
       <c r="AH109" s="7"/>
       <c r="AI109" s="7"/>
-      <c r="AJ109" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ109" s="7"/>
       <c r="AK109" s="7" t="s">
         <v>60</v>
       </c>
@@ -12468,18 +12723,18 @@
         <v>61</v>
       </c>
       <c r="C110" s="3">
-        <v>2026092160</v>
+        <v>2026092158</v>
       </c>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
       <c r="F110" s="3">
-        <v>3751</v>
+        <v>3883</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>805</v>
+        <v>858</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>730</v>
+        <v>140</v>
       </c>
       <c r="I110" s="3"/>
       <c r="J110" s="3"/>
@@ -12490,13 +12745,13 @@
       <c r="O110" s="4"/>
       <c r="P110" s="10"/>
       <c r="Q110" s="3" t="s">
-        <v>811</v>
+        <v>859</v>
       </c>
       <c r="R110" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S110" s="3" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="T110" s="3">
         <v>1</v>
@@ -12505,17 +12760,17 @@
         <v>53</v>
       </c>
       <c r="V110" s="3" t="s">
-        <v>851</v>
+        <v>860</v>
       </c>
       <c r="W110" s="3" t="s">
-        <v>814</v>
+        <v>861</v>
       </c>
       <c r="X110" s="3" t="s">
-        <v>852</v>
+        <v>813</v>
       </c>
       <c r="Y110" s="3"/>
       <c r="Z110" s="3">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA110" s="3"/>
       <c r="AB110" s="3" t="s">
@@ -12532,7 +12787,9 @@
       <c r="AG110" s="3"/>
       <c r="AH110" s="3"/>
       <c r="AI110" s="3"/>
-      <c r="AJ110" s="3"/>
+      <c r="AJ110" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AK110" s="3" t="s">
         <v>60</v>
       </c>
@@ -12545,18 +12802,18 @@
         <v>61</v>
       </c>
       <c r="C111" s="7">
-        <v>2026092181</v>
+        <v>2026092160</v>
       </c>
       <c r="D111" s="7"/>
       <c r="E111" s="7"/>
       <c r="F111" s="7">
-        <v>4341</v>
+        <v>3751</v>
       </c>
       <c r="G111" s="7" t="s">
-        <v>853</v>
+        <v>805</v>
       </c>
       <c r="H111" s="7" t="s">
-        <v>328</v>
+        <v>730</v>
       </c>
       <c r="I111" s="7"/>
       <c r="J111" s="7"/>
@@ -12567,13 +12824,13 @@
       <c r="O111" s="8"/>
       <c r="P111" s="9"/>
       <c r="Q111" s="7" t="s">
-        <v>854</v>
+        <v>811</v>
       </c>
       <c r="R111" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S111" s="7" t="s">
-        <v>320</v>
+        <v>92</v>
       </c>
       <c r="T111" s="7">
         <v>1</v>
@@ -12582,29 +12839,29 @@
         <v>53</v>
       </c>
       <c r="V111" s="7" t="s">
-        <v>855</v>
+        <v>862</v>
       </c>
       <c r="W111" s="7" t="s">
-        <v>856</v>
+        <v>814</v>
       </c>
       <c r="X111" s="7" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="Y111" s="7"/>
       <c r="Z111" s="7">
-        <v>3.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA111" s="7"/>
       <c r="AB111" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC111" s="9" t="s">
-        <v>450</v>
-      </c>
-      <c r="AD111" s="7"/>
-      <c r="AE111" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="AD111" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE111" s="7"/>
       <c r="AF111" s="7"/>
       <c r="AG111" s="7"/>
       <c r="AH111" s="7"/>
@@ -12622,7 +12879,7 @@
         <v>61</v>
       </c>
       <c r="C112" s="3">
-        <v>2026092182</v>
+        <v>2026092181</v>
       </c>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
@@ -12630,7 +12887,7 @@
         <v>4341</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>328</v>
@@ -12644,7 +12901,7 @@
       <c r="O112" s="4"/>
       <c r="P112" s="10"/>
       <c r="Q112" s="3" t="s">
-        <v>854</v>
+        <v>865</v>
       </c>
       <c r="R112" s="3" t="s">
         <v>51</v>
@@ -12659,13 +12916,13 @@
         <v>53</v>
       </c>
       <c r="V112" s="3" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
       <c r="W112" s="3" t="s">
-        <v>856</v>
+        <v>867</v>
       </c>
       <c r="X112" s="3" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="Y112" s="3"/>
       <c r="Z112" s="3">
@@ -12676,17 +12933,17 @@
         <v>58</v>
       </c>
       <c r="AC112" s="10" t="s">
-        <v>859</v>
+        <v>450</v>
       </c>
       <c r="AD112" s="3"/>
-      <c r="AE112" s="3"/>
+      <c r="AE112" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AF112" s="3"/>
       <c r="AG112" s="3"/>
       <c r="AH112" s="3"/>
       <c r="AI112" s="3"/>
-      <c r="AJ112" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ112" s="3"/>
       <c r="AK112" s="3" t="s">
         <v>60</v>
       </c>
@@ -12699,18 +12956,18 @@
         <v>61</v>
       </c>
       <c r="C113" s="7">
-        <v>2026092187</v>
+        <v>2026092182</v>
       </c>
       <c r="D113" s="7"/>
       <c r="E113" s="7"/>
       <c r="F113" s="7">
-        <v>5465</v>
+        <v>4341</v>
       </c>
       <c r="G113" s="7" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="H113" s="7" t="s">
-        <v>90</v>
+        <v>328</v>
       </c>
       <c r="I113" s="7"/>
       <c r="J113" s="7"/>
@@ -12721,13 +12978,13 @@
       <c r="O113" s="8"/>
       <c r="P113" s="9"/>
       <c r="Q113" s="7" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="R113" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S113" s="7" t="s">
-        <v>92</v>
+        <v>320</v>
       </c>
       <c r="T113" s="7">
         <v>1</v>
@@ -12736,34 +12993,34 @@
         <v>53</v>
       </c>
       <c r="V113" s="7" t="s">
-        <v>862</v>
+        <v>869</v>
       </c>
       <c r="W113" s="7" t="s">
-        <v>857</v>
+        <v>867</v>
       </c>
       <c r="X113" s="7" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="Y113" s="7"/>
       <c r="Z113" s="7">
-        <v>0.3</v>
+        <v>3.5</v>
       </c>
       <c r="AA113" s="7"/>
       <c r="AB113" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC113" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD113" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>870</v>
+      </c>
+      <c r="AD113" s="7"/>
       <c r="AE113" s="7"/>
       <c r="AF113" s="7"/>
       <c r="AG113" s="7"/>
       <c r="AH113" s="7"/>
       <c r="AI113" s="7"/>
-      <c r="AJ113" s="7"/>
+      <c r="AJ113" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AK113" s="7" t="s">
         <v>60</v>
       </c>
@@ -12776,18 +13033,18 @@
         <v>61</v>
       </c>
       <c r="C114" s="3">
-        <v>2026092195</v>
+        <v>2026092187</v>
       </c>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
       <c r="F114" s="3">
-        <v>2746</v>
+        <v>5465</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>828</v>
+        <v>871</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>153</v>
+        <v>90</v>
       </c>
       <c r="I114" s="3"/>
       <c r="J114" s="3"/>
@@ -12798,13 +13055,13 @@
       <c r="O114" s="4"/>
       <c r="P114" s="10"/>
       <c r="Q114" s="3" t="s">
-        <v>831</v>
+        <v>872</v>
       </c>
       <c r="R114" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S114" s="3" t="s">
-        <v>160</v>
+        <v>92</v>
       </c>
       <c r="T114" s="3">
         <v>1</v>
@@ -12813,13 +13070,13 @@
         <v>53</v>
       </c>
       <c r="V114" s="3" t="s">
-        <v>864</v>
+        <v>873</v>
       </c>
       <c r="W114" s="3" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
       <c r="X114" s="3" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
       <c r="Y114" s="3"/>
       <c r="Z114" s="3">
@@ -12853,18 +13110,18 @@
         <v>61</v>
       </c>
       <c r="C115" s="7">
-        <v>2026092203</v>
+        <v>2026092195</v>
       </c>
       <c r="D115" s="7"/>
       <c r="E115" s="7"/>
       <c r="F115" s="7">
-        <v>5251</v>
+        <v>2746</v>
       </c>
       <c r="G115" s="7" t="s">
-        <v>867</v>
+        <v>828</v>
       </c>
       <c r="H115" s="7" t="s">
-        <v>90</v>
+        <v>153</v>
       </c>
       <c r="I115" s="7"/>
       <c r="J115" s="7"/>
@@ -12873,15 +13130,15 @@
       <c r="M115" s="8"/>
       <c r="N115" s="7"/>
       <c r="O115" s="8"/>
-      <c r="P115" s="8"/>
+      <c r="P115" s="9"/>
       <c r="Q115" s="7" t="s">
-        <v>868</v>
+        <v>831</v>
       </c>
       <c r="R115" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S115" s="7" t="s">
-        <v>92</v>
+        <v>160</v>
       </c>
       <c r="T115" s="7">
         <v>1</v>
@@ -12890,13 +13147,13 @@
         <v>53</v>
       </c>
       <c r="V115" s="7" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="W115" s="7" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="X115" s="7" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="Y115" s="7"/>
       <c r="Z115" s="7">
@@ -12906,7 +13163,7 @@
       <c r="AB115" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC115" s="8" t="s">
+      <c r="AC115" s="9" t="s">
         <v>67</v>
       </c>
       <c r="AD115" s="7" t="s">
@@ -12919,6 +13176,1004 @@
       <c r="AI115" s="7"/>
       <c r="AJ115" s="7"/>
       <c r="AK115" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="116" spans="1:37">
+      <c r="A116" s="3">
+        <v>114</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C116" s="3">
+        <v>2026092203</v>
+      </c>
+      <c r="D116" s="3"/>
+      <c r="E116" s="3"/>
+      <c r="F116" s="3">
+        <v>5251</v>
+      </c>
+      <c r="G116" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="H116" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I116" s="3"/>
+      <c r="J116" s="3"/>
+      <c r="K116" s="3"/>
+      <c r="L116" s="3"/>
+      <c r="M116" s="4"/>
+      <c r="N116" s="3"/>
+      <c r="O116" s="4"/>
+      <c r="P116" s="10"/>
+      <c r="Q116" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="R116" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S116" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T116" s="3">
+        <v>1</v>
+      </c>
+      <c r="U116" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V116" s="3" t="s">
+        <v>880</v>
+      </c>
+      <c r="W116" s="3" t="s">
+        <v>881</v>
+      </c>
+      <c r="X116" s="3" t="s">
+        <v>882</v>
+      </c>
+      <c r="Y116" s="3"/>
+      <c r="Z116" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA116" s="3"/>
+      <c r="AB116" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC116" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD116" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE116" s="3"/>
+      <c r="AF116" s="3"/>
+      <c r="AG116" s="3"/>
+      <c r="AH116" s="3"/>
+      <c r="AI116" s="3"/>
+      <c r="AJ116" s="3"/>
+      <c r="AK116" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="117" spans="1:37">
+      <c r="A117" s="7">
+        <v>115</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C117" s="7">
+        <v>2026092322</v>
+      </c>
+      <c r="D117" s="7" t="s">
+        <v>883</v>
+      </c>
+      <c r="E117" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F117" s="7">
+        <v>3785</v>
+      </c>
+      <c r="G117" s="7" t="s">
+        <v>884</v>
+      </c>
+      <c r="H117" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I117" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="J117" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K117" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L117" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M117" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="N117" s="7">
+        <v>5801</v>
+      </c>
+      <c r="O117" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="P117" s="9" t="s">
+        <v>886</v>
+      </c>
+      <c r="Q117" s="7" t="s">
+        <v>887</v>
+      </c>
+      <c r="R117" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S117" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T117" s="7">
+        <v>1</v>
+      </c>
+      <c r="U117" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V117" s="7" t="s">
+        <v>888</v>
+      </c>
+      <c r="W117" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="X117" s="7" t="s">
+        <v>890</v>
+      </c>
+      <c r="Y117" s="7" t="s">
+        <v>891</v>
+      </c>
+      <c r="Z117" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA117" s="7"/>
+      <c r="AB117" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC117" s="9" t="s">
+        <v>892</v>
+      </c>
+      <c r="AD117" s="7"/>
+      <c r="AE117" s="7"/>
+      <c r="AF117" s="7"/>
+      <c r="AG117" s="7"/>
+      <c r="AH117" s="7"/>
+      <c r="AI117" s="7"/>
+      <c r="AJ117" s="7"/>
+      <c r="AK117" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="118" spans="1:37">
+      <c r="A118" s="3">
+        <v>116</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C118" s="3">
+        <v>2026092327</v>
+      </c>
+      <c r="D118" s="3"/>
+      <c r="E118" s="3"/>
+      <c r="F118" s="3">
+        <v>5671</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="H118" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="I118" s="3"/>
+      <c r="J118" s="3"/>
+      <c r="K118" s="3"/>
+      <c r="L118" s="3"/>
+      <c r="M118" s="4"/>
+      <c r="N118" s="3"/>
+      <c r="O118" s="4"/>
+      <c r="P118" s="10"/>
+      <c r="Q118" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="R118" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S118" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T118" s="3">
+        <v>1</v>
+      </c>
+      <c r="U118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V118" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="W118" s="3" t="s">
+        <v>896</v>
+      </c>
+      <c r="X118" s="3" t="s">
+        <v>897</v>
+      </c>
+      <c r="Y118" s="3"/>
+      <c r="Z118" s="3">
+        <v>3.3</v>
+      </c>
+      <c r="AA118" s="3"/>
+      <c r="AB118" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC118" s="10" t="s">
+        <v>898</v>
+      </c>
+      <c r="AD118" s="3"/>
+      <c r="AE118" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF118" s="3"/>
+      <c r="AG118" s="3"/>
+      <c r="AH118" s="3"/>
+      <c r="AI118" s="3"/>
+      <c r="AJ118" s="3"/>
+      <c r="AK118" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="119" spans="1:37">
+      <c r="A119" s="7">
+        <v>117</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C119" s="7">
+        <v>2026092329</v>
+      </c>
+      <c r="D119" s="7"/>
+      <c r="E119" s="7"/>
+      <c r="F119" s="7">
+        <v>3741</v>
+      </c>
+      <c r="G119" s="7" t="s">
+        <v>899</v>
+      </c>
+      <c r="H119" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I119" s="7"/>
+      <c r="J119" s="7"/>
+      <c r="K119" s="7"/>
+      <c r="L119" s="7"/>
+      <c r="M119" s="8"/>
+      <c r="N119" s="7"/>
+      <c r="O119" s="8"/>
+      <c r="P119" s="9"/>
+      <c r="Q119" s="7" t="s">
+        <v>900</v>
+      </c>
+      <c r="R119" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S119" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T119" s="7">
+        <v>1</v>
+      </c>
+      <c r="U119" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V119" s="7" t="s">
+        <v>901</v>
+      </c>
+      <c r="W119" s="7" t="s">
+        <v>902</v>
+      </c>
+      <c r="X119" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="Y119" s="7"/>
+      <c r="Z119" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="7"/>
+      <c r="AB119" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC119" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD119" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE119" s="7"/>
+      <c r="AF119" s="7"/>
+      <c r="AG119" s="7"/>
+      <c r="AH119" s="7"/>
+      <c r="AI119" s="7"/>
+      <c r="AJ119" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK119" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="120" spans="1:37">
+      <c r="A120" s="3">
+        <v>118</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C120" s="3">
+        <v>2026092334</v>
+      </c>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3"/>
+      <c r="F120" s="3">
+        <v>2302</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>904</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I120" s="3"/>
+      <c r="J120" s="3"/>
+      <c r="K120" s="3"/>
+      <c r="L120" s="3"/>
+      <c r="M120" s="4"/>
+      <c r="N120" s="3"/>
+      <c r="O120" s="4"/>
+      <c r="P120" s="10"/>
+      <c r="Q120" s="3" t="s">
+        <v>905</v>
+      </c>
+      <c r="R120" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S120" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T120" s="3">
+        <v>1</v>
+      </c>
+      <c r="U120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V120" s="3" t="s">
+        <v>906</v>
+      </c>
+      <c r="W120" s="3" t="s">
+        <v>907</v>
+      </c>
+      <c r="X120" s="3" t="s">
+        <v>908</v>
+      </c>
+      <c r="Y120" s="3"/>
+      <c r="Z120" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA120" s="3"/>
+      <c r="AB120" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC120" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD120" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE120" s="3"/>
+      <c r="AF120" s="3"/>
+      <c r="AG120" s="3"/>
+      <c r="AH120" s="3"/>
+      <c r="AI120" s="3"/>
+      <c r="AJ120" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK120" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="121" spans="1:37">
+      <c r="A121" s="7">
+        <v>119</v>
+      </c>
+      <c r="B121" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C121" s="7">
+        <v>2026092344</v>
+      </c>
+      <c r="D121" s="7" t="s">
+        <v>909</v>
+      </c>
+      <c r="E121" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F121" s="7">
+        <v>4977</v>
+      </c>
+      <c r="G121" s="7" t="s">
+        <v>910</v>
+      </c>
+      <c r="H121" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I121" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="J121" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K121" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L121" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="M121" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="N121" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="O121" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="P121" s="9" t="s">
+        <v>912</v>
+      </c>
+      <c r="Q121" s="7" t="s">
+        <v>913</v>
+      </c>
+      <c r="R121" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S121" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T121" s="7">
+        <v>1</v>
+      </c>
+      <c r="U121" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V121" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="W121" s="7" t="s">
+        <v>915</v>
+      </c>
+      <c r="X121" s="7" t="s">
+        <v>916</v>
+      </c>
+      <c r="Y121" s="7" t="s">
+        <v>917</v>
+      </c>
+      <c r="Z121" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA121" s="7"/>
+      <c r="AB121" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC121" s="9" t="s">
+        <v>918</v>
+      </c>
+      <c r="AD121" s="7"/>
+      <c r="AE121" s="7"/>
+      <c r="AF121" s="7"/>
+      <c r="AG121" s="7"/>
+      <c r="AH121" s="7"/>
+      <c r="AI121" s="7"/>
+      <c r="AJ121" s="7"/>
+      <c r="AK121" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="122" spans="1:37">
+      <c r="A122" s="3">
+        <v>120</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C122" s="3">
+        <v>2026092347</v>
+      </c>
+      <c r="D122" s="3"/>
+      <c r="E122" s="3"/>
+      <c r="F122" s="3">
+        <v>4083</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I122" s="3"/>
+      <c r="J122" s="3"/>
+      <c r="K122" s="3"/>
+      <c r="L122" s="3"/>
+      <c r="M122" s="4"/>
+      <c r="N122" s="3"/>
+      <c r="O122" s="4"/>
+      <c r="P122" s="10"/>
+      <c r="Q122" s="3" t="s">
+        <v>920</v>
+      </c>
+      <c r="R122" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T122" s="3">
+        <v>1</v>
+      </c>
+      <c r="U122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V122" s="3" t="s">
+        <v>921</v>
+      </c>
+      <c r="W122" s="3" t="s">
+        <v>922</v>
+      </c>
+      <c r="X122" s="3" t="s">
+        <v>923</v>
+      </c>
+      <c r="Y122" s="3"/>
+      <c r="Z122" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA122" s="3"/>
+      <c r="AB122" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC122" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD122" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE122" s="3"/>
+      <c r="AF122" s="3"/>
+      <c r="AG122" s="3"/>
+      <c r="AH122" s="3"/>
+      <c r="AI122" s="3"/>
+      <c r="AJ122" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK122" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="123" spans="1:37">
+      <c r="A123" s="7">
+        <v>121</v>
+      </c>
+      <c r="B123" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C123" s="7">
+        <v>2026092368</v>
+      </c>
+      <c r="D123" s="7"/>
+      <c r="E123" s="7"/>
+      <c r="F123" s="7">
+        <v>4313</v>
+      </c>
+      <c r="G123" s="7" t="s">
+        <v>924</v>
+      </c>
+      <c r="H123" s="7" t="s">
+        <v>925</v>
+      </c>
+      <c r="I123" s="7"/>
+      <c r="J123" s="7"/>
+      <c r="K123" s="7"/>
+      <c r="L123" s="7"/>
+      <c r="M123" s="8"/>
+      <c r="N123" s="7"/>
+      <c r="O123" s="8"/>
+      <c r="P123" s="9"/>
+      <c r="Q123" s="7" t="s">
+        <v>926</v>
+      </c>
+      <c r="R123" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S123" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T123" s="7">
+        <v>1</v>
+      </c>
+      <c r="U123" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V123" s="7" t="s">
+        <v>927</v>
+      </c>
+      <c r="W123" s="7" t="s">
+        <v>928</v>
+      </c>
+      <c r="X123" s="7" t="s">
+        <v>929</v>
+      </c>
+      <c r="Y123" s="7"/>
+      <c r="Z123" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA123" s="7"/>
+      <c r="AB123" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC123" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD123" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE123" s="7"/>
+      <c r="AF123" s="7"/>
+      <c r="AG123" s="7"/>
+      <c r="AH123" s="7"/>
+      <c r="AI123" s="7"/>
+      <c r="AJ123" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK123" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="124" spans="1:37">
+      <c r="A124" s="3">
+        <v>122</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C124" s="3">
+        <v>2026092370</v>
+      </c>
+      <c r="D124" s="3"/>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3">
+        <v>4312</v>
+      </c>
+      <c r="G124" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I124" s="3"/>
+      <c r="J124" s="3"/>
+      <c r="K124" s="3"/>
+      <c r="L124" s="3"/>
+      <c r="M124" s="4"/>
+      <c r="N124" s="3"/>
+      <c r="O124" s="4"/>
+      <c r="P124" s="10"/>
+      <c r="Q124" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="R124" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S124" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T124" s="3">
+        <v>1</v>
+      </c>
+      <c r="U124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V124" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="W124" s="3" t="s">
+        <v>928</v>
+      </c>
+      <c r="X124" s="3" t="s">
+        <v>929</v>
+      </c>
+      <c r="Y124" s="3"/>
+      <c r="Z124" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA124" s="3"/>
+      <c r="AB124" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC124" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD124" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE124" s="3"/>
+      <c r="AF124" s="3"/>
+      <c r="AG124" s="3"/>
+      <c r="AH124" s="3"/>
+      <c r="AI124" s="3"/>
+      <c r="AJ124" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK124" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="125" spans="1:37">
+      <c r="A125" s="7">
+        <v>123</v>
+      </c>
+      <c r="B125" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C125" s="7">
+        <v>2026092379</v>
+      </c>
+      <c r="D125" s="7"/>
+      <c r="E125" s="7"/>
+      <c r="F125" s="7">
+        <v>2209</v>
+      </c>
+      <c r="G125" s="7" t="s">
+        <v>933</v>
+      </c>
+      <c r="H125" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I125" s="7"/>
+      <c r="J125" s="7"/>
+      <c r="K125" s="7"/>
+      <c r="L125" s="7"/>
+      <c r="M125" s="8"/>
+      <c r="N125" s="7"/>
+      <c r="O125" s="8"/>
+      <c r="P125" s="9"/>
+      <c r="Q125" s="7" t="s">
+        <v>934</v>
+      </c>
+      <c r="R125" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S125" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T125" s="7">
+        <v>1</v>
+      </c>
+      <c r="U125" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V125" s="7" t="s">
+        <v>935</v>
+      </c>
+      <c r="W125" s="7" t="s">
+        <v>936</v>
+      </c>
+      <c r="X125" s="7" t="s">
+        <v>937</v>
+      </c>
+      <c r="Y125" s="7"/>
+      <c r="Z125" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA125" s="7"/>
+      <c r="AB125" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC125" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD125" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE125" s="7"/>
+      <c r="AF125" s="7"/>
+      <c r="AG125" s="7"/>
+      <c r="AH125" s="7"/>
+      <c r="AI125" s="7"/>
+      <c r="AJ125" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK125" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="126" spans="1:37">
+      <c r="A126" s="3">
+        <v>124</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C126" s="3">
+        <v>2026092440</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>938</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F126" s="3">
+        <v>5251</v>
+      </c>
+      <c r="G126" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="H126" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I126" s="3" t="s">
+        <v>939</v>
+      </c>
+      <c r="J126" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K126" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L126" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M126" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N126" s="3">
+        <v>2307</v>
+      </c>
+      <c r="O126" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="P126" s="10" t="s">
+        <v>940</v>
+      </c>
+      <c r="Q126" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="R126" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S126" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T126" s="3">
+        <v>1</v>
+      </c>
+      <c r="U126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V126" s="3" t="s">
+        <v>941</v>
+      </c>
+      <c r="W126" s="3" t="s">
+        <v>942</v>
+      </c>
+      <c r="X126" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="Y126" s="3" t="s">
+        <v>944</v>
+      </c>
+      <c r="Z126" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA126" s="3"/>
+      <c r="AB126" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC126" s="10" t="s">
+        <v>945</v>
+      </c>
+      <c r="AD126" s="3"/>
+      <c r="AE126" s="3"/>
+      <c r="AF126" s="3"/>
+      <c r="AG126" s="3"/>
+      <c r="AH126" s="3"/>
+      <c r="AI126" s="3"/>
+      <c r="AJ126" s="3"/>
+      <c r="AK126" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="127" spans="1:37">
+      <c r="A127" s="7">
+        <v>125</v>
+      </c>
+      <c r="B127" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C127" s="7">
+        <v>2026092457</v>
+      </c>
+      <c r="D127" s="7"/>
+      <c r="E127" s="7"/>
+      <c r="F127" s="7">
+        <v>5389</v>
+      </c>
+      <c r="G127" s="7" t="s">
+        <v>946</v>
+      </c>
+      <c r="H127" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I127" s="7"/>
+      <c r="J127" s="7"/>
+      <c r="K127" s="7"/>
+      <c r="L127" s="7"/>
+      <c r="M127" s="8"/>
+      <c r="N127" s="7"/>
+      <c r="O127" s="8"/>
+      <c r="P127" s="8"/>
+      <c r="Q127" s="7" t="s">
+        <v>947</v>
+      </c>
+      <c r="R127" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S127" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T127" s="7">
+        <v>1</v>
+      </c>
+      <c r="U127" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V127" s="7" t="s">
+        <v>948</v>
+      </c>
+      <c r="W127" s="7" t="s">
+        <v>949</v>
+      </c>
+      <c r="X127" s="7" t="s">
+        <v>950</v>
+      </c>
+      <c r="Y127" s="7"/>
+      <c r="Z127" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA127" s="7"/>
+      <c r="AB127" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC127" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD127" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE127" s="7"/>
+      <c r="AF127" s="7"/>
+      <c r="AG127" s="7"/>
+      <c r="AH127" s="7"/>
+      <c r="AI127" s="7"/>
+      <c r="AJ127" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK127" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09181743
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$127</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$138</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="951">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-17  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1025">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-18  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -2874,6 +2874,41 @@
     <t>2026-09-16 16:32:00</t>
   </si>
   <si>
+    <t>ED767115091602</t>
+  </si>
+  <si>
+    <t>D767</t>
+  </si>
+  <si>
+    <t>板橋寶翠店</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:51:04</t>
+  </si>
+  <si>
+    <t>門市反應tm1(TCX800) CCD掃描器(HC76TR)有亮燈有逼聲，但掃讀條碼及商品皆需掃很多次才成功，門市已有操作過掃描器校正仍異常....須請台芝到店協助(機一重置六步驟還是感應不良.帳單跟商品很難刷讀造成客人不滿.請盡速派人處理 謝謝)</t>
+  </si>
+  <si>
+    <t>THILF0D767</t>
+  </si>
+  <si>
+    <t>2026-09-16 16:58:07</t>
+  </si>
+  <si>
+    <t>2026-09-17 17:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 17:22:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 20:58:00</t>
+  </si>
+  <si>
+    <t>更換76掃槍
+換上：8119012850
+換下：8119012471</t>
+  </si>
+  <si>
     <t>15251115091701</t>
   </si>
   <si>
@@ -2911,6 +2946,195 @@
   </si>
   <si>
     <t>2026-09-17 14:50:00</t>
+  </si>
+  <si>
+    <t>新莊鼎苑店</t>
+  </si>
+  <si>
+    <t>THILF04194</t>
+  </si>
+  <si>
+    <t>2026-09-17 15:06:19</t>
+  </si>
+  <si>
+    <t>2026-09-17 15:10:00</t>
+  </si>
+  <si>
+    <t>新莊幸運店</t>
+  </si>
+  <si>
+    <t>THILF04679</t>
+  </si>
+  <si>
+    <t>2026-09-17 15:27:59</t>
+  </si>
+  <si>
+    <t>2026-09-17 15:30:00</t>
+  </si>
+  <si>
+    <t>中和和玉店</t>
+  </si>
+  <si>
+    <t>THILF03913</t>
+  </si>
+  <si>
+    <t>2026-09-17 16:40:11</t>
+  </si>
+  <si>
+    <t>2026-09-17 16:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-17 16:35:00</t>
+  </si>
+  <si>
+    <t>14560115091702</t>
+  </si>
+  <si>
+    <t>三重大院店</t>
+  </si>
+  <si>
+    <t>2026-09-17 21:10:09</t>
+  </si>
+  <si>
+    <t>hub(GS1900 24E)門市告知tm2刷卡機無法使用ping52不通，有先解mac將22port重新拔插仍異常，將22port移至20PORT並開放後ping52有通，應為22port孔異常，須請台芝到店協助確認相關設備及線路</t>
+  </si>
+  <si>
+    <t>THILF04560</t>
+  </si>
+  <si>
+    <t>2026-09-17 21:12:09</t>
+  </si>
+  <si>
+    <t>2026-09-18 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 01:12:00</t>
+  </si>
+  <si>
+    <t>重置hub.  插拔網路線</t>
+  </si>
+  <si>
+    <t>14341115091801</t>
+  </si>
+  <si>
+    <t>2026-09-18 08:47:56</t>
+  </si>
+  <si>
+    <t>2026/9/18 (週五) 上午 08:38 總公司明翰MAIL:有關 4341新莊莊美店請到店更換SC(SHUTTLE7S)第一顆硬碟，資料不要備份，請協助緊急派工，到店更換SC第一顆硬碟，資料不備份，謝謝。PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)與區經理確認帳關到09/17，與通訊圭連確認都有收到</t>
+  </si>
+  <si>
+    <t>2026-09-18 09:19:56</t>
+  </si>
+  <si>
+    <t>2026-09-18 09:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 11:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:19:00</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原。 已送跟店家告知回報代收會計。</t>
+  </si>
+  <si>
+    <t>15057115091801</t>
+  </si>
+  <si>
+    <t>新莊中港店</t>
+  </si>
+  <si>
+    <t>2026-09-18 10:31:02</t>
+  </si>
+  <si>
+    <t>門市反應TM1(TCX800)近期經常發生突然關機無電源反應的狀況，門市都需要重新拔插線路後才能開機...需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF05057</t>
+  </si>
+  <si>
+    <t>2026-09-18 10:32:52</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 16:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 14:32:00</t>
+  </si>
+  <si>
+    <t>重新固定變壓器排線</t>
+  </si>
+  <si>
+    <t>D346</t>
+  </si>
+  <si>
+    <t>三重維德店</t>
+  </si>
+  <si>
+    <t>THILF0D346</t>
+  </si>
+  <si>
+    <t>2026-09-18 14:57:29</t>
+  </si>
+  <si>
+    <t>2026-09-18 14:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 14:42:00</t>
+  </si>
+  <si>
+    <t>15057115091803</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:17:03</t>
+  </si>
+  <si>
+    <t>9/18 15:06 總公司玫君啟動緊急叫修：門市反應TM1(TCX800)近期經常發生突然關機無電源反應的狀況，門市都需要重新拔插線路後才能開機...需請台芝到店協助，PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)門市今日尚未清帳入帳日09/18有交易</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:20:35</t>
+  </si>
+  <si>
+    <t>2026-09-19 08:20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">重新固定變壓器排線 </t>
+  </si>
+  <si>
+    <t>三重商工店</t>
+  </si>
+  <si>
+    <t>THILF04652</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:24:25</t>
+  </si>
+  <si>
+    <t>2026-09-18 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:13:00</t>
+  </si>
+  <si>
+    <t>三重護山店</t>
+  </si>
+  <si>
+    <t>THILF05245</t>
+  </si>
+  <si>
+    <t>2026-09-18 16:01:33</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:36:00</t>
+  </si>
+  <si>
+    <t>2026-09-18 15:58:00</t>
   </si>
 </sst>
 </file>
@@ -3324,7 +3548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK127"/>
+  <dimension ref="A1:AK138"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -14009,7 +14233,7 @@
         <v>38</v>
       </c>
       <c r="C126" s="3">
-        <v>2026092440</v>
+        <v>2026092390</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>938</v>
@@ -14017,47 +14241,47 @@
       <c r="E126" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F126" s="3">
-        <v>5251</v>
+      <c r="F126" s="3" t="s">
+        <v>939</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>878</v>
+        <v>940</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>90</v>
+        <v>153</v>
       </c>
       <c r="I126" s="3" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="J126" s="3" t="s">
-        <v>236</v>
+        <v>126</v>
       </c>
       <c r="K126" s="3" t="s">
         <v>45</v>
       </c>
       <c r="L126" s="3" t="s">
-        <v>155</v>
+        <v>73</v>
       </c>
       <c r="M126" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="N126" s="3">
-        <v>2307</v>
+        <v>74</v>
+      </c>
+      <c r="N126" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="O126" s="4" t="s">
-        <v>157</v>
+        <v>76</v>
       </c>
       <c r="P126" s="10" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="Q126" s="3" t="s">
-        <v>879</v>
+        <v>943</v>
       </c>
       <c r="R126" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S126" s="3" t="s">
-        <v>92</v>
+        <v>160</v>
       </c>
       <c r="T126" s="3">
         <v>1</v>
@@ -14066,26 +14290,26 @@
         <v>53</v>
       </c>
       <c r="V126" s="3" t="s">
-        <v>941</v>
+        <v>944</v>
       </c>
       <c r="W126" s="3" t="s">
-        <v>942</v>
+        <v>945</v>
       </c>
       <c r="X126" s="3" t="s">
-        <v>943</v>
+        <v>946</v>
       </c>
       <c r="Y126" s="3" t="s">
-        <v>944</v>
+        <v>947</v>
       </c>
       <c r="Z126" s="3">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA126" s="3"/>
       <c r="AB126" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC126" s="10" t="s">
-        <v>945</v>
+        <v>948</v>
       </c>
       <c r="AD126" s="3"/>
       <c r="AE126" s="3"/>
@@ -14103,38 +14327,58 @@
         <v>125</v>
       </c>
       <c r="B127" s="7" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C127" s="7">
-        <v>2026092457</v>
-      </c>
-      <c r="D127" s="7"/>
-      <c r="E127" s="7"/>
+        <v>2026092440</v>
+      </c>
+      <c r="D127" s="7" t="s">
+        <v>949</v>
+      </c>
+      <c r="E127" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F127" s="7">
-        <v>5389</v>
+        <v>5251</v>
       </c>
       <c r="G127" s="7" t="s">
-        <v>946</v>
+        <v>878</v>
       </c>
       <c r="H127" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="I127" s="7"/>
-      <c r="J127" s="7"/>
-      <c r="K127" s="7"/>
-      <c r="L127" s="7"/>
-      <c r="M127" s="8"/>
-      <c r="N127" s="7"/>
-      <c r="O127" s="8"/>
-      <c r="P127" s="8"/>
+        <v>90</v>
+      </c>
+      <c r="I127" s="7" t="s">
+        <v>950</v>
+      </c>
+      <c r="J127" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K127" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L127" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M127" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N127" s="7">
+        <v>2307</v>
+      </c>
+      <c r="O127" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="P127" s="9" t="s">
+        <v>951</v>
+      </c>
       <c r="Q127" s="7" t="s">
-        <v>947</v>
+        <v>879</v>
       </c>
       <c r="R127" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S127" s="7" t="s">
-        <v>320</v>
+        <v>92</v>
       </c>
       <c r="T127" s="7">
         <v>1</v>
@@ -14143,37 +14387,976 @@
         <v>53</v>
       </c>
       <c r="V127" s="7" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="W127" s="7" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="X127" s="7" t="s">
-        <v>950</v>
-      </c>
-      <c r="Y127" s="7"/>
+        <v>954</v>
+      </c>
+      <c r="Y127" s="7" t="s">
+        <v>955</v>
+      </c>
       <c r="Z127" s="7">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA127" s="7"/>
       <c r="AB127" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC127" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD127" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AC127" s="9" t="s">
+        <v>956</v>
+      </c>
+      <c r="AD127" s="7"/>
       <c r="AE127" s="7"/>
       <c r="AF127" s="7"/>
       <c r="AG127" s="7"/>
       <c r="AH127" s="7"/>
       <c r="AI127" s="7"/>
-      <c r="AJ127" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ127" s="7"/>
       <c r="AK127" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="128" spans="1:37">
+      <c r="A128" s="3">
+        <v>126</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C128" s="3">
+        <v>2026092457</v>
+      </c>
+      <c r="D128" s="3"/>
+      <c r="E128" s="3"/>
+      <c r="F128" s="3">
+        <v>5389</v>
+      </c>
+      <c r="G128" s="3" t="s">
+        <v>957</v>
+      </c>
+      <c r="H128" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I128" s="3"/>
+      <c r="J128" s="3"/>
+      <c r="K128" s="3"/>
+      <c r="L128" s="3"/>
+      <c r="M128" s="4"/>
+      <c r="N128" s="3"/>
+      <c r="O128" s="4"/>
+      <c r="P128" s="10"/>
+      <c r="Q128" s="3" t="s">
+        <v>958</v>
+      </c>
+      <c r="R128" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S128" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T128" s="3">
+        <v>1</v>
+      </c>
+      <c r="U128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V128" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="W128" s="3" t="s">
+        <v>960</v>
+      </c>
+      <c r="X128" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="Y128" s="3"/>
+      <c r="Z128" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA128" s="3"/>
+      <c r="AB128" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC128" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD128" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE128" s="3"/>
+      <c r="AF128" s="3"/>
+      <c r="AG128" s="3"/>
+      <c r="AH128" s="3"/>
+      <c r="AI128" s="3"/>
+      <c r="AJ128" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK128" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="129" spans="1:37">
+      <c r="A129" s="7">
+        <v>127</v>
+      </c>
+      <c r="B129" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C129" s="7">
+        <v>2026092461</v>
+      </c>
+      <c r="D129" s="7"/>
+      <c r="E129" s="7"/>
+      <c r="F129" s="7">
+        <v>4194</v>
+      </c>
+      <c r="G129" s="7" t="s">
+        <v>962</v>
+      </c>
+      <c r="H129" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I129" s="7"/>
+      <c r="J129" s="7"/>
+      <c r="K129" s="7"/>
+      <c r="L129" s="7"/>
+      <c r="M129" s="8"/>
+      <c r="N129" s="7"/>
+      <c r="O129" s="8"/>
+      <c r="P129" s="9"/>
+      <c r="Q129" s="7" t="s">
+        <v>963</v>
+      </c>
+      <c r="R129" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S129" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T129" s="7">
+        <v>1</v>
+      </c>
+      <c r="U129" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V129" s="7" t="s">
+        <v>964</v>
+      </c>
+      <c r="W129" s="7" t="s">
+        <v>961</v>
+      </c>
+      <c r="X129" s="7" t="s">
+        <v>965</v>
+      </c>
+      <c r="Y129" s="7"/>
+      <c r="Z129" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA129" s="7"/>
+      <c r="AB129" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC129" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD129" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE129" s="7"/>
+      <c r="AF129" s="7"/>
+      <c r="AG129" s="7"/>
+      <c r="AH129" s="7"/>
+      <c r="AI129" s="7"/>
+      <c r="AJ129" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK129" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="130" spans="1:37">
+      <c r="A130" s="3">
+        <v>128</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C130" s="3">
+        <v>2026092462</v>
+      </c>
+      <c r="D130" s="3"/>
+      <c r="E130" s="3"/>
+      <c r="F130" s="3">
+        <v>4679</v>
+      </c>
+      <c r="G130" s="3" t="s">
+        <v>966</v>
+      </c>
+      <c r="H130" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I130" s="3"/>
+      <c r="J130" s="3"/>
+      <c r="K130" s="3"/>
+      <c r="L130" s="3"/>
+      <c r="M130" s="4"/>
+      <c r="N130" s="3"/>
+      <c r="O130" s="4"/>
+      <c r="P130" s="10"/>
+      <c r="Q130" s="3" t="s">
+        <v>967</v>
+      </c>
+      <c r="R130" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S130" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T130" s="3">
+        <v>1</v>
+      </c>
+      <c r="U130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V130" s="3" t="s">
+        <v>968</v>
+      </c>
+      <c r="W130" s="3" t="s">
+        <v>965</v>
+      </c>
+      <c r="X130" s="3" t="s">
+        <v>969</v>
+      </c>
+      <c r="Y130" s="3"/>
+      <c r="Z130" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA130" s="3"/>
+      <c r="AB130" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC130" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD130" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE130" s="3"/>
+      <c r="AF130" s="3"/>
+      <c r="AG130" s="3"/>
+      <c r="AH130" s="3"/>
+      <c r="AI130" s="3"/>
+      <c r="AJ130" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK130" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="131" spans="1:37">
+      <c r="A131" s="7">
+        <v>129</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C131" s="7">
+        <v>2026092472</v>
+      </c>
+      <c r="D131" s="7"/>
+      <c r="E131" s="7"/>
+      <c r="F131" s="7">
+        <v>3913</v>
+      </c>
+      <c r="G131" s="7" t="s">
+        <v>970</v>
+      </c>
+      <c r="H131" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I131" s="7"/>
+      <c r="J131" s="7"/>
+      <c r="K131" s="7"/>
+      <c r="L131" s="7"/>
+      <c r="M131" s="8"/>
+      <c r="N131" s="7"/>
+      <c r="O131" s="8"/>
+      <c r="P131" s="9"/>
+      <c r="Q131" s="7" t="s">
+        <v>971</v>
+      </c>
+      <c r="R131" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S131" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T131" s="7">
+        <v>1</v>
+      </c>
+      <c r="U131" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V131" s="7" t="s">
+        <v>972</v>
+      </c>
+      <c r="W131" s="7" t="s">
+        <v>973</v>
+      </c>
+      <c r="X131" s="7" t="s">
+        <v>974</v>
+      </c>
+      <c r="Y131" s="7"/>
+      <c r="Z131" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA131" s="7"/>
+      <c r="AB131" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC131" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD131" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE131" s="7"/>
+      <c r="AF131" s="7"/>
+      <c r="AG131" s="7"/>
+      <c r="AH131" s="7"/>
+      <c r="AI131" s="7"/>
+      <c r="AJ131" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK131" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="132" spans="1:37">
+      <c r="A132" s="3">
+        <v>130</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C132" s="3">
+        <v>2026092573</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>975</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F132" s="3">
+        <v>4560</v>
+      </c>
+      <c r="G132" s="3" t="s">
+        <v>976</v>
+      </c>
+      <c r="H132" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I132" s="3" t="s">
+        <v>977</v>
+      </c>
+      <c r="J132" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K132" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L132" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="M132" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="N132" s="3">
+        <v>3402</v>
+      </c>
+      <c r="O132" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="P132" s="10" t="s">
+        <v>978</v>
+      </c>
+      <c r="Q132" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="R132" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S132" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T132" s="3">
+        <v>1</v>
+      </c>
+      <c r="U132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V132" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="W132" s="3" t="s">
+        <v>981</v>
+      </c>
+      <c r="X132" s="3" t="s">
+        <v>982</v>
+      </c>
+      <c r="Y132" s="3" t="s">
+        <v>983</v>
+      </c>
+      <c r="Z132" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA132" s="3"/>
+      <c r="AB132" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC132" s="10" t="s">
+        <v>984</v>
+      </c>
+      <c r="AD132" s="3"/>
+      <c r="AE132" s="3"/>
+      <c r="AF132" s="3"/>
+      <c r="AG132" s="3"/>
+      <c r="AH132" s="3"/>
+      <c r="AI132" s="3"/>
+      <c r="AJ132" s="3"/>
+      <c r="AK132" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="133" spans="1:37">
+      <c r="A133" s="7">
+        <v>131</v>
+      </c>
+      <c r="B133" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C133" s="7">
+        <v>2026092583</v>
+      </c>
+      <c r="D133" s="7" t="s">
+        <v>985</v>
+      </c>
+      <c r="E133" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F133" s="7">
+        <v>4341</v>
+      </c>
+      <c r="G133" s="7" t="s">
+        <v>864</v>
+      </c>
+      <c r="H133" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I133" s="7" t="s">
+        <v>986</v>
+      </c>
+      <c r="J133" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="K133" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L133" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M133" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N133" s="7">
+        <v>2405</v>
+      </c>
+      <c r="O133" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="P133" s="9" t="s">
+        <v>987</v>
+      </c>
+      <c r="Q133" s="7" t="s">
+        <v>865</v>
+      </c>
+      <c r="R133" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S133" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T133" s="7">
+        <v>1</v>
+      </c>
+      <c r="U133" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V133" s="7" t="s">
+        <v>988</v>
+      </c>
+      <c r="W133" s="7" t="s">
+        <v>989</v>
+      </c>
+      <c r="X133" s="7" t="s">
+        <v>990</v>
+      </c>
+      <c r="Y133" s="7" t="s">
+        <v>991</v>
+      </c>
+      <c r="Z133" s="7">
+        <v>1.9</v>
+      </c>
+      <c r="AA133" s="7"/>
+      <c r="AB133" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC133" s="9" t="s">
+        <v>992</v>
+      </c>
+      <c r="AD133" s="7"/>
+      <c r="AE133" s="7"/>
+      <c r="AF133" s="7"/>
+      <c r="AG133" s="7"/>
+      <c r="AH133" s="7"/>
+      <c r="AI133" s="7"/>
+      <c r="AJ133" s="7"/>
+      <c r="AK133" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="134" spans="1:37">
+      <c r="A134" s="3">
+        <v>132</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C134" s="3">
+        <v>2026092594</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>993</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F134" s="3">
+        <v>5057</v>
+      </c>
+      <c r="G134" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="H134" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I134" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="J134" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K134" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L134" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M134" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N134" s="3">
+        <v>2306</v>
+      </c>
+      <c r="O134" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="P134" s="10" t="s">
+        <v>996</v>
+      </c>
+      <c r="Q134" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="R134" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S134" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T134" s="3">
+        <v>1</v>
+      </c>
+      <c r="U134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V134" s="3" t="s">
+        <v>998</v>
+      </c>
+      <c r="W134" s="3" t="s">
+        <v>999</v>
+      </c>
+      <c r="X134" s="3" t="s">
+        <v>1000</v>
+      </c>
+      <c r="Y134" s="3" t="s">
+        <v>1001</v>
+      </c>
+      <c r="Z134" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA134" s="3"/>
+      <c r="AB134" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC134" s="10" t="s">
+        <v>1002</v>
+      </c>
+      <c r="AD134" s="3"/>
+      <c r="AE134" s="3"/>
+      <c r="AF134" s="3"/>
+      <c r="AG134" s="3"/>
+      <c r="AH134" s="3"/>
+      <c r="AI134" s="3"/>
+      <c r="AJ134" s="3"/>
+      <c r="AK134" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="135" spans="1:37">
+      <c r="A135" s="7">
+        <v>133</v>
+      </c>
+      <c r="B135" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C135" s="7">
+        <v>2026092633</v>
+      </c>
+      <c r="D135" s="7"/>
+      <c r="E135" s="7"/>
+      <c r="F135" s="7" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G135" s="7" t="s">
+        <v>1004</v>
+      </c>
+      <c r="H135" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I135" s="7"/>
+      <c r="J135" s="7"/>
+      <c r="K135" s="7"/>
+      <c r="L135" s="7"/>
+      <c r="M135" s="8"/>
+      <c r="N135" s="7"/>
+      <c r="O135" s="8"/>
+      <c r="P135" s="9"/>
+      <c r="Q135" s="7" t="s">
+        <v>1005</v>
+      </c>
+      <c r="R135" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S135" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T135" s="7">
+        <v>1</v>
+      </c>
+      <c r="U135" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V135" s="7" t="s">
+        <v>1006</v>
+      </c>
+      <c r="W135" s="7" t="s">
+        <v>1007</v>
+      </c>
+      <c r="X135" s="7" t="s">
+        <v>1008</v>
+      </c>
+      <c r="Y135" s="7"/>
+      <c r="Z135" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA135" s="7"/>
+      <c r="AB135" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC135" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD135" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE135" s="7"/>
+      <c r="AF135" s="7"/>
+      <c r="AG135" s="7"/>
+      <c r="AH135" s="7"/>
+      <c r="AI135" s="7"/>
+      <c r="AJ135" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK135" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="136" spans="1:37">
+      <c r="A136" s="3">
+        <v>134</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C136" s="3">
+        <v>2026092641</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F136" s="3">
+        <v>5057</v>
+      </c>
+      <c r="G136" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="H136" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I136" s="3" t="s">
+        <v>1010</v>
+      </c>
+      <c r="J136" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K136" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L136" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M136" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N136" s="3">
+        <v>2306</v>
+      </c>
+      <c r="O136" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="P136" s="10" t="s">
+        <v>1011</v>
+      </c>
+      <c r="Q136" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="R136" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S136" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T136" s="3">
+        <v>1</v>
+      </c>
+      <c r="U136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V136" s="3" t="s">
+        <v>1012</v>
+      </c>
+      <c r="W136" s="3" t="s">
+        <v>999</v>
+      </c>
+      <c r="X136" s="3" t="s">
+        <v>1000</v>
+      </c>
+      <c r="Y136" s="3" t="s">
+        <v>1013</v>
+      </c>
+      <c r="Z136" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA136" s="3"/>
+      <c r="AB136" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC136" s="10" t="s">
+        <v>1014</v>
+      </c>
+      <c r="AD136" s="3"/>
+      <c r="AE136" s="3"/>
+      <c r="AF136" s="3"/>
+      <c r="AG136" s="3"/>
+      <c r="AH136" s="3"/>
+      <c r="AI136" s="3"/>
+      <c r="AJ136" s="3"/>
+      <c r="AK136" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="137" spans="1:37">
+      <c r="A137" s="7">
+        <v>135</v>
+      </c>
+      <c r="B137" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C137" s="7">
+        <v>2026092643</v>
+      </c>
+      <c r="D137" s="7"/>
+      <c r="E137" s="7"/>
+      <c r="F137" s="7">
+        <v>4652</v>
+      </c>
+      <c r="G137" s="7" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H137" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I137" s="7"/>
+      <c r="J137" s="7"/>
+      <c r="K137" s="7"/>
+      <c r="L137" s="7"/>
+      <c r="M137" s="8"/>
+      <c r="N137" s="7"/>
+      <c r="O137" s="8"/>
+      <c r="P137" s="9"/>
+      <c r="Q137" s="7" t="s">
+        <v>1016</v>
+      </c>
+      <c r="R137" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S137" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T137" s="7">
+        <v>1</v>
+      </c>
+      <c r="U137" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V137" s="7" t="s">
+        <v>1017</v>
+      </c>
+      <c r="W137" s="7" t="s">
+        <v>1018</v>
+      </c>
+      <c r="X137" s="7" t="s">
+        <v>1019</v>
+      </c>
+      <c r="Y137" s="7"/>
+      <c r="Z137" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA137" s="7"/>
+      <c r="AB137" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC137" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD137" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE137" s="7"/>
+      <c r="AF137" s="7"/>
+      <c r="AG137" s="7"/>
+      <c r="AH137" s="7"/>
+      <c r="AI137" s="7"/>
+      <c r="AJ137" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK137" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="138" spans="1:37">
+      <c r="A138" s="3">
+        <v>136</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C138" s="3">
+        <v>2026092650</v>
+      </c>
+      <c r="D138" s="3"/>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3">
+        <v>5245</v>
+      </c>
+      <c r="G138" s="3" t="s">
+        <v>1020</v>
+      </c>
+      <c r="H138" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I138" s="3"/>
+      <c r="J138" s="3"/>
+      <c r="K138" s="3"/>
+      <c r="L138" s="3"/>
+      <c r="M138" s="4"/>
+      <c r="N138" s="3"/>
+      <c r="O138" s="4"/>
+      <c r="P138" s="4"/>
+      <c r="Q138" s="3" t="s">
+        <v>1021</v>
+      </c>
+      <c r="R138" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S138" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T138" s="3">
+        <v>1</v>
+      </c>
+      <c r="U138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V138" s="3" t="s">
+        <v>1022</v>
+      </c>
+      <c r="W138" s="3" t="s">
+        <v>1023</v>
+      </c>
+      <c r="X138" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="Y138" s="3"/>
+      <c r="Z138" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA138" s="3"/>
+      <c r="AB138" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC138" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD138" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE138" s="3"/>
+      <c r="AF138" s="3"/>
+      <c r="AG138" s="3"/>
+      <c r="AH138" s="3"/>
+      <c r="AI138" s="3"/>
+      <c r="AJ138" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK138" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09221114
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$138</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$145</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1025">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-18  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1069">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-22  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -3135,6 +3135,138 @@
   </si>
   <si>
     <t>2026-09-18 15:58:00</t>
+  </si>
+  <si>
+    <t>1C672115091901</t>
+  </si>
+  <si>
+    <t>C672</t>
+  </si>
+  <si>
+    <t>中和橋安店</t>
+  </si>
+  <si>
+    <t>2026-09-19 10:31:52</t>
+  </si>
+  <si>
+    <t>門市TM2 CCD掃描器(HC56IITR)線路鬆脫，一旦鬆脫時掃描任何商品條碼都無反應，目前使用膠帶黏貼後有稍微改善但仍會再鬆脫，TM重啟無法排除...還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0C672</t>
+  </si>
+  <si>
+    <t>2026-09-19 10:33:21</t>
+  </si>
+  <si>
+    <t>2026-09-21 16:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 16:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 13:00:00</t>
+  </si>
+  <si>
+    <t>轉接頭螺絲鬆動。鎖回正常操作</t>
+  </si>
+  <si>
+    <t>13551115091902</t>
+  </si>
+  <si>
+    <t>2026-09-19 15:22:55</t>
+  </si>
+  <si>
+    <t>印字不清</t>
+  </si>
+  <si>
+    <t>門市反應LIFE ET印票機(印票機L90)亮綠燈，但印票時字體模糊，已有重開重裝紙捲仍異常...需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-19 15:34:56</t>
+  </si>
+  <si>
+    <t>2026-09-22 09:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 10:10:00</t>
+  </si>
+  <si>
+    <t>新紙捲開封貼紙捲入，排除後測試正常</t>
+  </si>
+  <si>
+    <t>蘆洲希望店</t>
+  </si>
+  <si>
+    <t>THILF05354</t>
+  </si>
+  <si>
+    <t>2026-09-21 14:23:05</t>
+  </si>
+  <si>
+    <t>2026-09-21 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 14:20:00</t>
+  </si>
+  <si>
+    <t>D193</t>
+  </si>
+  <si>
+    <t>蘆洲權義店</t>
+  </si>
+  <si>
+    <t>THILF0D193</t>
+  </si>
+  <si>
+    <t>2026-09-21 15:01:55</t>
+  </si>
+  <si>
+    <t>2026-09-21 14:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 15:52:44</t>
+  </si>
+  <si>
+    <t>2026-09-21 15:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-21 15:50:00</t>
+  </si>
+  <si>
+    <t>永和貞寧店</t>
+  </si>
+  <si>
+    <t>THILF03968</t>
+  </si>
+  <si>
+    <t>2026-09-22 09:45:59</t>
+  </si>
+  <si>
+    <t>2026-09-22 09:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 09:42:00</t>
+  </si>
+  <si>
+    <t>C388</t>
+  </si>
+  <si>
+    <t>中和水源店</t>
+  </si>
+  <si>
+    <t>THILF0C388</t>
+  </si>
+  <si>
+    <t>2026-09-22 10:42:01</t>
+  </si>
+  <si>
+    <t>2026-09-22 10:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 10:40:00</t>
   </si>
 </sst>
 </file>
@@ -3548,7 +3680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK138"/>
+  <dimension ref="A1:AK145"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -15309,7 +15441,7 @@
       <c r="M138" s="4"/>
       <c r="N138" s="3"/>
       <c r="O138" s="4"/>
-      <c r="P138" s="4"/>
+      <c r="P138" s="10"/>
       <c r="Q138" s="3" t="s">
         <v>1021</v>
       </c>
@@ -15342,7 +15474,7 @@
       <c r="AB138" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC138" s="4" t="s">
+      <c r="AC138" s="10" t="s">
         <v>67</v>
       </c>
       <c r="AD138" s="3" t="s">
@@ -15357,6 +15489,595 @@
         <v>60</v>
       </c>
       <c r="AK138" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="139" spans="1:37">
+      <c r="A139" s="7">
+        <v>137</v>
+      </c>
+      <c r="B139" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C139" s="7">
+        <v>2026092691</v>
+      </c>
+      <c r="D139" s="7" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E139" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F139" s="7" t="s">
+        <v>1026</v>
+      </c>
+      <c r="G139" s="7" t="s">
+        <v>1027</v>
+      </c>
+      <c r="H139" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I139" s="7" t="s">
+        <v>1028</v>
+      </c>
+      <c r="J139" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="K139" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L139" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="M139" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="N139" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="O139" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="P139" s="9" t="s">
+        <v>1029</v>
+      </c>
+      <c r="Q139" s="7" t="s">
+        <v>1030</v>
+      </c>
+      <c r="R139" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S139" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T139" s="7">
+        <v>1</v>
+      </c>
+      <c r="U139" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V139" s="7" t="s">
+        <v>1031</v>
+      </c>
+      <c r="W139" s="7" t="s">
+        <v>1032</v>
+      </c>
+      <c r="X139" s="7" t="s">
+        <v>1033</v>
+      </c>
+      <c r="Y139" s="7" t="s">
+        <v>1034</v>
+      </c>
+      <c r="Z139" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA139" s="7"/>
+      <c r="AB139" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC139" s="9" t="s">
+        <v>1035</v>
+      </c>
+      <c r="AD139" s="7"/>
+      <c r="AE139" s="7"/>
+      <c r="AF139" s="7"/>
+      <c r="AG139" s="7"/>
+      <c r="AH139" s="7"/>
+      <c r="AI139" s="7"/>
+      <c r="AJ139" s="7"/>
+      <c r="AK139" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="140" spans="1:37">
+      <c r="A140" s="3">
+        <v>138</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C140" s="3">
+        <v>2026092697</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>1036</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F140" s="3">
+        <v>3551</v>
+      </c>
+      <c r="G140" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="H140" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I140" s="3" t="s">
+        <v>1037</v>
+      </c>
+      <c r="J140" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="K140" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L140" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M140" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N140" s="3">
+        <v>6002</v>
+      </c>
+      <c r="O140" s="4" t="s">
+        <v>1038</v>
+      </c>
+      <c r="P140" s="10" t="s">
+        <v>1039</v>
+      </c>
+      <c r="Q140" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="R140" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S140" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T140" s="3">
+        <v>1</v>
+      </c>
+      <c r="U140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V140" s="3" t="s">
+        <v>1040</v>
+      </c>
+      <c r="W140" s="3" t="s">
+        <v>1041</v>
+      </c>
+      <c r="X140" s="3" t="s">
+        <v>1042</v>
+      </c>
+      <c r="Y140" s="3" t="s">
+        <v>1034</v>
+      </c>
+      <c r="Z140" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA140" s="3"/>
+      <c r="AB140" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC140" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="AD140" s="3"/>
+      <c r="AE140" s="3"/>
+      <c r="AF140" s="3"/>
+      <c r="AG140" s="3"/>
+      <c r="AH140" s="3"/>
+      <c r="AI140" s="3"/>
+      <c r="AJ140" s="3"/>
+      <c r="AK140" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="141" spans="1:37">
+      <c r="A141" s="7">
+        <v>139</v>
+      </c>
+      <c r="B141" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C141" s="7">
+        <v>2026092828</v>
+      </c>
+      <c r="D141" s="7"/>
+      <c r="E141" s="7"/>
+      <c r="F141" s="7">
+        <v>5354</v>
+      </c>
+      <c r="G141" s="7" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H141" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="I141" s="7"/>
+      <c r="J141" s="7"/>
+      <c r="K141" s="7"/>
+      <c r="L141" s="7"/>
+      <c r="M141" s="8"/>
+      <c r="N141" s="7"/>
+      <c r="O141" s="8"/>
+      <c r="P141" s="9"/>
+      <c r="Q141" s="7" t="s">
+        <v>1045</v>
+      </c>
+      <c r="R141" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S141" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T141" s="7">
+        <v>1</v>
+      </c>
+      <c r="U141" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V141" s="7" t="s">
+        <v>1046</v>
+      </c>
+      <c r="W141" s="7" t="s">
+        <v>1047</v>
+      </c>
+      <c r="X141" s="7" t="s">
+        <v>1048</v>
+      </c>
+      <c r="Y141" s="7"/>
+      <c r="Z141" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA141" s="7"/>
+      <c r="AB141" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC141" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD141" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE141" s="7"/>
+      <c r="AF141" s="7"/>
+      <c r="AG141" s="7"/>
+      <c r="AH141" s="7"/>
+      <c r="AI141" s="7"/>
+      <c r="AJ141" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK141" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="142" spans="1:37">
+      <c r="A142" s="3">
+        <v>140</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C142" s="3">
+        <v>2026092848</v>
+      </c>
+      <c r="D142" s="3"/>
+      <c r="E142" s="3"/>
+      <c r="F142" s="3" t="s">
+        <v>1049</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>1050</v>
+      </c>
+      <c r="H142" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="I142" s="3"/>
+      <c r="J142" s="3"/>
+      <c r="K142" s="3"/>
+      <c r="L142" s="3"/>
+      <c r="M142" s="4"/>
+      <c r="N142" s="3"/>
+      <c r="O142" s="4"/>
+      <c r="P142" s="10"/>
+      <c r="Q142" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="R142" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S142" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T142" s="3">
+        <v>1</v>
+      </c>
+      <c r="U142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V142" s="3" t="s">
+        <v>1052</v>
+      </c>
+      <c r="W142" s="3" t="s">
+        <v>1053</v>
+      </c>
+      <c r="X142" s="3" t="s">
+        <v>1054</v>
+      </c>
+      <c r="Y142" s="3"/>
+      <c r="Z142" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA142" s="3"/>
+      <c r="AB142" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC142" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD142" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE142" s="3"/>
+      <c r="AF142" s="3"/>
+      <c r="AG142" s="3"/>
+      <c r="AH142" s="3"/>
+      <c r="AI142" s="3"/>
+      <c r="AJ142" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK142" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="143" spans="1:37">
+      <c r="A143" s="7">
+        <v>141</v>
+      </c>
+      <c r="B143" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C143" s="7">
+        <v>2026092867</v>
+      </c>
+      <c r="D143" s="7"/>
+      <c r="E143" s="7"/>
+      <c r="F143" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="G143" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="H143" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="I143" s="7"/>
+      <c r="J143" s="7"/>
+      <c r="K143" s="7"/>
+      <c r="L143" s="7"/>
+      <c r="M143" s="8"/>
+      <c r="N143" s="7"/>
+      <c r="O143" s="8"/>
+      <c r="P143" s="9"/>
+      <c r="Q143" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="R143" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S143" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T143" s="7">
+        <v>1</v>
+      </c>
+      <c r="U143" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V143" s="7" t="s">
+        <v>1055</v>
+      </c>
+      <c r="W143" s="7" t="s">
+        <v>1056</v>
+      </c>
+      <c r="X143" s="7" t="s">
+        <v>1057</v>
+      </c>
+      <c r="Y143" s="7"/>
+      <c r="Z143" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA143" s="7"/>
+      <c r="AB143" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC143" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD143" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE143" s="7"/>
+      <c r="AF143" s="7"/>
+      <c r="AG143" s="7"/>
+      <c r="AH143" s="7"/>
+      <c r="AI143" s="7"/>
+      <c r="AJ143" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK143" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="144" spans="1:37">
+      <c r="A144" s="3">
+        <v>142</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C144" s="3">
+        <v>2026092919</v>
+      </c>
+      <c r="D144" s="3"/>
+      <c r="E144" s="3"/>
+      <c r="F144" s="3">
+        <v>3968</v>
+      </c>
+      <c r="G144" s="3" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H144" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="I144" s="3"/>
+      <c r="J144" s="3"/>
+      <c r="K144" s="3"/>
+      <c r="L144" s="3"/>
+      <c r="M144" s="4"/>
+      <c r="N144" s="3"/>
+      <c r="O144" s="4"/>
+      <c r="P144" s="10"/>
+      <c r="Q144" s="3" t="s">
+        <v>1059</v>
+      </c>
+      <c r="R144" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S144" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T144" s="3">
+        <v>1</v>
+      </c>
+      <c r="U144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V144" s="3" t="s">
+        <v>1060</v>
+      </c>
+      <c r="W144" s="3" t="s">
+        <v>1061</v>
+      </c>
+      <c r="X144" s="3" t="s">
+        <v>1062</v>
+      </c>
+      <c r="Y144" s="3"/>
+      <c r="Z144" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA144" s="3"/>
+      <c r="AB144" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC144" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD144" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE144" s="3"/>
+      <c r="AF144" s="3"/>
+      <c r="AG144" s="3"/>
+      <c r="AH144" s="3"/>
+      <c r="AI144" s="3"/>
+      <c r="AJ144" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK144" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="145" spans="1:37">
+      <c r="A145" s="7">
+        <v>143</v>
+      </c>
+      <c r="B145" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C145" s="7">
+        <v>2026092928</v>
+      </c>
+      <c r="D145" s="7"/>
+      <c r="E145" s="7"/>
+      <c r="F145" s="7" t="s">
+        <v>1063</v>
+      </c>
+      <c r="G145" s="7" t="s">
+        <v>1064</v>
+      </c>
+      <c r="H145" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I145" s="7"/>
+      <c r="J145" s="7"/>
+      <c r="K145" s="7"/>
+      <c r="L145" s="7"/>
+      <c r="M145" s="8"/>
+      <c r="N145" s="7"/>
+      <c r="O145" s="8"/>
+      <c r="P145" s="8"/>
+      <c r="Q145" s="7" t="s">
+        <v>1065</v>
+      </c>
+      <c r="R145" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S145" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T145" s="7">
+        <v>1</v>
+      </c>
+      <c r="U145" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V145" s="7" t="s">
+        <v>1066</v>
+      </c>
+      <c r="W145" s="7" t="s">
+        <v>1067</v>
+      </c>
+      <c r="X145" s="7" t="s">
+        <v>1068</v>
+      </c>
+      <c r="Y145" s="7"/>
+      <c r="Z145" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA145" s="7"/>
+      <c r="AB145" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC145" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD145" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE145" s="7"/>
+      <c r="AF145" s="7"/>
+      <c r="AG145" s="7"/>
+      <c r="AH145" s="7"/>
+      <c r="AI145" s="7"/>
+      <c r="AJ145" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK145" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09221814
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$145</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$153</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1069">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1126">
   <si>
     <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-22  )</t>
   </si>
@@ -3209,6 +3209,38 @@
     <t>2026-09-21 14:20:00</t>
   </si>
   <si>
+    <t>E5060115092101</t>
+  </si>
+  <si>
+    <t>淡水魚市店</t>
+  </si>
+  <si>
+    <t>2026-09-21 13:57:16</t>
+  </si>
+  <si>
+    <t>門市反應tm1 ccd掃描器(HC56IITR)刷讀所有條碼都感應不良，需刷很多次才有反應，已有執行校正仍異常...請台芝到店協助(掃描無反應)09/21 14:12  請門市執行艘描器校正，稍晚確認...廖</t>
+  </si>
+  <si>
+    <t>THILF05060</t>
+  </si>
+  <si>
+    <t>2026-09-21 14:29:19</t>
+  </si>
+  <si>
+    <t>2026-09-22 12:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 13:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 18:29:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119010411
+換上8119014266</t>
+  </si>
+  <si>
     <t>D193</t>
   </si>
   <si>
@@ -3236,6 +3268,68 @@
     <t>2026-09-21 15:50:00</t>
   </si>
   <si>
+    <t>13008115092102</t>
+  </si>
+  <si>
+    <t>龜山香品店</t>
+  </si>
+  <si>
+    <t>2026-09-21 20:51:46</t>
+  </si>
+  <si>
+    <t>門市反應MMK四代機螢幕跟主機連接的螢幕蓋未上鎖，可隨意掀起來，影響到操作...需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF03008</t>
+  </si>
+  <si>
+    <t>2026-09-21 20:56:22</t>
+  </si>
+  <si>
+    <t>2026-09-22 13:57:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 14:27:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 00:56:00</t>
+  </si>
+  <si>
+    <t>現場已鎖上</t>
+  </si>
+  <si>
+    <t>E2749115092201</t>
+  </si>
+  <si>
+    <t>淡水灰瑤子</t>
+  </si>
+  <si>
+    <t>2026-09-22 06:12:33</t>
+  </si>
+  <si>
+    <t>門市反應TM2 CCD掃描器(HC56IITR、HC76TR)刷讀所有條碼都感應不良，已有執行校正仍異常....請台芝到店協助(每件物品都得感應個2-3次，還不一定刷的出，只能手動輸入貨號。)</t>
+  </si>
+  <si>
+    <t>THILF02749</t>
+  </si>
+  <si>
+    <t>2026-09-22 09:04:25</t>
+  </si>
+  <si>
+    <t>2026-09-22 11:37:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 12:07:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:04:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119007468
+換上8119014265</t>
+  </si>
+  <si>
     <t>永和貞寧店</t>
   </si>
   <si>
@@ -3267,6 +3361,87 @@
   </si>
   <si>
     <t>2026-09-22 10:40:00</t>
+  </si>
+  <si>
+    <t>中和和圓店</t>
+  </si>
+  <si>
+    <t>THILF02570</t>
+  </si>
+  <si>
+    <t>2026-09-22 12:08:33</t>
+  </si>
+  <si>
+    <t>2026-09-22 11:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 12:02:00</t>
+  </si>
+  <si>
+    <t>五股五工店</t>
+  </si>
+  <si>
+    <t>THILF02535</t>
+  </si>
+  <si>
+    <t>2026-09-22 14:43:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 14:30:00</t>
+  </si>
+  <si>
+    <t>PM1 PM2掃搶POC</t>
+  </si>
+  <si>
+    <t>TT01</t>
+  </si>
+  <si>
+    <t>五股訓練教室</t>
+  </si>
+  <si>
+    <t>THILF0TT01</t>
+  </si>
+  <si>
+    <t>2026-09-22 15:08:27</t>
+  </si>
+  <si>
+    <t>2026-09-22 15:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 15:28:17</t>
+  </si>
+  <si>
+    <t>2026-09-22 15:35:00</t>
+  </si>
+  <si>
+    <t>1C052115092201</t>
+  </si>
+  <si>
+    <t>2026-09-22 16:03:23</t>
+  </si>
+  <si>
+    <t>無法進紙、印表機無反應</t>
+  </si>
+  <si>
+    <t>門市反應SC雷射印表機(M6600NW)無法使用畫面跳到電話傳真的畫面但重啟設備拔插頭重差仍異常，且門市測試傳真也無法使用，重新拔插後方線路仍異常，查看SC印表機設定顯示離線....需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-22 16:08:09</t>
+  </si>
+  <si>
+    <t>2026-09-22 17:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 17:31:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 20:08:00</t>
+  </si>
+  <si>
+    <t>現場確認電話線路無聲音。 已請店家改報修中華電信。</t>
   </si>
 </sst>
 </file>
@@ -3680,7 +3855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK145"/>
+  <dimension ref="A1:AK153"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -15770,38 +15945,58 @@
         <v>140</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C142" s="3">
-        <v>2026092848</v>
-      </c>
-      <c r="D142" s="3"/>
-      <c r="E142" s="3"/>
-      <c r="F142" s="3" t="s">
+        <v>2026092832</v>
+      </c>
+      <c r="D142" s="3" t="s">
         <v>1049</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F142" s="3">
+        <v>5060</v>
       </c>
       <c r="G142" s="3" t="s">
         <v>1050</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="I142" s="3"/>
-      <c r="J142" s="3"/>
-      <c r="K142" s="3"/>
-      <c r="L142" s="3"/>
-      <c r="M142" s="4"/>
-      <c r="N142" s="3"/>
-      <c r="O142" s="4"/>
-      <c r="P142" s="10"/>
+        <v>730</v>
+      </c>
+      <c r="I142" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J142" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K142" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L142" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="M142" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="N142" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="O142" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P142" s="10" t="s">
+        <v>1052</v>
+      </c>
       <c r="Q142" s="3" t="s">
-        <v>1051</v>
+        <v>1053</v>
       </c>
       <c r="R142" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S142" s="3" t="s">
-        <v>320</v>
+        <v>92</v>
       </c>
       <c r="T142" s="3">
         <v>1</v>
@@ -15810,36 +16005,34 @@
         <v>53</v>
       </c>
       <c r="V142" s="3" t="s">
-        <v>1052</v>
+        <v>1054</v>
       </c>
       <c r="W142" s="3" t="s">
-        <v>1053</v>
+        <v>1055</v>
       </c>
       <c r="X142" s="3" t="s">
-        <v>1054</v>
-      </c>
-      <c r="Y142" s="3"/>
+        <v>1056</v>
+      </c>
+      <c r="Y142" s="3" t="s">
+        <v>1057</v>
+      </c>
       <c r="Z142" s="3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA142" s="3"/>
       <c r="AB142" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC142" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD142" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>1058</v>
+      </c>
+      <c r="AD142" s="3"/>
       <c r="AE142" s="3"/>
       <c r="AF142" s="3"/>
       <c r="AG142" s="3"/>
       <c r="AH142" s="3"/>
       <c r="AI142" s="3"/>
-      <c r="AJ142" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ142" s="3"/>
       <c r="AK142" s="3" t="s">
         <v>60</v>
       </c>
@@ -15852,15 +16045,15 @@
         <v>61</v>
       </c>
       <c r="C143" s="7">
-        <v>2026092867</v>
+        <v>2026092848</v>
       </c>
       <c r="D143" s="7"/>
       <c r="E143" s="7"/>
       <c r="F143" s="7" t="s">
-        <v>358</v>
+        <v>1059</v>
       </c>
       <c r="G143" s="7" t="s">
-        <v>359</v>
+        <v>1060</v>
       </c>
       <c r="H143" s="7" t="s">
         <v>360</v>
@@ -15874,7 +16067,7 @@
       <c r="O143" s="8"/>
       <c r="P143" s="9"/>
       <c r="Q143" s="7" t="s">
-        <v>364</v>
+        <v>1061</v>
       </c>
       <c r="R143" s="7" t="s">
         <v>51</v>
@@ -15889,17 +16082,17 @@
         <v>53</v>
       </c>
       <c r="V143" s="7" t="s">
-        <v>1055</v>
+        <v>1062</v>
       </c>
       <c r="W143" s="7" t="s">
-        <v>1056</v>
+        <v>1063</v>
       </c>
       <c r="X143" s="7" t="s">
-        <v>1057</v>
+        <v>1064</v>
       </c>
       <c r="Y143" s="7"/>
       <c r="Z143" s="7">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="AA143" s="7"/>
       <c r="AB143" s="7" t="s">
@@ -15931,18 +16124,18 @@
         <v>61</v>
       </c>
       <c r="C144" s="3">
-        <v>2026092919</v>
+        <v>2026092867</v>
       </c>
       <c r="D144" s="3"/>
       <c r="E144" s="3"/>
-      <c r="F144" s="3">
-        <v>3968</v>
+      <c r="F144" s="3" t="s">
+        <v>358</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>1058</v>
+        <v>359</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>263</v>
+        <v>360</v>
       </c>
       <c r="I144" s="3"/>
       <c r="J144" s="3"/>
@@ -15953,13 +16146,13 @@
       <c r="O144" s="4"/>
       <c r="P144" s="10"/>
       <c r="Q144" s="3" t="s">
-        <v>1059</v>
+        <v>364</v>
       </c>
       <c r="R144" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S144" s="3" t="s">
-        <v>52</v>
+        <v>320</v>
       </c>
       <c r="T144" s="3">
         <v>1</v>
@@ -15968,17 +16161,17 @@
         <v>53</v>
       </c>
       <c r="V144" s="3" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="W144" s="3" t="s">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="X144" s="3" t="s">
-        <v>1062</v>
+        <v>1067</v>
       </c>
       <c r="Y144" s="3"/>
       <c r="Z144" s="3">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="AA144" s="3"/>
       <c r="AB144" s="3" t="s">
@@ -16007,38 +16200,58 @@
         <v>143</v>
       </c>
       <c r="B145" s="7" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C145" s="7">
-        <v>2026092928</v>
-      </c>
-      <c r="D145" s="7"/>
-      <c r="E145" s="7"/>
-      <c r="F145" s="7" t="s">
-        <v>1063</v>
+        <v>2026092914</v>
+      </c>
+      <c r="D145" s="7" t="s">
+        <v>1068</v>
+      </c>
+      <c r="E145" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F145" s="7">
+        <v>3008</v>
       </c>
       <c r="G145" s="7" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="H145" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I145" s="7"/>
-      <c r="J145" s="7"/>
-      <c r="K145" s="7"/>
-      <c r="L145" s="7"/>
-      <c r="M145" s="8"/>
-      <c r="N145" s="7"/>
-      <c r="O145" s="8"/>
-      <c r="P145" s="8"/>
+        <v>90</v>
+      </c>
+      <c r="I145" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="J145" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="K145" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="L145" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M145" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="N145" s="7">
+        <v>5801</v>
+      </c>
+      <c r="O145" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="P145" s="9" t="s">
+        <v>1071</v>
+      </c>
       <c r="Q145" s="7" t="s">
-        <v>1065</v>
+        <v>1072</v>
       </c>
       <c r="R145" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S145" s="7" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="T145" s="7">
         <v>1</v>
@@ -16047,37 +16260,703 @@
         <v>53</v>
       </c>
       <c r="V145" s="7" t="s">
-        <v>1066</v>
+        <v>1073</v>
       </c>
       <c r="W145" s="7" t="s">
-        <v>1067</v>
+        <v>1074</v>
       </c>
       <c r="X145" s="7" t="s">
-        <v>1068</v>
-      </c>
-      <c r="Y145" s="7"/>
+        <v>1075</v>
+      </c>
+      <c r="Y145" s="7" t="s">
+        <v>1076</v>
+      </c>
       <c r="Z145" s="7">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA145" s="7"/>
       <c r="AB145" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC145" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD145" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AC145" s="9" t="s">
+        <v>1077</v>
+      </c>
+      <c r="AD145" s="7"/>
       <c r="AE145" s="7"/>
       <c r="AF145" s="7"/>
       <c r="AG145" s="7"/>
       <c r="AH145" s="7"/>
       <c r="AI145" s="7"/>
-      <c r="AJ145" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ145" s="7"/>
       <c r="AK145" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="146" spans="1:37">
+      <c r="A146" s="3">
+        <v>144</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C146" s="3">
+        <v>2026092917</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>1078</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F146" s="3">
+        <v>2749</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>1079</v>
+      </c>
+      <c r="H146" s="3" t="s">
+        <v>730</v>
+      </c>
+      <c r="I146" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="J146" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K146" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L146" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="M146" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="N146" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="O146" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P146" s="10" t="s">
+        <v>1081</v>
+      </c>
+      <c r="Q146" s="3" t="s">
+        <v>1082</v>
+      </c>
+      <c r="R146" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S146" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T146" s="3">
+        <v>1</v>
+      </c>
+      <c r="U146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V146" s="3" t="s">
+        <v>1083</v>
+      </c>
+      <c r="W146" s="3" t="s">
+        <v>1084</v>
+      </c>
+      <c r="X146" s="3" t="s">
+        <v>1085</v>
+      </c>
+      <c r="Y146" s="3" t="s">
+        <v>1086</v>
+      </c>
+      <c r="Z146" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA146" s="3"/>
+      <c r="AB146" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC146" s="10" t="s">
+        <v>1087</v>
+      </c>
+      <c r="AD146" s="3"/>
+      <c r="AE146" s="3"/>
+      <c r="AF146" s="3"/>
+      <c r="AG146" s="3"/>
+      <c r="AH146" s="3"/>
+      <c r="AI146" s="3"/>
+      <c r="AJ146" s="3"/>
+      <c r="AK146" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="147" spans="1:37">
+      <c r="A147" s="7">
+        <v>145</v>
+      </c>
+      <c r="B147" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C147" s="7">
+        <v>2026092919</v>
+      </c>
+      <c r="D147" s="7"/>
+      <c r="E147" s="7"/>
+      <c r="F147" s="7">
+        <v>3968</v>
+      </c>
+      <c r="G147" s="7" t="s">
+        <v>1088</v>
+      </c>
+      <c r="H147" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="I147" s="7"/>
+      <c r="J147" s="7"/>
+      <c r="K147" s="7"/>
+      <c r="L147" s="7"/>
+      <c r="M147" s="8"/>
+      <c r="N147" s="7"/>
+      <c r="O147" s="8"/>
+      <c r="P147" s="9"/>
+      <c r="Q147" s="7" t="s">
+        <v>1089</v>
+      </c>
+      <c r="R147" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S147" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T147" s="7">
+        <v>1</v>
+      </c>
+      <c r="U147" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V147" s="7" t="s">
+        <v>1090</v>
+      </c>
+      <c r="W147" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="X147" s="7" t="s">
+        <v>1092</v>
+      </c>
+      <c r="Y147" s="7"/>
+      <c r="Z147" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA147" s="7"/>
+      <c r="AB147" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC147" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD147" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE147" s="7"/>
+      <c r="AF147" s="7"/>
+      <c r="AG147" s="7"/>
+      <c r="AH147" s="7"/>
+      <c r="AI147" s="7"/>
+      <c r="AJ147" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK147" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="148" spans="1:37">
+      <c r="A148" s="3">
+        <v>146</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C148" s="3">
+        <v>2026092928</v>
+      </c>
+      <c r="D148" s="3"/>
+      <c r="E148" s="3"/>
+      <c r="F148" s="3" t="s">
+        <v>1093</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>1094</v>
+      </c>
+      <c r="H148" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I148" s="3"/>
+      <c r="J148" s="3"/>
+      <c r="K148" s="3"/>
+      <c r="L148" s="3"/>
+      <c r="M148" s="4"/>
+      <c r="N148" s="3"/>
+      <c r="O148" s="4"/>
+      <c r="P148" s="10"/>
+      <c r="Q148" s="3" t="s">
+        <v>1095</v>
+      </c>
+      <c r="R148" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S148" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T148" s="3">
+        <v>1</v>
+      </c>
+      <c r="U148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V148" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="W148" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="X148" s="3" t="s">
+        <v>1098</v>
+      </c>
+      <c r="Y148" s="3"/>
+      <c r="Z148" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA148" s="3"/>
+      <c r="AB148" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC148" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD148" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE148" s="3"/>
+      <c r="AF148" s="3"/>
+      <c r="AG148" s="3"/>
+      <c r="AH148" s="3"/>
+      <c r="AI148" s="3"/>
+      <c r="AJ148" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK148" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="149" spans="1:37">
+      <c r="A149" s="7">
+        <v>147</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C149" s="7">
+        <v>2026092978</v>
+      </c>
+      <c r="D149" s="7"/>
+      <c r="E149" s="7"/>
+      <c r="F149" s="7">
+        <v>2570</v>
+      </c>
+      <c r="G149" s="7" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H149" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I149" s="7"/>
+      <c r="J149" s="7"/>
+      <c r="K149" s="7"/>
+      <c r="L149" s="7"/>
+      <c r="M149" s="8"/>
+      <c r="N149" s="7"/>
+      <c r="O149" s="8"/>
+      <c r="P149" s="9"/>
+      <c r="Q149" s="7" t="s">
+        <v>1100</v>
+      </c>
+      <c r="R149" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S149" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T149" s="7">
+        <v>1</v>
+      </c>
+      <c r="U149" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V149" s="7" t="s">
+        <v>1101</v>
+      </c>
+      <c r="W149" s="7" t="s">
+        <v>1102</v>
+      </c>
+      <c r="X149" s="7" t="s">
+        <v>1103</v>
+      </c>
+      <c r="Y149" s="7"/>
+      <c r="Z149" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA149" s="7"/>
+      <c r="AB149" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC149" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD149" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE149" s="7"/>
+      <c r="AF149" s="7"/>
+      <c r="AG149" s="7"/>
+      <c r="AH149" s="7"/>
+      <c r="AI149" s="7"/>
+      <c r="AJ149" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK149" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="150" spans="1:37">
+      <c r="A150" s="3">
+        <v>148</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C150" s="3">
+        <v>2026093004</v>
+      </c>
+      <c r="D150" s="3"/>
+      <c r="E150" s="3"/>
+      <c r="F150" s="3">
+        <v>2535</v>
+      </c>
+      <c r="G150" s="3" t="s">
+        <v>1104</v>
+      </c>
+      <c r="H150" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="I150" s="3"/>
+      <c r="J150" s="3"/>
+      <c r="K150" s="3"/>
+      <c r="L150" s="3"/>
+      <c r="M150" s="4"/>
+      <c r="N150" s="3"/>
+      <c r="O150" s="4"/>
+      <c r="P150" s="10"/>
+      <c r="Q150" s="3" t="s">
+        <v>1105</v>
+      </c>
+      <c r="R150" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S150" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T150" s="3">
+        <v>1</v>
+      </c>
+      <c r="U150" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V150" s="3" t="s">
+        <v>1106</v>
+      </c>
+      <c r="W150" s="3" t="s">
+        <v>1107</v>
+      </c>
+      <c r="X150" s="3" t="s">
+        <v>1108</v>
+      </c>
+      <c r="Y150" s="3"/>
+      <c r="Z150" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA150" s="3"/>
+      <c r="AB150" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC150" s="10" t="s">
+        <v>1109</v>
+      </c>
+      <c r="AD150" s="3"/>
+      <c r="AE150" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF150" s="3"/>
+      <c r="AG150" s="3"/>
+      <c r="AH150" s="3"/>
+      <c r="AI150" s="3"/>
+      <c r="AJ150" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK150" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="151" spans="1:37">
+      <c r="A151" s="7">
+        <v>149</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C151" s="7">
+        <v>2026093028</v>
+      </c>
+      <c r="D151" s="7"/>
+      <c r="E151" s="7"/>
+      <c r="F151" s="7" t="s">
+        <v>1110</v>
+      </c>
+      <c r="G151" s="7" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H151" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="I151" s="7"/>
+      <c r="J151" s="7"/>
+      <c r="K151" s="7"/>
+      <c r="L151" s="7"/>
+      <c r="M151" s="8"/>
+      <c r="N151" s="7"/>
+      <c r="O151" s="8"/>
+      <c r="P151" s="9"/>
+      <c r="Q151" s="7" t="s">
+        <v>1112</v>
+      </c>
+      <c r="R151" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S151" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T151" s="7">
+        <v>1</v>
+      </c>
+      <c r="U151" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V151" s="7" t="s">
+        <v>1113</v>
+      </c>
+      <c r="W151" s="7" t="s">
+        <v>1108</v>
+      </c>
+      <c r="X151" s="7" t="s">
+        <v>1114</v>
+      </c>
+      <c r="Y151" s="7"/>
+      <c r="Z151" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="AA151" s="7"/>
+      <c r="AB151" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC151" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD151" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE151" s="7"/>
+      <c r="AF151" s="7"/>
+      <c r="AG151" s="7"/>
+      <c r="AH151" s="7"/>
+      <c r="AI151" s="7"/>
+      <c r="AJ151" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK151" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="152" spans="1:37">
+      <c r="A152" s="3">
+        <v>150</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C152" s="3">
+        <v>2026093032</v>
+      </c>
+      <c r="D152" s="3"/>
+      <c r="E152" s="3"/>
+      <c r="F152" s="3">
+        <v>2535</v>
+      </c>
+      <c r="G152" s="3" t="s">
+        <v>1104</v>
+      </c>
+      <c r="H152" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="I152" s="3"/>
+      <c r="J152" s="3"/>
+      <c r="K152" s="3"/>
+      <c r="L152" s="3"/>
+      <c r="M152" s="4"/>
+      <c r="N152" s="3"/>
+      <c r="O152" s="4"/>
+      <c r="P152" s="10"/>
+      <c r="Q152" s="3" t="s">
+        <v>1105</v>
+      </c>
+      <c r="R152" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S152" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T152" s="3">
+        <v>1</v>
+      </c>
+      <c r="U152" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V152" s="3" t="s">
+        <v>1115</v>
+      </c>
+      <c r="W152" s="3" t="s">
+        <v>1114</v>
+      </c>
+      <c r="X152" s="3" t="s">
+        <v>1116</v>
+      </c>
+      <c r="Y152" s="3"/>
+      <c r="Z152" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA152" s="3"/>
+      <c r="AB152" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC152" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD152" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE152" s="3"/>
+      <c r="AF152" s="3"/>
+      <c r="AG152" s="3"/>
+      <c r="AH152" s="3"/>
+      <c r="AI152" s="3"/>
+      <c r="AJ152" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK152" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="153" spans="1:37">
+      <c r="A153" s="7">
+        <v>151</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C153" s="7">
+        <v>2026093041</v>
+      </c>
+      <c r="D153" s="7" t="s">
+        <v>1117</v>
+      </c>
+      <c r="E153" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F153" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="G153" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="H153" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I153" s="7" t="s">
+        <v>1118</v>
+      </c>
+      <c r="J153" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K153" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L153" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="M153" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="N153" s="7">
+        <v>2702</v>
+      </c>
+      <c r="O153" s="8" t="s">
+        <v>1119</v>
+      </c>
+      <c r="P153" s="8" t="s">
+        <v>1120</v>
+      </c>
+      <c r="Q153" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="R153" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S153" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T153" s="7">
+        <v>1</v>
+      </c>
+      <c r="U153" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V153" s="7" t="s">
+        <v>1121</v>
+      </c>
+      <c r="W153" s="7" t="s">
+        <v>1122</v>
+      </c>
+      <c r="X153" s="7" t="s">
+        <v>1123</v>
+      </c>
+      <c r="Y153" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="Z153" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA153" s="7"/>
+      <c r="AB153" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC153" s="8" t="s">
+        <v>1125</v>
+      </c>
+      <c r="AD153" s="7"/>
+      <c r="AE153" s="7"/>
+      <c r="AF153" s="7"/>
+      <c r="AG153" s="7"/>
+      <c r="AH153" s="7"/>
+      <c r="AI153" s="7"/>
+      <c r="AJ153" s="7"/>
+      <c r="AK153" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09231747
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$153</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$166</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1126">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-22  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1203">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-23  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -3417,6 +3417,39 @@
     <t>2026-09-22 15:35:00</t>
   </si>
   <si>
+    <t>14933115092201</t>
+  </si>
+  <si>
+    <t>2026-09-22 15:39:10</t>
+  </si>
+  <si>
+    <t>HLN9</t>
+  </si>
+  <si>
+    <t>HL-電子看板機上盒</t>
+  </si>
+  <si>
+    <t>N901</t>
+  </si>
+  <si>
+    <t>門市反應咖啡價目電子看板畫面都會跳到應用程式畫面要門市做點選，門市重新調整訊號源後會正常但過個10到20分鐘後又跳掉，已有重啟數據機+店長桌前開關並休息20分鐘後仍黑畫面，查看內外部連線正常...2026/9/22 (週二) 下午 03:33總公司娟慧MAIL:4933龜山連莊店，請先派台芝更換機上盒，謝謝您.....還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-22 15:40:39</t>
+  </si>
+  <si>
+    <t>2026-09-23 12:21:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 12:51:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 19:40:00</t>
+  </si>
+  <si>
+    <t>現場檢測商顯無法正常開機，更換機上盒一樣無效，無更換機上盒</t>
+  </si>
+  <si>
     <t>1C052115092201</t>
   </si>
   <si>
@@ -3442,6 +3475,206 @@
   </si>
   <si>
     <t>現場確認電話線路無聲音。 已請店家改報修中華電信。</t>
+  </si>
+  <si>
+    <t>1C388115092201</t>
+  </si>
+  <si>
+    <t>2026-09-22 17:26:51</t>
+  </si>
+  <si>
+    <t>門市反應TM1收銀機(TCX800)(抽屜顏色:白色、鑰匙孔位子(中)、鎖頭編號:5001)抽屜關不起來..請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-22 17:28:47</t>
+  </si>
+  <si>
+    <t>2026-09-22 17:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-22 18:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 21:28:00</t>
+  </si>
+  <si>
+    <t>抽屜後方鐵柱歪斜。</t>
+  </si>
+  <si>
+    <t>13749115092201</t>
+  </si>
+  <si>
+    <t>2026-09-22 18:23:05</t>
+  </si>
+  <si>
+    <t>門市反應tm1(TCX800)經常觸控不良、都要點很多下或是點了之後要隔5~10秒才會有反應，確認無張貼文宣或商品壓到，且門市每天都會擦螢幕，此情況已有一段時間，先前有協助門市進行觸控校正，門市告知也沒有改善，9/14有派工台芝(案13749115091401),9/15台芝到店進行螢幕觸控校正後門市告知當下有好，但沒隔多久就又開始同情況，要求備註請工程師到店評估可否更換一台新主機......還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-22 18:26:38</t>
+  </si>
+  <si>
+    <t>2026-09-23 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:51:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 22:26:00</t>
+  </si>
+  <si>
+    <t>更換主機及更換第一顆不備份還原
+換下8185000818
+換上8185002866</t>
+  </si>
+  <si>
+    <t>蘆洲信義店</t>
+  </si>
+  <si>
+    <t>THILF03452</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:37:49</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:20:00</t>
+  </si>
+  <si>
+    <t>蘆洲切仔麵</t>
+  </si>
+  <si>
+    <t>THILF05341</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:50:16</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:40:00</t>
+  </si>
+  <si>
+    <t>蘆洲湧蓮店</t>
+  </si>
+  <si>
+    <t>THILF04218</t>
+  </si>
+  <si>
+    <t>2026-09-23 14:04:41</t>
+  </si>
+  <si>
+    <t>2026-09-23 13:41:00</t>
+  </si>
+  <si>
+    <t>D072</t>
+  </si>
+  <si>
+    <t>板橋僑福店</t>
+  </si>
+  <si>
+    <t>THILF0D072</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:28:54</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:28:00</t>
+  </si>
+  <si>
+    <t>D161</t>
+  </si>
+  <si>
+    <t>板橋僑中三</t>
+  </si>
+  <si>
+    <t>THILF0D161</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:49:35</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:46:00</t>
+  </si>
+  <si>
+    <t>板橋僑興店</t>
+  </si>
+  <si>
+    <t>THILF04145</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:11:20</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:48:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:59:00</t>
+  </si>
+  <si>
+    <t>中和泰和店</t>
+  </si>
+  <si>
+    <t>THILF02398</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:21:42</t>
+  </si>
+  <si>
+    <t>2026-09-23 11:00:00</t>
+  </si>
+  <si>
+    <t>裝潢回裝已完工</t>
+  </si>
+  <si>
+    <t>板橋板龍店</t>
+  </si>
+  <si>
+    <t>THILF02403</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:26:47</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:05:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:24:00</t>
+  </si>
+  <si>
+    <t>板橋海龍店</t>
+  </si>
+  <si>
+    <t>THILF03955</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:49:30</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:47:00</t>
+  </si>
+  <si>
+    <t>板橋互助店</t>
+  </si>
+  <si>
+    <t>THILF03853</t>
+  </si>
+  <si>
+    <t>2026-09-23 17:10:40</t>
+  </si>
+  <si>
+    <t>2026-09-23 16:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-23 17:08:00</t>
   </si>
 </sst>
 </file>
@@ -3855,7 +4088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK153"/>
+  <dimension ref="A1:AK166"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -16871,7 +17104,7 @@
         <v>38</v>
       </c>
       <c r="C153" s="7">
-        <v>2026093041</v>
+        <v>2026093035</v>
       </c>
       <c r="D153" s="7" t="s">
         <v>1117</v>
@@ -16879,14 +17112,14 @@
       <c r="E153" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F153" s="7" t="s">
-        <v>233</v>
+      <c r="F153" s="7">
+        <v>4933</v>
       </c>
       <c r="G153" s="7" t="s">
-        <v>234</v>
+        <v>493</v>
       </c>
       <c r="H153" s="7" t="s">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="I153" s="7" t="s">
         <v>1118</v>
@@ -16898,28 +17131,28 @@
         <v>45</v>
       </c>
       <c r="L153" s="7" t="s">
-        <v>237</v>
+        <v>1119</v>
       </c>
       <c r="M153" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="N153" s="7">
-        <v>2702</v>
+        <v>1120</v>
+      </c>
+      <c r="N153" s="7" t="s">
+        <v>1121</v>
       </c>
       <c r="O153" s="8" t="s">
-        <v>1119</v>
-      </c>
-      <c r="P153" s="8" t="s">
-        <v>1120</v>
+        <v>411</v>
+      </c>
+      <c r="P153" s="9" t="s">
+        <v>1122</v>
       </c>
       <c r="Q153" s="7" t="s">
-        <v>241</v>
+        <v>494</v>
       </c>
       <c r="R153" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S153" s="7" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="T153" s="7">
         <v>1</v>
@@ -16928,26 +17161,26 @@
         <v>53</v>
       </c>
       <c r="V153" s="7" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="W153" s="7" t="s">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="X153" s="7" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="Y153" s="7" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="Z153" s="7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA153" s="7"/>
       <c r="AB153" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC153" s="8" t="s">
-        <v>1125</v>
+      <c r="AC153" s="9" t="s">
+        <v>1127</v>
       </c>
       <c r="AD153" s="7"/>
       <c r="AE153" s="7"/>
@@ -16957,6 +17190,1073 @@
       <c r="AI153" s="7"/>
       <c r="AJ153" s="7"/>
       <c r="AK153" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="154" spans="1:37">
+      <c r="A154" s="3">
+        <v>152</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C154" s="3">
+        <v>2026093041</v>
+      </c>
+      <c r="D154" s="3" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E154" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="G154" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="H154" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I154" s="3" t="s">
+        <v>1129</v>
+      </c>
+      <c r="J154" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K154" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L154" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="M154" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="N154" s="3">
+        <v>2702</v>
+      </c>
+      <c r="O154" s="4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="P154" s="10" t="s">
+        <v>1131</v>
+      </c>
+      <c r="Q154" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="R154" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S154" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T154" s="3">
+        <v>1</v>
+      </c>
+      <c r="U154" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V154" s="3" t="s">
+        <v>1132</v>
+      </c>
+      <c r="W154" s="3" t="s">
+        <v>1133</v>
+      </c>
+      <c r="X154" s="3" t="s">
+        <v>1134</v>
+      </c>
+      <c r="Y154" s="3" t="s">
+        <v>1135</v>
+      </c>
+      <c r="Z154" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA154" s="3"/>
+      <c r="AB154" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC154" s="10" t="s">
+        <v>1136</v>
+      </c>
+      <c r="AD154" s="3"/>
+      <c r="AE154" s="3"/>
+      <c r="AF154" s="3"/>
+      <c r="AG154" s="3"/>
+      <c r="AH154" s="3"/>
+      <c r="AI154" s="3"/>
+      <c r="AJ154" s="3"/>
+      <c r="AK154" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="155" spans="1:37">
+      <c r="A155" s="7">
+        <v>153</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C155" s="7">
+        <v>2026093047</v>
+      </c>
+      <c r="D155" s="7" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E155" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F155" s="7" t="s">
+        <v>1093</v>
+      </c>
+      <c r="G155" s="7" t="s">
+        <v>1094</v>
+      </c>
+      <c r="H155" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I155" s="7" t="s">
+        <v>1138</v>
+      </c>
+      <c r="J155" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K155" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L155" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M155" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N155" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O155" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="P155" s="9" t="s">
+        <v>1139</v>
+      </c>
+      <c r="Q155" s="7" t="s">
+        <v>1095</v>
+      </c>
+      <c r="R155" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S155" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T155" s="7">
+        <v>1</v>
+      </c>
+      <c r="U155" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V155" s="7" t="s">
+        <v>1140</v>
+      </c>
+      <c r="W155" s="7" t="s">
+        <v>1141</v>
+      </c>
+      <c r="X155" s="7" t="s">
+        <v>1142</v>
+      </c>
+      <c r="Y155" s="7" t="s">
+        <v>1143</v>
+      </c>
+      <c r="Z155" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA155" s="7"/>
+      <c r="AB155" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC155" s="9" t="s">
+        <v>1144</v>
+      </c>
+      <c r="AD155" s="7"/>
+      <c r="AE155" s="7"/>
+      <c r="AF155" s="7"/>
+      <c r="AG155" s="7"/>
+      <c r="AH155" s="7"/>
+      <c r="AI155" s="7"/>
+      <c r="AJ155" s="7"/>
+      <c r="AK155" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="156" spans="1:37">
+      <c r="A156" s="3">
+        <v>154</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C156" s="3">
+        <v>2026093050</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E156" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F156" s="3">
+        <v>3749</v>
+      </c>
+      <c r="G156" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="H156" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I156" s="3" t="s">
+        <v>1146</v>
+      </c>
+      <c r="J156" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K156" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L156" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M156" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N156" s="3">
+        <v>2307</v>
+      </c>
+      <c r="O156" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="P156" s="10" t="s">
+        <v>1147</v>
+      </c>
+      <c r="Q156" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="R156" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S156" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T156" s="3">
+        <v>1</v>
+      </c>
+      <c r="U156" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V156" s="3" t="s">
+        <v>1148</v>
+      </c>
+      <c r="W156" s="3" t="s">
+        <v>1149</v>
+      </c>
+      <c r="X156" s="3" t="s">
+        <v>1150</v>
+      </c>
+      <c r="Y156" s="3" t="s">
+        <v>1151</v>
+      </c>
+      <c r="Z156" s="3">
+        <v>1.9</v>
+      </c>
+      <c r="AA156" s="3"/>
+      <c r="AB156" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC156" s="10" t="s">
+        <v>1152</v>
+      </c>
+      <c r="AD156" s="3"/>
+      <c r="AE156" s="3"/>
+      <c r="AF156" s="3"/>
+      <c r="AG156" s="3"/>
+      <c r="AH156" s="3"/>
+      <c r="AI156" s="3"/>
+      <c r="AJ156" s="3"/>
+      <c r="AK156" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="157" spans="1:37">
+      <c r="A157" s="7">
+        <v>155</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C157" s="7">
+        <v>2026093122</v>
+      </c>
+      <c r="D157" s="7"/>
+      <c r="E157" s="7"/>
+      <c r="F157" s="7">
+        <v>3452</v>
+      </c>
+      <c r="G157" s="7" t="s">
+        <v>1153</v>
+      </c>
+      <c r="H157" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="I157" s="7"/>
+      <c r="J157" s="7"/>
+      <c r="K157" s="7"/>
+      <c r="L157" s="7"/>
+      <c r="M157" s="8"/>
+      <c r="N157" s="7"/>
+      <c r="O157" s="8"/>
+      <c r="P157" s="9"/>
+      <c r="Q157" s="7" t="s">
+        <v>1154</v>
+      </c>
+      <c r="R157" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S157" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T157" s="7">
+        <v>1</v>
+      </c>
+      <c r="U157" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V157" s="7" t="s">
+        <v>1155</v>
+      </c>
+      <c r="W157" s="7" t="s">
+        <v>1156</v>
+      </c>
+      <c r="X157" s="7" t="s">
+        <v>1157</v>
+      </c>
+      <c r="Y157" s="7"/>
+      <c r="Z157" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA157" s="7"/>
+      <c r="AB157" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC157" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD157" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE157" s="7"/>
+      <c r="AF157" s="7"/>
+      <c r="AG157" s="7"/>
+      <c r="AH157" s="7"/>
+      <c r="AI157" s="7"/>
+      <c r="AJ157" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK157" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="158" spans="1:37">
+      <c r="A158" s="3">
+        <v>156</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C158" s="3">
+        <v>2026093123</v>
+      </c>
+      <c r="D158" s="3"/>
+      <c r="E158" s="3"/>
+      <c r="F158" s="3">
+        <v>5341</v>
+      </c>
+      <c r="G158" s="3" t="s">
+        <v>1158</v>
+      </c>
+      <c r="H158" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="I158" s="3"/>
+      <c r="J158" s="3"/>
+      <c r="K158" s="3"/>
+      <c r="L158" s="3"/>
+      <c r="M158" s="4"/>
+      <c r="N158" s="3"/>
+      <c r="O158" s="4"/>
+      <c r="P158" s="10"/>
+      <c r="Q158" s="3" t="s">
+        <v>1159</v>
+      </c>
+      <c r="R158" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S158" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T158" s="3">
+        <v>1</v>
+      </c>
+      <c r="U158" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V158" s="3" t="s">
+        <v>1160</v>
+      </c>
+      <c r="W158" s="3" t="s">
+        <v>1157</v>
+      </c>
+      <c r="X158" s="3" t="s">
+        <v>1161</v>
+      </c>
+      <c r="Y158" s="3"/>
+      <c r="Z158" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA158" s="3"/>
+      <c r="AB158" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC158" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD158" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE158" s="3"/>
+      <c r="AF158" s="3"/>
+      <c r="AG158" s="3"/>
+      <c r="AH158" s="3"/>
+      <c r="AI158" s="3"/>
+      <c r="AJ158" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK158" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="159" spans="1:37">
+      <c r="A159" s="7">
+        <v>157</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C159" s="7">
+        <v>2026093124</v>
+      </c>
+      <c r="D159" s="7"/>
+      <c r="E159" s="7"/>
+      <c r="F159" s="7">
+        <v>4218</v>
+      </c>
+      <c r="G159" s="7" t="s">
+        <v>1162</v>
+      </c>
+      <c r="H159" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="I159" s="7"/>
+      <c r="J159" s="7"/>
+      <c r="K159" s="7"/>
+      <c r="L159" s="7"/>
+      <c r="M159" s="8"/>
+      <c r="N159" s="7"/>
+      <c r="O159" s="8"/>
+      <c r="P159" s="9"/>
+      <c r="Q159" s="7" t="s">
+        <v>1163</v>
+      </c>
+      <c r="R159" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S159" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T159" s="7">
+        <v>1</v>
+      </c>
+      <c r="U159" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V159" s="7" t="s">
+        <v>1164</v>
+      </c>
+      <c r="W159" s="7" t="s">
+        <v>1165</v>
+      </c>
+      <c r="X159" s="7" t="s">
+        <v>1149</v>
+      </c>
+      <c r="Y159" s="7"/>
+      <c r="Z159" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA159" s="7"/>
+      <c r="AB159" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC159" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD159" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE159" s="7"/>
+      <c r="AF159" s="7"/>
+      <c r="AG159" s="7"/>
+      <c r="AH159" s="7"/>
+      <c r="AI159" s="7"/>
+      <c r="AJ159" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK159" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="160" spans="1:37">
+      <c r="A160" s="3">
+        <v>158</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C160" s="3">
+        <v>2026093144</v>
+      </c>
+      <c r="D160" s="3"/>
+      <c r="E160" s="3"/>
+      <c r="F160" s="3" t="s">
+        <v>1166</v>
+      </c>
+      <c r="G160" s="3" t="s">
+        <v>1167</v>
+      </c>
+      <c r="H160" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I160" s="3"/>
+      <c r="J160" s="3"/>
+      <c r="K160" s="3"/>
+      <c r="L160" s="3"/>
+      <c r="M160" s="4"/>
+      <c r="N160" s="3"/>
+      <c r="O160" s="4"/>
+      <c r="P160" s="10"/>
+      <c r="Q160" s="3" t="s">
+        <v>1168</v>
+      </c>
+      <c r="R160" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S160" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T160" s="3">
+        <v>1</v>
+      </c>
+      <c r="U160" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V160" s="3" t="s">
+        <v>1169</v>
+      </c>
+      <c r="W160" s="3" t="s">
+        <v>1170</v>
+      </c>
+      <c r="X160" s="3" t="s">
+        <v>1171</v>
+      </c>
+      <c r="Y160" s="3"/>
+      <c r="Z160" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA160" s="3"/>
+      <c r="AB160" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC160" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD160" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE160" s="3"/>
+      <c r="AF160" s="3"/>
+      <c r="AG160" s="3"/>
+      <c r="AH160" s="3"/>
+      <c r="AI160" s="3"/>
+      <c r="AJ160" s="3"/>
+      <c r="AK160" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="161" spans="1:37">
+      <c r="A161" s="7">
+        <v>159</v>
+      </c>
+      <c r="B161" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C161" s="7">
+        <v>2026093151</v>
+      </c>
+      <c r="D161" s="7"/>
+      <c r="E161" s="7"/>
+      <c r="F161" s="7" t="s">
+        <v>1172</v>
+      </c>
+      <c r="G161" s="7" t="s">
+        <v>1173</v>
+      </c>
+      <c r="H161" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I161" s="7"/>
+      <c r="J161" s="7"/>
+      <c r="K161" s="7"/>
+      <c r="L161" s="7"/>
+      <c r="M161" s="8"/>
+      <c r="N161" s="7"/>
+      <c r="O161" s="8"/>
+      <c r="P161" s="9"/>
+      <c r="Q161" s="7" t="s">
+        <v>1174</v>
+      </c>
+      <c r="R161" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S161" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T161" s="7">
+        <v>1</v>
+      </c>
+      <c r="U161" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V161" s="7" t="s">
+        <v>1175</v>
+      </c>
+      <c r="W161" s="7" t="s">
+        <v>1176</v>
+      </c>
+      <c r="X161" s="7" t="s">
+        <v>1177</v>
+      </c>
+      <c r="Y161" s="7"/>
+      <c r="Z161" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA161" s="7"/>
+      <c r="AB161" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC161" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD161" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE161" s="7"/>
+      <c r="AF161" s="7"/>
+      <c r="AG161" s="7"/>
+      <c r="AH161" s="7"/>
+      <c r="AI161" s="7"/>
+      <c r="AJ161" s="7"/>
+      <c r="AK161" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="162" spans="1:37">
+      <c r="A162" s="3">
+        <v>160</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C162" s="3">
+        <v>2026093158</v>
+      </c>
+      <c r="D162" s="3"/>
+      <c r="E162" s="3"/>
+      <c r="F162" s="3">
+        <v>4145</v>
+      </c>
+      <c r="G162" s="3" t="s">
+        <v>1178</v>
+      </c>
+      <c r="H162" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I162" s="3"/>
+      <c r="J162" s="3"/>
+      <c r="K162" s="3"/>
+      <c r="L162" s="3"/>
+      <c r="M162" s="4"/>
+      <c r="N162" s="3"/>
+      <c r="O162" s="4"/>
+      <c r="P162" s="10"/>
+      <c r="Q162" s="3" t="s">
+        <v>1179</v>
+      </c>
+      <c r="R162" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S162" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T162" s="3">
+        <v>1</v>
+      </c>
+      <c r="U162" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V162" s="3" t="s">
+        <v>1180</v>
+      </c>
+      <c r="W162" s="3" t="s">
+        <v>1181</v>
+      </c>
+      <c r="X162" s="3" t="s">
+        <v>1182</v>
+      </c>
+      <c r="Y162" s="3"/>
+      <c r="Z162" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA162" s="3"/>
+      <c r="AB162" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC162" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD162" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE162" s="3"/>
+      <c r="AF162" s="3"/>
+      <c r="AG162" s="3"/>
+      <c r="AH162" s="3"/>
+      <c r="AI162" s="3"/>
+      <c r="AJ162" s="3"/>
+      <c r="AK162" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="163" spans="1:37">
+      <c r="A163" s="7">
+        <v>161</v>
+      </c>
+      <c r="B163" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C163" s="7">
+        <v>2026093159</v>
+      </c>
+      <c r="D163" s="7"/>
+      <c r="E163" s="7"/>
+      <c r="F163" s="7">
+        <v>2398</v>
+      </c>
+      <c r="G163" s="7" t="s">
+        <v>1183</v>
+      </c>
+      <c r="H163" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I163" s="7"/>
+      <c r="J163" s="7"/>
+      <c r="K163" s="7"/>
+      <c r="L163" s="7"/>
+      <c r="M163" s="8"/>
+      <c r="N163" s="7"/>
+      <c r="O163" s="8"/>
+      <c r="P163" s="9"/>
+      <c r="Q163" s="7" t="s">
+        <v>1184</v>
+      </c>
+      <c r="R163" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S163" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T163" s="7">
+        <v>1</v>
+      </c>
+      <c r="U163" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V163" s="7" t="s">
+        <v>1185</v>
+      </c>
+      <c r="W163" s="7" t="s">
+        <v>1186</v>
+      </c>
+      <c r="X163" s="7" t="s">
+        <v>1176</v>
+      </c>
+      <c r="Y163" s="7"/>
+      <c r="Z163" s="7">
+        <v>4.5</v>
+      </c>
+      <c r="AA163" s="7"/>
+      <c r="AB163" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC163" s="9" t="s">
+        <v>1187</v>
+      </c>
+      <c r="AD163" s="7"/>
+      <c r="AE163" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF163" s="7"/>
+      <c r="AG163" s="7"/>
+      <c r="AH163" s="7"/>
+      <c r="AI163" s="7"/>
+      <c r="AJ163" s="7"/>
+      <c r="AK163" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="164" spans="1:37">
+      <c r="A164" s="3">
+        <v>162</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C164" s="3">
+        <v>2026093177</v>
+      </c>
+      <c r="D164" s="3"/>
+      <c r="E164" s="3"/>
+      <c r="F164" s="3">
+        <v>2403</v>
+      </c>
+      <c r="G164" s="3" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H164" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I164" s="3"/>
+      <c r="J164" s="3"/>
+      <c r="K164" s="3"/>
+      <c r="L164" s="3"/>
+      <c r="M164" s="4"/>
+      <c r="N164" s="3"/>
+      <c r="O164" s="4"/>
+      <c r="P164" s="10"/>
+      <c r="Q164" s="3" t="s">
+        <v>1189</v>
+      </c>
+      <c r="R164" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S164" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T164" s="3">
+        <v>1</v>
+      </c>
+      <c r="U164" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V164" s="3" t="s">
+        <v>1190</v>
+      </c>
+      <c r="W164" s="3" t="s">
+        <v>1191</v>
+      </c>
+      <c r="X164" s="3" t="s">
+        <v>1192</v>
+      </c>
+      <c r="Y164" s="3"/>
+      <c r="Z164" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA164" s="3"/>
+      <c r="AB164" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC164" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD164" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE164" s="3"/>
+      <c r="AF164" s="3"/>
+      <c r="AG164" s="3"/>
+      <c r="AH164" s="3"/>
+      <c r="AI164" s="3"/>
+      <c r="AJ164" s="3"/>
+      <c r="AK164" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="165" spans="1:37">
+      <c r="A165" s="7">
+        <v>163</v>
+      </c>
+      <c r="B165" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C165" s="7">
+        <v>2026093198</v>
+      </c>
+      <c r="D165" s="7"/>
+      <c r="E165" s="7"/>
+      <c r="F165" s="7">
+        <v>3955</v>
+      </c>
+      <c r="G165" s="7" t="s">
+        <v>1193</v>
+      </c>
+      <c r="H165" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I165" s="7"/>
+      <c r="J165" s="7"/>
+      <c r="K165" s="7"/>
+      <c r="L165" s="7"/>
+      <c r="M165" s="8"/>
+      <c r="N165" s="7"/>
+      <c r="O165" s="8"/>
+      <c r="P165" s="9"/>
+      <c r="Q165" s="7" t="s">
+        <v>1194</v>
+      </c>
+      <c r="R165" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S165" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T165" s="7">
+        <v>1</v>
+      </c>
+      <c r="U165" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V165" s="7" t="s">
+        <v>1195</v>
+      </c>
+      <c r="W165" s="7" t="s">
+        <v>1196</v>
+      </c>
+      <c r="X165" s="7" t="s">
+        <v>1197</v>
+      </c>
+      <c r="Y165" s="7"/>
+      <c r="Z165" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA165" s="7"/>
+      <c r="AB165" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC165" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD165" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE165" s="7"/>
+      <c r="AF165" s="7"/>
+      <c r="AG165" s="7"/>
+      <c r="AH165" s="7"/>
+      <c r="AI165" s="7"/>
+      <c r="AJ165" s="7"/>
+      <c r="AK165" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="166" spans="1:37">
+      <c r="A166" s="3">
+        <v>164</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C166" s="3">
+        <v>2026093210</v>
+      </c>
+      <c r="D166" s="3"/>
+      <c r="E166" s="3"/>
+      <c r="F166" s="3">
+        <v>3853</v>
+      </c>
+      <c r="G166" s="3" t="s">
+        <v>1198</v>
+      </c>
+      <c r="H166" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I166" s="3"/>
+      <c r="J166" s="3"/>
+      <c r="K166" s="3"/>
+      <c r="L166" s="3"/>
+      <c r="M166" s="4"/>
+      <c r="N166" s="3"/>
+      <c r="O166" s="4"/>
+      <c r="P166" s="4"/>
+      <c r="Q166" s="3" t="s">
+        <v>1199</v>
+      </c>
+      <c r="R166" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S166" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T166" s="3">
+        <v>1</v>
+      </c>
+      <c r="U166" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V166" s="3" t="s">
+        <v>1200</v>
+      </c>
+      <c r="W166" s="3" t="s">
+        <v>1201</v>
+      </c>
+      <c r="X166" s="3" t="s">
+        <v>1202</v>
+      </c>
+      <c r="Y166" s="3"/>
+      <c r="Z166" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA166" s="3"/>
+      <c r="AB166" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC166" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD166" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE166" s="3"/>
+      <c r="AF166" s="3"/>
+      <c r="AG166" s="3"/>
+      <c r="AH166" s="3"/>
+      <c r="AI166" s="3"/>
+      <c r="AJ166" s="3"/>
+      <c r="AK166" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09241129
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$166</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$167</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1203">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-23  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1216">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-24  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -3564,6 +3564,45 @@
   </si>
   <si>
     <t>2026-09-23 13:41:00</t>
+  </si>
+  <si>
+    <t>15536115092301</t>
+  </si>
+  <si>
+    <t>新莊青山店</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:06:44</t>
+  </si>
+  <si>
+    <t>HLF3</t>
+  </si>
+  <si>
+    <t>HL-LIFE-ET QRcode掃描器</t>
+  </si>
+  <si>
+    <t>F301</t>
+  </si>
+  <si>
+    <t>門市反應mmk QRCODE掃描器無法使用未亮燈，門市已有自行重啟、客服協助遠端重啟，請門市操作掃描器測試仍無反應未亮燈....需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF05536</t>
+  </si>
+  <si>
+    <t>2026-09-23 15:16:48</t>
+  </si>
+  <si>
+    <t>2026-09-24 09:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 19:16:00</t>
+  </si>
+  <si>
+    <t>重拔插排線 測試正常</t>
   </si>
   <si>
     <t>D072</t>
@@ -4088,7 +4127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK166"/>
+  <dimension ref="A1:AK167"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -17726,38 +17765,58 @@
         <v>158</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C160" s="3">
-        <v>2026093144</v>
-      </c>
-      <c r="D160" s="3"/>
-      <c r="E160" s="3"/>
-      <c r="F160" s="3" t="s">
+        <v>2026093140</v>
+      </c>
+      <c r="D160" s="3" t="s">
         <v>1166</v>
+      </c>
+      <c r="E160" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F160" s="3">
+        <v>5536</v>
       </c>
       <c r="G160" s="3" t="s">
         <v>1167</v>
       </c>
       <c r="H160" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="I160" s="3"/>
-      <c r="J160" s="3"/>
-      <c r="K160" s="3"/>
-      <c r="L160" s="3"/>
-      <c r="M160" s="4"/>
-      <c r="N160" s="3"/>
-      <c r="O160" s="4"/>
-      <c r="P160" s="10"/>
+        <v>328</v>
+      </c>
+      <c r="I160" s="3" t="s">
+        <v>1168</v>
+      </c>
+      <c r="J160" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K160" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L160" s="3" t="s">
+        <v>1169</v>
+      </c>
+      <c r="M160" s="4" t="s">
+        <v>1170</v>
+      </c>
+      <c r="N160" s="3" t="s">
+        <v>1171</v>
+      </c>
+      <c r="O160" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P160" s="10" t="s">
+        <v>1172</v>
+      </c>
       <c r="Q160" s="3" t="s">
-        <v>1168</v>
+        <v>1173</v>
       </c>
       <c r="R160" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S160" s="3" t="s">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="T160" s="3">
         <v>1</v>
@@ -17766,28 +17825,28 @@
         <v>53</v>
       </c>
       <c r="V160" s="3" t="s">
-        <v>1169</v>
+        <v>1174</v>
       </c>
       <c r="W160" s="3" t="s">
-        <v>1170</v>
+        <v>1175</v>
       </c>
       <c r="X160" s="3" t="s">
-        <v>1171</v>
-      </c>
-      <c r="Y160" s="3"/>
+        <v>1176</v>
+      </c>
+      <c r="Y160" s="3" t="s">
+        <v>1177</v>
+      </c>
       <c r="Z160" s="3">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="AA160" s="3"/>
       <c r="AB160" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC160" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD160" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>1178</v>
+      </c>
+      <c r="AD160" s="3"/>
       <c r="AE160" s="3"/>
       <c r="AF160" s="3"/>
       <c r="AG160" s="3"/>
@@ -17806,15 +17865,15 @@
         <v>61</v>
       </c>
       <c r="C161" s="7">
-        <v>2026093151</v>
+        <v>2026093144</v>
       </c>
       <c r="D161" s="7"/>
       <c r="E161" s="7"/>
       <c r="F161" s="7" t="s">
-        <v>1172</v>
+        <v>1179</v>
       </c>
       <c r="G161" s="7" t="s">
-        <v>1173</v>
+        <v>1180</v>
       </c>
       <c r="H161" s="7" t="s">
         <v>153</v>
@@ -17828,7 +17887,7 @@
       <c r="O161" s="8"/>
       <c r="P161" s="9"/>
       <c r="Q161" s="7" t="s">
-        <v>1174</v>
+        <v>1181</v>
       </c>
       <c r="R161" s="7" t="s">
         <v>51</v>
@@ -17843,17 +17902,17 @@
         <v>53</v>
       </c>
       <c r="V161" s="7" t="s">
-        <v>1175</v>
+        <v>1182</v>
       </c>
       <c r="W161" s="7" t="s">
-        <v>1176</v>
+        <v>1183</v>
       </c>
       <c r="X161" s="7" t="s">
-        <v>1177</v>
+        <v>1184</v>
       </c>
       <c r="Y161" s="7"/>
       <c r="Z161" s="7">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="AA161" s="7"/>
       <c r="AB161" s="7" t="s">
@@ -17883,15 +17942,15 @@
         <v>61</v>
       </c>
       <c r="C162" s="3">
-        <v>2026093158</v>
+        <v>2026093151</v>
       </c>
       <c r="D162" s="3"/>
       <c r="E162" s="3"/>
-      <c r="F162" s="3">
-        <v>4145</v>
+      <c r="F162" s="3" t="s">
+        <v>1185</v>
       </c>
       <c r="G162" s="3" t="s">
-        <v>1178</v>
+        <v>1186</v>
       </c>
       <c r="H162" s="3" t="s">
         <v>153</v>
@@ -17905,7 +17964,7 @@
       <c r="O162" s="4"/>
       <c r="P162" s="10"/>
       <c r="Q162" s="3" t="s">
-        <v>1179</v>
+        <v>1187</v>
       </c>
       <c r="R162" s="3" t="s">
         <v>51</v>
@@ -17920,17 +17979,17 @@
         <v>53</v>
       </c>
       <c r="V162" s="3" t="s">
-        <v>1180</v>
+        <v>1188</v>
       </c>
       <c r="W162" s="3" t="s">
-        <v>1181</v>
+        <v>1189</v>
       </c>
       <c r="X162" s="3" t="s">
-        <v>1182</v>
+        <v>1190</v>
       </c>
       <c r="Y162" s="3"/>
       <c r="Z162" s="3">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="AA162" s="3"/>
       <c r="AB162" s="3" t="s">
@@ -17960,18 +18019,18 @@
         <v>61</v>
       </c>
       <c r="C163" s="7">
-        <v>2026093159</v>
+        <v>2026093158</v>
       </c>
       <c r="D163" s="7"/>
       <c r="E163" s="7"/>
       <c r="F163" s="7">
-        <v>2398</v>
+        <v>4145</v>
       </c>
       <c r="G163" s="7" t="s">
-        <v>1183</v>
+        <v>1191</v>
       </c>
       <c r="H163" s="7" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="I163" s="7"/>
       <c r="J163" s="7"/>
@@ -17982,13 +18041,13 @@
       <c r="O163" s="8"/>
       <c r="P163" s="9"/>
       <c r="Q163" s="7" t="s">
-        <v>1184</v>
+        <v>1192</v>
       </c>
       <c r="R163" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S163" s="7" t="s">
-        <v>52</v>
+        <v>160</v>
       </c>
       <c r="T163" s="7">
         <v>1</v>
@@ -17997,29 +18056,29 @@
         <v>53</v>
       </c>
       <c r="V163" s="7" t="s">
-        <v>1185</v>
+        <v>1193</v>
       </c>
       <c r="W163" s="7" t="s">
-        <v>1186</v>
+        <v>1194</v>
       </c>
       <c r="X163" s="7" t="s">
-        <v>1176</v>
+        <v>1195</v>
       </c>
       <c r="Y163" s="7"/>
       <c r="Z163" s="7">
-        <v>4.5</v>
+        <v>0.2</v>
       </c>
       <c r="AA163" s="7"/>
       <c r="AB163" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC163" s="9" t="s">
-        <v>1187</v>
-      </c>
-      <c r="AD163" s="7"/>
-      <c r="AE163" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="AD163" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE163" s="7"/>
       <c r="AF163" s="7"/>
       <c r="AG163" s="7"/>
       <c r="AH163" s="7"/>
@@ -18037,18 +18096,18 @@
         <v>61</v>
       </c>
       <c r="C164" s="3">
-        <v>2026093177</v>
+        <v>2026093159</v>
       </c>
       <c r="D164" s="3"/>
       <c r="E164" s="3"/>
       <c r="F164" s="3">
-        <v>2403</v>
+        <v>2398</v>
       </c>
       <c r="G164" s="3" t="s">
-        <v>1188</v>
+        <v>1196</v>
       </c>
       <c r="H164" s="3" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="I164" s="3"/>
       <c r="J164" s="3"/>
@@ -18059,13 +18118,13 @@
       <c r="O164" s="4"/>
       <c r="P164" s="10"/>
       <c r="Q164" s="3" t="s">
-        <v>1189</v>
+        <v>1197</v>
       </c>
       <c r="R164" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S164" s="3" t="s">
-        <v>160</v>
+        <v>52</v>
       </c>
       <c r="T164" s="3">
         <v>1</v>
@@ -18074,29 +18133,29 @@
         <v>53</v>
       </c>
       <c r="V164" s="3" t="s">
-        <v>1190</v>
+        <v>1198</v>
       </c>
       <c r="W164" s="3" t="s">
-        <v>1191</v>
+        <v>1199</v>
       </c>
       <c r="X164" s="3" t="s">
-        <v>1192</v>
+        <v>1189</v>
       </c>
       <c r="Y164" s="3"/>
       <c r="Z164" s="3">
-        <v>0.3</v>
+        <v>4.5</v>
       </c>
       <c r="AA164" s="3"/>
       <c r="AB164" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC164" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD164" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE164" s="3"/>
+        <v>1200</v>
+      </c>
+      <c r="AD164" s="3"/>
+      <c r="AE164" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AF164" s="3"/>
       <c r="AG164" s="3"/>
       <c r="AH164" s="3"/>
@@ -18114,15 +18173,15 @@
         <v>61</v>
       </c>
       <c r="C165" s="7">
-        <v>2026093198</v>
+        <v>2026093177</v>
       </c>
       <c r="D165" s="7"/>
       <c r="E165" s="7"/>
       <c r="F165" s="7">
-        <v>3955</v>
+        <v>2403</v>
       </c>
       <c r="G165" s="7" t="s">
-        <v>1193</v>
+        <v>1201</v>
       </c>
       <c r="H165" s="7" t="s">
         <v>153</v>
@@ -18136,7 +18195,7 @@
       <c r="O165" s="8"/>
       <c r="P165" s="9"/>
       <c r="Q165" s="7" t="s">
-        <v>1194</v>
+        <v>1202</v>
       </c>
       <c r="R165" s="7" t="s">
         <v>51</v>
@@ -18151,13 +18210,13 @@
         <v>53</v>
       </c>
       <c r="V165" s="7" t="s">
-        <v>1195</v>
+        <v>1203</v>
       </c>
       <c r="W165" s="7" t="s">
-        <v>1196</v>
+        <v>1204</v>
       </c>
       <c r="X165" s="7" t="s">
-        <v>1197</v>
+        <v>1205</v>
       </c>
       <c r="Y165" s="7"/>
       <c r="Z165" s="7">
@@ -18191,15 +18250,15 @@
         <v>61</v>
       </c>
       <c r="C166" s="3">
-        <v>2026093210</v>
+        <v>2026093198</v>
       </c>
       <c r="D166" s="3"/>
       <c r="E166" s="3"/>
       <c r="F166" s="3">
-        <v>3853</v>
+        <v>3955</v>
       </c>
       <c r="G166" s="3" t="s">
-        <v>1198</v>
+        <v>1206</v>
       </c>
       <c r="H166" s="3" t="s">
         <v>153</v>
@@ -18211,9 +18270,9 @@
       <c r="M166" s="4"/>
       <c r="N166" s="3"/>
       <c r="O166" s="4"/>
-      <c r="P166" s="4"/>
+      <c r="P166" s="10"/>
       <c r="Q166" s="3" t="s">
-        <v>1199</v>
+        <v>1207</v>
       </c>
       <c r="R166" s="3" t="s">
         <v>51</v>
@@ -18228,13 +18287,13 @@
         <v>53</v>
       </c>
       <c r="V166" s="3" t="s">
-        <v>1200</v>
+        <v>1208</v>
       </c>
       <c r="W166" s="3" t="s">
-        <v>1201</v>
+        <v>1209</v>
       </c>
       <c r="X166" s="3" t="s">
-        <v>1202</v>
+        <v>1210</v>
       </c>
       <c r="Y166" s="3"/>
       <c r="Z166" s="3">
@@ -18244,7 +18303,7 @@
       <c r="AB166" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC166" s="4" t="s">
+      <c r="AC166" s="10" t="s">
         <v>67</v>
       </c>
       <c r="AD166" s="3" t="s">
@@ -18257,6 +18316,83 @@
       <c r="AI166" s="3"/>
       <c r="AJ166" s="3"/>
       <c r="AK166" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="167" spans="1:37">
+      <c r="A167" s="7">
+        <v>165</v>
+      </c>
+      <c r="B167" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C167" s="7">
+        <v>2026093210</v>
+      </c>
+      <c r="D167" s="7"/>
+      <c r="E167" s="7"/>
+      <c r="F167" s="7">
+        <v>3853</v>
+      </c>
+      <c r="G167" s="7" t="s">
+        <v>1211</v>
+      </c>
+      <c r="H167" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I167" s="7"/>
+      <c r="J167" s="7"/>
+      <c r="K167" s="7"/>
+      <c r="L167" s="7"/>
+      <c r="M167" s="8"/>
+      <c r="N167" s="7"/>
+      <c r="O167" s="8"/>
+      <c r="P167" s="8"/>
+      <c r="Q167" s="7" t="s">
+        <v>1212</v>
+      </c>
+      <c r="R167" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S167" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T167" s="7">
+        <v>1</v>
+      </c>
+      <c r="U167" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V167" s="7" t="s">
+        <v>1213</v>
+      </c>
+      <c r="W167" s="7" t="s">
+        <v>1214</v>
+      </c>
+      <c r="X167" s="7" t="s">
+        <v>1215</v>
+      </c>
+      <c r="Y167" s="7"/>
+      <c r="Z167" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA167" s="7"/>
+      <c r="AB167" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC167" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD167" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE167" s="7"/>
+      <c r="AF167" s="7"/>
+      <c r="AG167" s="7"/>
+      <c r="AH167" s="7"/>
+      <c r="AI167" s="7"/>
+      <c r="AJ167" s="7"/>
+      <c r="AK167" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09241831
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$167</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$187</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1322">
   <si>
     <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-24  )</t>
   </si>
@@ -3714,6 +3714,324 @@
   </si>
   <si>
     <t>2026-09-23 17:08:00</t>
+  </si>
+  <si>
+    <t>12315115092401</t>
+  </si>
+  <si>
+    <t>蘆竹坑口店</t>
+  </si>
+  <si>
+    <t>2026-09-24 08:45:04</t>
+  </si>
+  <si>
+    <t>SC(SHUTTLE6S) 2026/9/24 (週四) 上午 08:37  總公司明翰來信:有關 2315門市自行安裝應用程式，請先安排更換SC兩顆硬碟，不要備份。請協助一般派工，到店更換SC第一、二顆硬碟，資料不備分，謝謝。...需請台芝到店協助。PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 與店長確認帳關到09/23，與通訊小晶確認09/23銷售資料都有</t>
+  </si>
+  <si>
+    <t>THILF02315</t>
+  </si>
+  <si>
+    <t>2026-09-24 09:04:56</t>
+  </si>
+  <si>
+    <t>2026-09-24 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:11:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 13:04:00</t>
+  </si>
+  <si>
+    <t>更換第一顆及第二顆硬碟不備份完成</t>
+  </si>
+  <si>
+    <t>12315115092402</t>
+  </si>
+  <si>
+    <t>2026-09-24 10:45:04</t>
+  </si>
+  <si>
+    <t>2026/09/24 10:42總公司明翰來電啟動緊急叫修:SC(SHUTTLE6S) 2026/9/24 (週四) 上午 08:37  總公司明翰來信:有關 2315門市自行安裝應用程式，請先安排更換SC兩顆硬碟，不要備份。請協助一般派工，到店更換SC第一、二顆硬碟，資料不備分，謝謝。...需請台芝到店協助。PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 與店長確認帳關到09/23，與通訊小晶確認09/23銷售資料都有</t>
+  </si>
+  <si>
+    <t>2026-09-24 10:45:46</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:45:00</t>
+  </si>
+  <si>
+    <t>L516</t>
+  </si>
+  <si>
+    <t>車麗屋新莊店</t>
+  </si>
+  <si>
+    <t>THILF0L516</t>
+  </si>
+  <si>
+    <t>2026-09-24 11:33:09</t>
+  </si>
+  <si>
+    <t>2026-09-24 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 11:30:00</t>
+  </si>
+  <si>
+    <t>板橋民生站</t>
+  </si>
+  <si>
+    <t>THILF05384</t>
+  </si>
+  <si>
+    <t>2026-09-24 12:53:13</t>
+  </si>
+  <si>
+    <t>2026-09-24 12:25:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 12:36:00</t>
+  </si>
+  <si>
+    <t>板橋江寧店</t>
+  </si>
+  <si>
+    <t>THILF04680</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:16:10</t>
+  </si>
+  <si>
+    <t>2026-09-24 12:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:13:00</t>
+  </si>
+  <si>
+    <t>板橋雙十店</t>
+  </si>
+  <si>
+    <t>THILF02221</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:53:20</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:26:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:40:00</t>
+  </si>
+  <si>
+    <t>板橋江子翠站</t>
+  </si>
+  <si>
+    <t>THILF02069</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:17:38</t>
+  </si>
+  <si>
+    <t>2026-09-24 13:56:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:14:00</t>
+  </si>
+  <si>
+    <t>13962115092401</t>
+  </si>
+  <si>
+    <t>板橋仁化店</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:35:38</t>
+  </si>
+  <si>
+    <t>THILF03962</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:36:41</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:42:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 18:36:00</t>
+  </si>
+  <si>
+    <t>+HUB重設0800測試正常</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:47:06</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:21:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:36:00</t>
+  </si>
+  <si>
+    <t>板橋民治店</t>
+  </si>
+  <si>
+    <t>THILF03965</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:05:24</t>
+  </si>
+  <si>
+    <t>2026-09-24 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:03:00</t>
+  </si>
+  <si>
+    <t>板橋翠華店</t>
+  </si>
+  <si>
+    <t>THILF04917</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:24:53</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:23:00</t>
+  </si>
+  <si>
+    <t>板橋懷仁店</t>
+  </si>
+  <si>
+    <t>THILF05451</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:41:14</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:38:00</t>
+  </si>
+  <si>
+    <t>板橋板莊店</t>
+  </si>
+  <si>
+    <t>THILF02154</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:55:14</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:42:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:53:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:09:44</t>
+  </si>
+  <si>
+    <t>2026-09-24 15:56:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:07:00</t>
+  </si>
+  <si>
+    <t>中和興南店</t>
+  </si>
+  <si>
+    <t>THILF02171</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:28:44</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:02:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:24:00</t>
+  </si>
+  <si>
+    <t>D349</t>
+  </si>
+  <si>
+    <t>板橋成都店</t>
+  </si>
+  <si>
+    <t>THILF0D349</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:39:05</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:12:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:36:00</t>
+  </si>
+  <si>
+    <t>板橋國慶店</t>
+  </si>
+  <si>
+    <t>THILF03416</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:57:26</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 16:55:00</t>
+  </si>
+  <si>
+    <t>板橋湳雅夜市</t>
+  </si>
+  <si>
+    <t>THILF02995</t>
+  </si>
+  <si>
+    <t>2026-09-24 17:19:36</t>
+  </si>
+  <si>
+    <t>2026-09-24 17:05:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 17:17:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 17:49:20</t>
+  </si>
+  <si>
+    <t>2026-09-24 17:25:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 17:46:00</t>
+  </si>
+  <si>
+    <t>板橋福康店</t>
+  </si>
+  <si>
+    <t>THILF04046</t>
+  </si>
+  <si>
+    <t>2026-09-24 18:23:45</t>
+  </si>
+  <si>
+    <t>2026-09-24 18:06:00</t>
+  </si>
+  <si>
+    <t>2026-09-24 18:21:00</t>
   </si>
 </sst>
 </file>
@@ -4127,7 +4445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK167"/>
+  <dimension ref="A1:AK187"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -18347,7 +18665,7 @@
       <c r="M167" s="8"/>
       <c r="N167" s="7"/>
       <c r="O167" s="8"/>
-      <c r="P167" s="8"/>
+      <c r="P167" s="9"/>
       <c r="Q167" s="7" t="s">
         <v>1212</v>
       </c>
@@ -18380,7 +18698,7 @@
       <c r="AB167" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC167" s="8" t="s">
+      <c r="AC167" s="9" t="s">
         <v>67</v>
       </c>
       <c r="AD167" s="7" t="s">
@@ -18393,6 +18711,1610 @@
       <c r="AI167" s="7"/>
       <c r="AJ167" s="7"/>
       <c r="AK167" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="168" spans="1:37">
+      <c r="A168" s="3">
+        <v>166</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C168" s="3">
+        <v>2026093231</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>1216</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F168" s="3">
+        <v>2315</v>
+      </c>
+      <c r="G168" s="3" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H168" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I168" s="3" t="s">
+        <v>1218</v>
+      </c>
+      <c r="J168" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K168" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L168" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M168" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N168" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O168" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="P168" s="10" t="s">
+        <v>1219</v>
+      </c>
+      <c r="Q168" s="3" t="s">
+        <v>1220</v>
+      </c>
+      <c r="R168" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S168" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T168" s="3">
+        <v>1</v>
+      </c>
+      <c r="U168" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V168" s="3" t="s">
+        <v>1221</v>
+      </c>
+      <c r="W168" s="3" t="s">
+        <v>1222</v>
+      </c>
+      <c r="X168" s="3" t="s">
+        <v>1223</v>
+      </c>
+      <c r="Y168" s="3" t="s">
+        <v>1224</v>
+      </c>
+      <c r="Z168" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="AA168" s="3"/>
+      <c r="AB168" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC168" s="10" t="s">
+        <v>1225</v>
+      </c>
+      <c r="AD168" s="3"/>
+      <c r="AE168" s="3"/>
+      <c r="AF168" s="3"/>
+      <c r="AG168" s="3"/>
+      <c r="AH168" s="3"/>
+      <c r="AI168" s="3"/>
+      <c r="AJ168" s="3"/>
+      <c r="AK168" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="169" spans="1:37">
+      <c r="A169" s="7">
+        <v>167</v>
+      </c>
+      <c r="B169" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C169" s="7">
+        <v>2026093267</v>
+      </c>
+      <c r="D169" s="7" t="s">
+        <v>1226</v>
+      </c>
+      <c r="E169" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F169" s="7">
+        <v>2315</v>
+      </c>
+      <c r="G169" s="7" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H169" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I169" s="7" t="s">
+        <v>1227</v>
+      </c>
+      <c r="J169" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K169" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L169" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M169" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N169" s="7">
+        <v>2405</v>
+      </c>
+      <c r="O169" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="P169" s="9" t="s">
+        <v>1228</v>
+      </c>
+      <c r="Q169" s="7" t="s">
+        <v>1220</v>
+      </c>
+      <c r="R169" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S169" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T169" s="7">
+        <v>1</v>
+      </c>
+      <c r="U169" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V169" s="7" t="s">
+        <v>1229</v>
+      </c>
+      <c r="W169" s="7" t="s">
+        <v>1222</v>
+      </c>
+      <c r="X169" s="7" t="s">
+        <v>1230</v>
+      </c>
+      <c r="Y169" s="7" t="s">
+        <v>1231</v>
+      </c>
+      <c r="Z169" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="AA169" s="7"/>
+      <c r="AB169" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC169" s="9" t="s">
+        <v>1225</v>
+      </c>
+      <c r="AD169" s="7"/>
+      <c r="AE169" s="7"/>
+      <c r="AF169" s="7"/>
+      <c r="AG169" s="7"/>
+      <c r="AH169" s="7"/>
+      <c r="AI169" s="7"/>
+      <c r="AJ169" s="7"/>
+      <c r="AK169" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="170" spans="1:37">
+      <c r="A170" s="3">
+        <v>168</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C170" s="3">
+        <v>2026093279</v>
+      </c>
+      <c r="D170" s="3"/>
+      <c r="E170" s="3"/>
+      <c r="F170" s="3" t="s">
+        <v>1232</v>
+      </c>
+      <c r="G170" s="3" t="s">
+        <v>1233</v>
+      </c>
+      <c r="H170" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I170" s="3"/>
+      <c r="J170" s="3"/>
+      <c r="K170" s="3"/>
+      <c r="L170" s="3"/>
+      <c r="M170" s="4"/>
+      <c r="N170" s="3"/>
+      <c r="O170" s="4"/>
+      <c r="P170" s="10"/>
+      <c r="Q170" s="3" t="s">
+        <v>1234</v>
+      </c>
+      <c r="R170" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S170" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T170" s="3">
+        <v>1</v>
+      </c>
+      <c r="U170" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V170" s="3" t="s">
+        <v>1235</v>
+      </c>
+      <c r="W170" s="3" t="s">
+        <v>1236</v>
+      </c>
+      <c r="X170" s="3" t="s">
+        <v>1237</v>
+      </c>
+      <c r="Y170" s="3"/>
+      <c r="Z170" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA170" s="3"/>
+      <c r="AB170" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC170" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD170" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE170" s="3"/>
+      <c r="AF170" s="3"/>
+      <c r="AG170" s="3"/>
+      <c r="AH170" s="3"/>
+      <c r="AI170" s="3"/>
+      <c r="AJ170" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK170" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="171" spans="1:37">
+      <c r="A171" s="7">
+        <v>169</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C171" s="7">
+        <v>2026093293</v>
+      </c>
+      <c r="D171" s="7"/>
+      <c r="E171" s="7"/>
+      <c r="F171" s="7">
+        <v>5384</v>
+      </c>
+      <c r="G171" s="7" t="s">
+        <v>1238</v>
+      </c>
+      <c r="H171" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I171" s="7"/>
+      <c r="J171" s="7"/>
+      <c r="K171" s="7"/>
+      <c r="L171" s="7"/>
+      <c r="M171" s="8"/>
+      <c r="N171" s="7"/>
+      <c r="O171" s="8"/>
+      <c r="P171" s="9"/>
+      <c r="Q171" s="7" t="s">
+        <v>1239</v>
+      </c>
+      <c r="R171" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S171" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T171" s="7">
+        <v>1</v>
+      </c>
+      <c r="U171" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V171" s="7" t="s">
+        <v>1240</v>
+      </c>
+      <c r="W171" s="7" t="s">
+        <v>1241</v>
+      </c>
+      <c r="X171" s="7" t="s">
+        <v>1242</v>
+      </c>
+      <c r="Y171" s="7"/>
+      <c r="Z171" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA171" s="7"/>
+      <c r="AB171" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC171" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD171" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE171" s="7"/>
+      <c r="AF171" s="7"/>
+      <c r="AG171" s="7"/>
+      <c r="AH171" s="7"/>
+      <c r="AI171" s="7"/>
+      <c r="AJ171" s="7"/>
+      <c r="AK171" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="172" spans="1:37">
+      <c r="A172" s="3">
+        <v>170</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C172" s="3">
+        <v>2026093295</v>
+      </c>
+      <c r="D172" s="3"/>
+      <c r="E172" s="3"/>
+      <c r="F172" s="3">
+        <v>4680</v>
+      </c>
+      <c r="G172" s="3" t="s">
+        <v>1243</v>
+      </c>
+      <c r="H172" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I172" s="3"/>
+      <c r="J172" s="3"/>
+      <c r="K172" s="3"/>
+      <c r="L172" s="3"/>
+      <c r="M172" s="4"/>
+      <c r="N172" s="3"/>
+      <c r="O172" s="4"/>
+      <c r="P172" s="10"/>
+      <c r="Q172" s="3" t="s">
+        <v>1244</v>
+      </c>
+      <c r="R172" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S172" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T172" s="3">
+        <v>1</v>
+      </c>
+      <c r="U172" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V172" s="3" t="s">
+        <v>1245</v>
+      </c>
+      <c r="W172" s="3" t="s">
+        <v>1246</v>
+      </c>
+      <c r="X172" s="3" t="s">
+        <v>1247</v>
+      </c>
+      <c r="Y172" s="3"/>
+      <c r="Z172" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA172" s="3"/>
+      <c r="AB172" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC172" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD172" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE172" s="3"/>
+      <c r="AF172" s="3"/>
+      <c r="AG172" s="3"/>
+      <c r="AH172" s="3"/>
+      <c r="AI172" s="3"/>
+      <c r="AJ172" s="3"/>
+      <c r="AK172" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="173" spans="1:37">
+      <c r="A173" s="7">
+        <v>171</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C173" s="7">
+        <v>2026093301</v>
+      </c>
+      <c r="D173" s="7"/>
+      <c r="E173" s="7"/>
+      <c r="F173" s="7">
+        <v>2221</v>
+      </c>
+      <c r="G173" s="7" t="s">
+        <v>1248</v>
+      </c>
+      <c r="H173" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I173" s="7"/>
+      <c r="J173" s="7"/>
+      <c r="K173" s="7"/>
+      <c r="L173" s="7"/>
+      <c r="M173" s="8"/>
+      <c r="N173" s="7"/>
+      <c r="O173" s="8"/>
+      <c r="P173" s="9"/>
+      <c r="Q173" s="7" t="s">
+        <v>1249</v>
+      </c>
+      <c r="R173" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S173" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T173" s="7">
+        <v>1</v>
+      </c>
+      <c r="U173" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V173" s="7" t="s">
+        <v>1250</v>
+      </c>
+      <c r="W173" s="7" t="s">
+        <v>1251</v>
+      </c>
+      <c r="X173" s="7" t="s">
+        <v>1252</v>
+      </c>
+      <c r="Y173" s="7"/>
+      <c r="Z173" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA173" s="7"/>
+      <c r="AB173" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC173" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD173" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE173" s="7"/>
+      <c r="AF173" s="7"/>
+      <c r="AG173" s="7"/>
+      <c r="AH173" s="7"/>
+      <c r="AI173" s="7"/>
+      <c r="AJ173" s="7"/>
+      <c r="AK173" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="174" spans="1:37">
+      <c r="A174" s="3">
+        <v>172</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C174" s="3">
+        <v>2026093306</v>
+      </c>
+      <c r="D174" s="3"/>
+      <c r="E174" s="3"/>
+      <c r="F174" s="3">
+        <v>2069</v>
+      </c>
+      <c r="G174" s="3" t="s">
+        <v>1253</v>
+      </c>
+      <c r="H174" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I174" s="3"/>
+      <c r="J174" s="3"/>
+      <c r="K174" s="3"/>
+      <c r="L174" s="3"/>
+      <c r="M174" s="4"/>
+      <c r="N174" s="3"/>
+      <c r="O174" s="4"/>
+      <c r="P174" s="10"/>
+      <c r="Q174" s="3" t="s">
+        <v>1254</v>
+      </c>
+      <c r="R174" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S174" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T174" s="3">
+        <v>1</v>
+      </c>
+      <c r="U174" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V174" s="3" t="s">
+        <v>1255</v>
+      </c>
+      <c r="W174" s="3" t="s">
+        <v>1256</v>
+      </c>
+      <c r="X174" s="3" t="s">
+        <v>1257</v>
+      </c>
+      <c r="Y174" s="3"/>
+      <c r="Z174" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA174" s="3"/>
+      <c r="AB174" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC174" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD174" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE174" s="3"/>
+      <c r="AF174" s="3"/>
+      <c r="AG174" s="3"/>
+      <c r="AH174" s="3"/>
+      <c r="AI174" s="3"/>
+      <c r="AJ174" s="3"/>
+      <c r="AK174" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="175" spans="1:37">
+      <c r="A175" s="7">
+        <v>173</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C175" s="7">
+        <v>2026093311</v>
+      </c>
+      <c r="D175" s="7" t="s">
+        <v>1258</v>
+      </c>
+      <c r="E175" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F175" s="7">
+        <v>3962</v>
+      </c>
+      <c r="G175" s="7" t="s">
+        <v>1259</v>
+      </c>
+      <c r="H175" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I175" s="7" t="s">
+        <v>1260</v>
+      </c>
+      <c r="J175" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K175" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L175" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="M175" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="N175" s="7">
+        <v>3404</v>
+      </c>
+      <c r="O175" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="P175" s="9" t="s">
+        <v>559</v>
+      </c>
+      <c r="Q175" s="7" t="s">
+        <v>1261</v>
+      </c>
+      <c r="R175" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S175" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T175" s="7">
+        <v>1</v>
+      </c>
+      <c r="U175" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V175" s="7" t="s">
+        <v>1262</v>
+      </c>
+      <c r="W175" s="7" t="s">
+        <v>1263</v>
+      </c>
+      <c r="X175" s="7" t="s">
+        <v>1264</v>
+      </c>
+      <c r="Y175" s="7" t="s">
+        <v>1265</v>
+      </c>
+      <c r="Z175" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA175" s="7"/>
+      <c r="AB175" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC175" s="9" t="s">
+        <v>1266</v>
+      </c>
+      <c r="AD175" s="7"/>
+      <c r="AE175" s="7"/>
+      <c r="AF175" s="7"/>
+      <c r="AG175" s="7"/>
+      <c r="AH175" s="7"/>
+      <c r="AI175" s="7"/>
+      <c r="AJ175" s="7"/>
+      <c r="AK175" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="176" spans="1:37">
+      <c r="A176" s="3">
+        <v>174</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C176" s="3">
+        <v>2026093313</v>
+      </c>
+      <c r="D176" s="3"/>
+      <c r="E176" s="3"/>
+      <c r="F176" s="3">
+        <v>3962</v>
+      </c>
+      <c r="G176" s="3" t="s">
+        <v>1259</v>
+      </c>
+      <c r="H176" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I176" s="3"/>
+      <c r="J176" s="3"/>
+      <c r="K176" s="3"/>
+      <c r="L176" s="3"/>
+      <c r="M176" s="4"/>
+      <c r="N176" s="3"/>
+      <c r="O176" s="4"/>
+      <c r="P176" s="10"/>
+      <c r="Q176" s="3" t="s">
+        <v>1261</v>
+      </c>
+      <c r="R176" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S176" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T176" s="3">
+        <v>1</v>
+      </c>
+      <c r="U176" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V176" s="3" t="s">
+        <v>1267</v>
+      </c>
+      <c r="W176" s="3" t="s">
+        <v>1268</v>
+      </c>
+      <c r="X176" s="3" t="s">
+        <v>1269</v>
+      </c>
+      <c r="Y176" s="3"/>
+      <c r="Z176" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA176" s="3"/>
+      <c r="AB176" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC176" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD176" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE176" s="3"/>
+      <c r="AF176" s="3"/>
+      <c r="AG176" s="3"/>
+      <c r="AH176" s="3"/>
+      <c r="AI176" s="3"/>
+      <c r="AJ176" s="3"/>
+      <c r="AK176" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="177" spans="1:37">
+      <c r="A177" s="7">
+        <v>175</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C177" s="7">
+        <v>2026093318</v>
+      </c>
+      <c r="D177" s="7"/>
+      <c r="E177" s="7"/>
+      <c r="F177" s="7">
+        <v>3965</v>
+      </c>
+      <c r="G177" s="7" t="s">
+        <v>1270</v>
+      </c>
+      <c r="H177" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I177" s="7"/>
+      <c r="J177" s="7"/>
+      <c r="K177" s="7"/>
+      <c r="L177" s="7"/>
+      <c r="M177" s="8"/>
+      <c r="N177" s="7"/>
+      <c r="O177" s="8"/>
+      <c r="P177" s="9"/>
+      <c r="Q177" s="7" t="s">
+        <v>1271</v>
+      </c>
+      <c r="R177" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S177" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T177" s="7">
+        <v>1</v>
+      </c>
+      <c r="U177" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V177" s="7" t="s">
+        <v>1272</v>
+      </c>
+      <c r="W177" s="7" t="s">
+        <v>1273</v>
+      </c>
+      <c r="X177" s="7" t="s">
+        <v>1274</v>
+      </c>
+      <c r="Y177" s="7"/>
+      <c r="Z177" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA177" s="7"/>
+      <c r="AB177" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC177" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD177" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE177" s="7"/>
+      <c r="AF177" s="7"/>
+      <c r="AG177" s="7"/>
+      <c r="AH177" s="7"/>
+      <c r="AI177" s="7"/>
+      <c r="AJ177" s="7"/>
+      <c r="AK177" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="178" spans="1:37">
+      <c r="A178" s="3">
+        <v>176</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C178" s="3">
+        <v>2026093320</v>
+      </c>
+      <c r="D178" s="3"/>
+      <c r="E178" s="3"/>
+      <c r="F178" s="3">
+        <v>4917</v>
+      </c>
+      <c r="G178" s="3" t="s">
+        <v>1275</v>
+      </c>
+      <c r="H178" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I178" s="3"/>
+      <c r="J178" s="3"/>
+      <c r="K178" s="3"/>
+      <c r="L178" s="3"/>
+      <c r="M178" s="4"/>
+      <c r="N178" s="3"/>
+      <c r="O178" s="4"/>
+      <c r="P178" s="10"/>
+      <c r="Q178" s="3" t="s">
+        <v>1276</v>
+      </c>
+      <c r="R178" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S178" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T178" s="3">
+        <v>1</v>
+      </c>
+      <c r="U178" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V178" s="3" t="s">
+        <v>1277</v>
+      </c>
+      <c r="W178" s="3" t="s">
+        <v>1278</v>
+      </c>
+      <c r="X178" s="3" t="s">
+        <v>1279</v>
+      </c>
+      <c r="Y178" s="3"/>
+      <c r="Z178" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA178" s="3"/>
+      <c r="AB178" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC178" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD178" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE178" s="3"/>
+      <c r="AF178" s="3"/>
+      <c r="AG178" s="3"/>
+      <c r="AH178" s="3"/>
+      <c r="AI178" s="3"/>
+      <c r="AJ178" s="3"/>
+      <c r="AK178" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="179" spans="1:37">
+      <c r="A179" s="7">
+        <v>177</v>
+      </c>
+      <c r="B179" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C179" s="7">
+        <v>2026093330</v>
+      </c>
+      <c r="D179" s="7"/>
+      <c r="E179" s="7"/>
+      <c r="F179" s="7">
+        <v>5451</v>
+      </c>
+      <c r="G179" s="7" t="s">
+        <v>1280</v>
+      </c>
+      <c r="H179" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I179" s="7"/>
+      <c r="J179" s="7"/>
+      <c r="K179" s="7"/>
+      <c r="L179" s="7"/>
+      <c r="M179" s="8"/>
+      <c r="N179" s="7"/>
+      <c r="O179" s="8"/>
+      <c r="P179" s="9"/>
+      <c r="Q179" s="7" t="s">
+        <v>1281</v>
+      </c>
+      <c r="R179" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S179" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T179" s="7">
+        <v>1</v>
+      </c>
+      <c r="U179" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V179" s="7" t="s">
+        <v>1282</v>
+      </c>
+      <c r="W179" s="7" t="s">
+        <v>1283</v>
+      </c>
+      <c r="X179" s="7" t="s">
+        <v>1284</v>
+      </c>
+      <c r="Y179" s="7"/>
+      <c r="Z179" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA179" s="7"/>
+      <c r="AB179" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC179" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD179" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE179" s="7"/>
+      <c r="AF179" s="7"/>
+      <c r="AG179" s="7"/>
+      <c r="AH179" s="7"/>
+      <c r="AI179" s="7"/>
+      <c r="AJ179" s="7"/>
+      <c r="AK179" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="180" spans="1:37">
+      <c r="A180" s="3">
+        <v>178</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C180" s="3">
+        <v>2026093335</v>
+      </c>
+      <c r="D180" s="3"/>
+      <c r="E180" s="3"/>
+      <c r="F180" s="3">
+        <v>2154</v>
+      </c>
+      <c r="G180" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="H180" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I180" s="3"/>
+      <c r="J180" s="3"/>
+      <c r="K180" s="3"/>
+      <c r="L180" s="3"/>
+      <c r="M180" s="4"/>
+      <c r="N180" s="3"/>
+      <c r="O180" s="4"/>
+      <c r="P180" s="10"/>
+      <c r="Q180" s="3" t="s">
+        <v>1286</v>
+      </c>
+      <c r="R180" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S180" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T180" s="3">
+        <v>1</v>
+      </c>
+      <c r="U180" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V180" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="W180" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="X180" s="3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="Y180" s="3"/>
+      <c r="Z180" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA180" s="3"/>
+      <c r="AB180" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC180" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD180" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE180" s="3"/>
+      <c r="AF180" s="3"/>
+      <c r="AG180" s="3"/>
+      <c r="AH180" s="3"/>
+      <c r="AI180" s="3"/>
+      <c r="AJ180" s="3"/>
+      <c r="AK180" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="181" spans="1:37">
+      <c r="A181" s="7">
+        <v>179</v>
+      </c>
+      <c r="B181" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C181" s="7">
+        <v>2026093336</v>
+      </c>
+      <c r="D181" s="7"/>
+      <c r="E181" s="7"/>
+      <c r="F181" s="7">
+        <v>2224</v>
+      </c>
+      <c r="G181" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="H181" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I181" s="7"/>
+      <c r="J181" s="7"/>
+      <c r="K181" s="7"/>
+      <c r="L181" s="7"/>
+      <c r="M181" s="8"/>
+      <c r="N181" s="7"/>
+      <c r="O181" s="8"/>
+      <c r="P181" s="9"/>
+      <c r="Q181" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="R181" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S181" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T181" s="7">
+        <v>1</v>
+      </c>
+      <c r="U181" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V181" s="7" t="s">
+        <v>1290</v>
+      </c>
+      <c r="W181" s="7" t="s">
+        <v>1291</v>
+      </c>
+      <c r="X181" s="7" t="s">
+        <v>1292</v>
+      </c>
+      <c r="Y181" s="7"/>
+      <c r="Z181" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA181" s="7"/>
+      <c r="AB181" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC181" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD181" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE181" s="7"/>
+      <c r="AF181" s="7"/>
+      <c r="AG181" s="7"/>
+      <c r="AH181" s="7"/>
+      <c r="AI181" s="7"/>
+      <c r="AJ181" s="7"/>
+      <c r="AK181" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="182" spans="1:37">
+      <c r="A182" s="3">
+        <v>180</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C182" s="3">
+        <v>2026093339</v>
+      </c>
+      <c r="D182" s="3"/>
+      <c r="E182" s="3"/>
+      <c r="F182" s="3">
+        <v>2171</v>
+      </c>
+      <c r="G182" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H182" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I182" s="3"/>
+      <c r="J182" s="3"/>
+      <c r="K182" s="3"/>
+      <c r="L182" s="3"/>
+      <c r="M182" s="4"/>
+      <c r="N182" s="3"/>
+      <c r="O182" s="4"/>
+      <c r="P182" s="10"/>
+      <c r="Q182" s="3" t="s">
+        <v>1294</v>
+      </c>
+      <c r="R182" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S182" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T182" s="3">
+        <v>1</v>
+      </c>
+      <c r="U182" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V182" s="3" t="s">
+        <v>1295</v>
+      </c>
+      <c r="W182" s="3" t="s">
+        <v>1296</v>
+      </c>
+      <c r="X182" s="3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="Y182" s="3"/>
+      <c r="Z182" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA182" s="3"/>
+      <c r="AB182" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC182" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD182" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE182" s="3"/>
+      <c r="AF182" s="3"/>
+      <c r="AG182" s="3"/>
+      <c r="AH182" s="3"/>
+      <c r="AI182" s="3"/>
+      <c r="AJ182" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK182" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="183" spans="1:37">
+      <c r="A183" s="7">
+        <v>181</v>
+      </c>
+      <c r="B183" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C183" s="7">
+        <v>2026093341</v>
+      </c>
+      <c r="D183" s="7"/>
+      <c r="E183" s="7"/>
+      <c r="F183" s="7" t="s">
+        <v>1298</v>
+      </c>
+      <c r="G183" s="7" t="s">
+        <v>1299</v>
+      </c>
+      <c r="H183" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I183" s="7"/>
+      <c r="J183" s="7"/>
+      <c r="K183" s="7"/>
+      <c r="L183" s="7"/>
+      <c r="M183" s="8"/>
+      <c r="N183" s="7"/>
+      <c r="O183" s="8"/>
+      <c r="P183" s="9"/>
+      <c r="Q183" s="7" t="s">
+        <v>1300</v>
+      </c>
+      <c r="R183" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S183" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T183" s="7">
+        <v>1</v>
+      </c>
+      <c r="U183" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V183" s="7" t="s">
+        <v>1301</v>
+      </c>
+      <c r="W183" s="7" t="s">
+        <v>1302</v>
+      </c>
+      <c r="X183" s="7" t="s">
+        <v>1303</v>
+      </c>
+      <c r="Y183" s="7"/>
+      <c r="Z183" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA183" s="7"/>
+      <c r="AB183" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC183" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD183" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE183" s="7"/>
+      <c r="AF183" s="7"/>
+      <c r="AG183" s="7"/>
+      <c r="AH183" s="7"/>
+      <c r="AI183" s="7"/>
+      <c r="AJ183" s="7"/>
+      <c r="AK183" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="184" spans="1:37">
+      <c r="A184" s="3">
+        <v>182</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C184" s="3">
+        <v>2026093367</v>
+      </c>
+      <c r="D184" s="3"/>
+      <c r="E184" s="3"/>
+      <c r="F184" s="3">
+        <v>3416</v>
+      </c>
+      <c r="G184" s="3" t="s">
+        <v>1304</v>
+      </c>
+      <c r="H184" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I184" s="3"/>
+      <c r="J184" s="3"/>
+      <c r="K184" s="3"/>
+      <c r="L184" s="3"/>
+      <c r="M184" s="4"/>
+      <c r="N184" s="3"/>
+      <c r="O184" s="4"/>
+      <c r="P184" s="10"/>
+      <c r="Q184" s="3" t="s">
+        <v>1305</v>
+      </c>
+      <c r="R184" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S184" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T184" s="3">
+        <v>1</v>
+      </c>
+      <c r="U184" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V184" s="3" t="s">
+        <v>1306</v>
+      </c>
+      <c r="W184" s="3" t="s">
+        <v>1307</v>
+      </c>
+      <c r="X184" s="3" t="s">
+        <v>1308</v>
+      </c>
+      <c r="Y184" s="3"/>
+      <c r="Z184" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA184" s="3"/>
+      <c r="AB184" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC184" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD184" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE184" s="3"/>
+      <c r="AF184" s="3"/>
+      <c r="AG184" s="3"/>
+      <c r="AH184" s="3"/>
+      <c r="AI184" s="3"/>
+      <c r="AJ184" s="3"/>
+      <c r="AK184" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="185" spans="1:37">
+      <c r="A185" s="7">
+        <v>183</v>
+      </c>
+      <c r="B185" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C185" s="7">
+        <v>2026093388</v>
+      </c>
+      <c r="D185" s="7"/>
+      <c r="E185" s="7"/>
+      <c r="F185" s="7">
+        <v>2995</v>
+      </c>
+      <c r="G185" s="7" t="s">
+        <v>1309</v>
+      </c>
+      <c r="H185" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I185" s="7"/>
+      <c r="J185" s="7"/>
+      <c r="K185" s="7"/>
+      <c r="L185" s="7"/>
+      <c r="M185" s="8"/>
+      <c r="N185" s="7"/>
+      <c r="O185" s="8"/>
+      <c r="P185" s="9"/>
+      <c r="Q185" s="7" t="s">
+        <v>1310</v>
+      </c>
+      <c r="R185" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S185" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T185" s="7">
+        <v>1</v>
+      </c>
+      <c r="U185" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V185" s="7" t="s">
+        <v>1311</v>
+      </c>
+      <c r="W185" s="7" t="s">
+        <v>1312</v>
+      </c>
+      <c r="X185" s="7" t="s">
+        <v>1313</v>
+      </c>
+      <c r="Y185" s="7"/>
+      <c r="Z185" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA185" s="7"/>
+      <c r="AB185" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC185" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD185" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE185" s="7"/>
+      <c r="AF185" s="7"/>
+      <c r="AG185" s="7"/>
+      <c r="AH185" s="7"/>
+      <c r="AI185" s="7"/>
+      <c r="AJ185" s="7"/>
+      <c r="AK185" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="186" spans="1:37">
+      <c r="A186" s="3">
+        <v>184</v>
+      </c>
+      <c r="B186" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C186" s="3">
+        <v>2026093392</v>
+      </c>
+      <c r="D186" s="3"/>
+      <c r="E186" s="3"/>
+      <c r="F186" s="3" t="s">
+        <v>1179</v>
+      </c>
+      <c r="G186" s="3" t="s">
+        <v>1180</v>
+      </c>
+      <c r="H186" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I186" s="3"/>
+      <c r="J186" s="3"/>
+      <c r="K186" s="3"/>
+      <c r="L186" s="3"/>
+      <c r="M186" s="4"/>
+      <c r="N186" s="3"/>
+      <c r="O186" s="4"/>
+      <c r="P186" s="10"/>
+      <c r="Q186" s="3" t="s">
+        <v>1181</v>
+      </c>
+      <c r="R186" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S186" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T186" s="3">
+        <v>1</v>
+      </c>
+      <c r="U186" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V186" s="3" t="s">
+        <v>1314</v>
+      </c>
+      <c r="W186" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="X186" s="3" t="s">
+        <v>1316</v>
+      </c>
+      <c r="Y186" s="3"/>
+      <c r="Z186" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA186" s="3"/>
+      <c r="AB186" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC186" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD186" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE186" s="3"/>
+      <c r="AF186" s="3"/>
+      <c r="AG186" s="3"/>
+      <c r="AH186" s="3"/>
+      <c r="AI186" s="3"/>
+      <c r="AJ186" s="3"/>
+      <c r="AK186" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="187" spans="1:37">
+      <c r="A187" s="7">
+        <v>185</v>
+      </c>
+      <c r="B187" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C187" s="7">
+        <v>2026093393</v>
+      </c>
+      <c r="D187" s="7"/>
+      <c r="E187" s="7"/>
+      <c r="F187" s="7">
+        <v>4046</v>
+      </c>
+      <c r="G187" s="7" t="s">
+        <v>1317</v>
+      </c>
+      <c r="H187" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I187" s="7"/>
+      <c r="J187" s="7"/>
+      <c r="K187" s="7"/>
+      <c r="L187" s="7"/>
+      <c r="M187" s="8"/>
+      <c r="N187" s="7"/>
+      <c r="O187" s="8"/>
+      <c r="P187" s="8"/>
+      <c r="Q187" s="7" t="s">
+        <v>1318</v>
+      </c>
+      <c r="R187" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S187" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T187" s="7">
+        <v>1</v>
+      </c>
+      <c r="U187" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V187" s="7" t="s">
+        <v>1319</v>
+      </c>
+      <c r="W187" s="7" t="s">
+        <v>1320</v>
+      </c>
+      <c r="X187" s="7" t="s">
+        <v>1321</v>
+      </c>
+      <c r="Y187" s="7"/>
+      <c r="Z187" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA187" s="7"/>
+      <c r="AB187" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC187" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD187" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE187" s="7"/>
+      <c r="AF187" s="7"/>
+      <c r="AG187" s="7"/>
+      <c r="AH187" s="7"/>
+      <c r="AI187" s="7"/>
+      <c r="AJ187" s="7"/>
+      <c r="AK187" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09291812
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$187</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$195</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1322">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-24  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1359">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-29  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -4032,6 +4032,120 @@
   </si>
   <si>
     <t>2026-09-24 18:21:00</t>
+  </si>
+  <si>
+    <t>14698115092701</t>
+  </si>
+  <si>
+    <t>2026-09-27 10:28:18</t>
+  </si>
+  <si>
+    <t>09/27 10:40 啟動緊急叫修:sc(SHUTTLE7S)門市告知無法使用訂貨3.0訂貨和提前訂貨功能，vnc時發現ping1不通無法vnc，與門市確認無法連上e網，查看tm右下sc燈號紅燈，請門市將hub 1port重新拔插以及更換孔位後ping1仍不通，重開機仍異常....需請台芝到店協助PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)與門市確認帳關到09/26，與通訊小晶確認都有收到</t>
+  </si>
+  <si>
+    <t>2026-09-27 10:42:57</t>
+  </si>
+  <si>
+    <t>2026-09-27 11:05:00</t>
+  </si>
+  <si>
+    <t>2026-09-27 11:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-27 16:42:00</t>
+  </si>
+  <si>
+    <t>HUB1號孔位重插拔後目前可正常連線</t>
+  </si>
+  <si>
+    <t>12315115092901</t>
+  </si>
+  <si>
+    <t>2026-09-29 09:05:10</t>
+  </si>
+  <si>
+    <t>SC(SHUTTLE6S)2026/9/29 (週二) 上午 09:01 總公司玫君啟動緊急叫修來信:有關 2315門市又自行安裝應用程式，請先安排更換SC兩顆硬碟，不要備份。請協助緊急派工，到店更換SC第一、二顆硬碟，資料不備分，謝謝。...需請台芝到店協助。PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 與店長確認帳關到09/28，與通訊圭連確認09/28銷售資料都有</t>
+  </si>
+  <si>
+    <t>2026-09-29 09:11:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 15:11:00</t>
+  </si>
+  <si>
+    <t>更換主機
+換下8114003356
+換上8114003741
+更換第一顆及第二顆硬碟不備份還原</t>
+  </si>
+  <si>
+    <t>14456115092901</t>
+  </si>
+  <si>
+    <t>蘆竹華麗店</t>
+  </si>
+  <si>
+    <t>2026-09-29 15:28:18</t>
+  </si>
+  <si>
+    <t>台芝吳先生告知今日回裝發現SC滑鼠故障，需更換，請客服協助派工</t>
+  </si>
+  <si>
+    <t>THILF04456</t>
+  </si>
+  <si>
+    <t>2026-09-29 15:29:24</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 19:29:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:13:53</t>
+  </si>
+  <si>
+    <t>2026-09-29 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:13:00</t>
+  </si>
+  <si>
+    <t>裝潢回裝完工</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:14:00</t>
+  </si>
+  <si>
+    <t>D024</t>
+  </si>
+  <si>
+    <t>三重三民店</t>
+  </si>
+  <si>
+    <t>THILF0D024</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:33:27</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:01:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:23:00</t>
+  </si>
+  <si>
+    <t>2026-09-29 16:33:59</t>
   </si>
 </sst>
 </file>
@@ -4445,7 +4559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK187"/>
+  <dimension ref="A1:AK195"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -20269,7 +20383,7 @@
       <c r="M187" s="8"/>
       <c r="N187" s="7"/>
       <c r="O187" s="8"/>
-      <c r="P187" s="8"/>
+      <c r="P187" s="9"/>
       <c r="Q187" s="7" t="s">
         <v>1318</v>
       </c>
@@ -20302,7 +20416,7 @@
       <c r="AB187" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC187" s="8" t="s">
+      <c r="AC187" s="9" t="s">
         <v>67</v>
       </c>
       <c r="AD187" s="7" t="s">
@@ -20315,6 +20429,704 @@
       <c r="AI187" s="7"/>
       <c r="AJ187" s="7"/>
       <c r="AK187" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="188" spans="1:37">
+      <c r="A188" s="3">
+        <v>186</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C188" s="3">
+        <v>2026093417</v>
+      </c>
+      <c r="D188" s="3" t="s">
+        <v>1322</v>
+      </c>
+      <c r="E188" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F188" s="3">
+        <v>4698</v>
+      </c>
+      <c r="G188" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="H188" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I188" s="3" t="s">
+        <v>1323</v>
+      </c>
+      <c r="J188" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K188" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L188" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M188" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N188" s="3">
+        <v>2401</v>
+      </c>
+      <c r="O188" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="P188" s="10" t="s">
+        <v>1324</v>
+      </c>
+      <c r="Q188" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="R188" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S188" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T188" s="3">
+        <v>1</v>
+      </c>
+      <c r="U188" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V188" s="3" t="s">
+        <v>1325</v>
+      </c>
+      <c r="W188" s="3" t="s">
+        <v>1326</v>
+      </c>
+      <c r="X188" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="Y188" s="3" t="s">
+        <v>1328</v>
+      </c>
+      <c r="Z188" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA188" s="3"/>
+      <c r="AB188" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC188" s="10" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AD188" s="3"/>
+      <c r="AE188" s="3"/>
+      <c r="AF188" s="3"/>
+      <c r="AG188" s="3"/>
+      <c r="AH188" s="3"/>
+      <c r="AI188" s="3"/>
+      <c r="AJ188" s="3"/>
+      <c r="AK188" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="189" spans="1:37">
+      <c r="A189" s="7">
+        <v>187</v>
+      </c>
+      <c r="B189" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C189" s="7">
+        <v>2026093433</v>
+      </c>
+      <c r="D189" s="7" t="s">
+        <v>1330</v>
+      </c>
+      <c r="E189" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F189" s="7">
+        <v>2315</v>
+      </c>
+      <c r="G189" s="7" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H189" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I189" s="7" t="s">
+        <v>1331</v>
+      </c>
+      <c r="J189" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K189" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L189" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M189" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N189" s="7">
+        <v>2405</v>
+      </c>
+      <c r="O189" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="P189" s="9" t="s">
+        <v>1332</v>
+      </c>
+      <c r="Q189" s="7" t="s">
+        <v>1220</v>
+      </c>
+      <c r="R189" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S189" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T189" s="7">
+        <v>1</v>
+      </c>
+      <c r="U189" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V189" s="7" t="s">
+        <v>1333</v>
+      </c>
+      <c r="W189" s="7" t="s">
+        <v>1334</v>
+      </c>
+      <c r="X189" s="7" t="s">
+        <v>1335</v>
+      </c>
+      <c r="Y189" s="7" t="s">
+        <v>1336</v>
+      </c>
+      <c r="Z189" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="AA189" s="7"/>
+      <c r="AB189" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC189" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="AD189" s="7"/>
+      <c r="AE189" s="7"/>
+      <c r="AF189" s="7"/>
+      <c r="AG189" s="7"/>
+      <c r="AH189" s="7"/>
+      <c r="AI189" s="7"/>
+      <c r="AJ189" s="7"/>
+      <c r="AK189" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="190" spans="1:37">
+      <c r="A190" s="3">
+        <v>188</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C190" s="3">
+        <v>2026093516</v>
+      </c>
+      <c r="D190" s="3" t="s">
+        <v>1338</v>
+      </c>
+      <c r="E190" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F190" s="3">
+        <v>4456</v>
+      </c>
+      <c r="G190" s="3" t="s">
+        <v>1339</v>
+      </c>
+      <c r="H190" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I190" s="3" t="s">
+        <v>1340</v>
+      </c>
+      <c r="J190" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="K190" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L190" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M190" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N190" s="3">
+        <v>2403</v>
+      </c>
+      <c r="O190" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="P190" s="10" t="s">
+        <v>1341</v>
+      </c>
+      <c r="Q190" s="3" t="s">
+        <v>1342</v>
+      </c>
+      <c r="R190" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S190" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T190" s="3">
+        <v>1</v>
+      </c>
+      <c r="U190" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V190" s="3" t="s">
+        <v>1343</v>
+      </c>
+      <c r="W190" s="3" t="s">
+        <v>1344</v>
+      </c>
+      <c r="X190" s="3" t="s">
+        <v>1345</v>
+      </c>
+      <c r="Y190" s="3" t="s">
+        <v>1346</v>
+      </c>
+      <c r="Z190" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA190" s="3"/>
+      <c r="AB190" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC190" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD190" s="3"/>
+      <c r="AE190" s="3"/>
+      <c r="AF190" s="3"/>
+      <c r="AG190" s="3"/>
+      <c r="AH190" s="3"/>
+      <c r="AI190" s="3"/>
+      <c r="AJ190" s="3"/>
+      <c r="AK190" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="191" spans="1:37">
+      <c r="A191" s="7">
+        <v>189</v>
+      </c>
+      <c r="B191" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C191" s="7">
+        <v>2026093516</v>
+      </c>
+      <c r="D191" s="7" t="s">
+        <v>1338</v>
+      </c>
+      <c r="E191" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F191" s="7">
+        <v>4456</v>
+      </c>
+      <c r="G191" s="7" t="s">
+        <v>1339</v>
+      </c>
+      <c r="H191" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I191" s="7" t="s">
+        <v>1340</v>
+      </c>
+      <c r="J191" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K191" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L191" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M191" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N191" s="7">
+        <v>2403</v>
+      </c>
+      <c r="O191" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="P191" s="9" t="s">
+        <v>1341</v>
+      </c>
+      <c r="Q191" s="7" t="s">
+        <v>1342</v>
+      </c>
+      <c r="R191" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S191" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T191" s="7">
+        <v>2</v>
+      </c>
+      <c r="U191" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V191" s="7" t="s">
+        <v>1343</v>
+      </c>
+      <c r="W191" s="7" t="s">
+        <v>1344</v>
+      </c>
+      <c r="X191" s="7" t="s">
+        <v>1345</v>
+      </c>
+      <c r="Y191" s="7" t="s">
+        <v>1346</v>
+      </c>
+      <c r="Z191" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA191" s="7"/>
+      <c r="AB191" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC191" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD191" s="7"/>
+      <c r="AE191" s="7"/>
+      <c r="AF191" s="7"/>
+      <c r="AG191" s="7"/>
+      <c r="AH191" s="7"/>
+      <c r="AI191" s="7"/>
+      <c r="AJ191" s="7"/>
+      <c r="AK191" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="192" spans="1:37">
+      <c r="A192" s="3">
+        <v>190</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C192" s="3">
+        <v>2026093520</v>
+      </c>
+      <c r="D192" s="3"/>
+      <c r="E192" s="3"/>
+      <c r="F192" s="3">
+        <v>4456</v>
+      </c>
+      <c r="G192" s="3" t="s">
+        <v>1339</v>
+      </c>
+      <c r="H192" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I192" s="3"/>
+      <c r="J192" s="3"/>
+      <c r="K192" s="3"/>
+      <c r="L192" s="3"/>
+      <c r="M192" s="4"/>
+      <c r="N192" s="3"/>
+      <c r="O192" s="4"/>
+      <c r="P192" s="10"/>
+      <c r="Q192" s="3" t="s">
+        <v>1342</v>
+      </c>
+      <c r="R192" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S192" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T192" s="3">
+        <v>1</v>
+      </c>
+      <c r="U192" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V192" s="3" t="s">
+        <v>1347</v>
+      </c>
+      <c r="W192" s="3" t="s">
+        <v>1348</v>
+      </c>
+      <c r="X192" s="3" t="s">
+        <v>1349</v>
+      </c>
+      <c r="Y192" s="3"/>
+      <c r="Z192" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="AA192" s="3"/>
+      <c r="AB192" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC192" s="10" t="s">
+        <v>1350</v>
+      </c>
+      <c r="AD192" s="3"/>
+      <c r="AE192" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF192" s="3"/>
+      <c r="AG192" s="3"/>
+      <c r="AH192" s="3"/>
+      <c r="AI192" s="3"/>
+      <c r="AJ192" s="3"/>
+      <c r="AK192" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="193" spans="1:37">
+      <c r="A193" s="7">
+        <v>191</v>
+      </c>
+      <c r="B193" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C193" s="7">
+        <v>2026093521</v>
+      </c>
+      <c r="D193" s="7"/>
+      <c r="E193" s="7"/>
+      <c r="F193" s="7">
+        <v>4456</v>
+      </c>
+      <c r="G193" s="7" t="s">
+        <v>1339</v>
+      </c>
+      <c r="H193" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I193" s="7"/>
+      <c r="J193" s="7"/>
+      <c r="K193" s="7"/>
+      <c r="L193" s="7"/>
+      <c r="M193" s="8"/>
+      <c r="N193" s="7"/>
+      <c r="O193" s="8"/>
+      <c r="P193" s="9"/>
+      <c r="Q193" s="7" t="s">
+        <v>1342</v>
+      </c>
+      <c r="R193" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S193" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T193" s="7">
+        <v>1</v>
+      </c>
+      <c r="U193" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V193" s="7" t="s">
+        <v>1351</v>
+      </c>
+      <c r="W193" s="7" t="s">
+        <v>1348</v>
+      </c>
+      <c r="X193" s="7" t="s">
+        <v>1344</v>
+      </c>
+      <c r="Y193" s="7"/>
+      <c r="Z193" s="7">
+        <v>5</v>
+      </c>
+      <c r="AA193" s="7"/>
+      <c r="AB193" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC193" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="AD193" s="7"/>
+      <c r="AE193" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF193" s="7"/>
+      <c r="AG193" s="7"/>
+      <c r="AH193" s="7"/>
+      <c r="AI193" s="7"/>
+      <c r="AJ193" s="7"/>
+      <c r="AK193" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="194" spans="1:37">
+      <c r="A194" s="3">
+        <v>192</v>
+      </c>
+      <c r="B194" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C194" s="3">
+        <v>2026093523</v>
+      </c>
+      <c r="D194" s="3"/>
+      <c r="E194" s="3"/>
+      <c r="F194" s="3" t="s">
+        <v>1352</v>
+      </c>
+      <c r="G194" s="3" t="s">
+        <v>1353</v>
+      </c>
+      <c r="H194" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I194" s="3"/>
+      <c r="J194" s="3"/>
+      <c r="K194" s="3"/>
+      <c r="L194" s="3"/>
+      <c r="M194" s="4"/>
+      <c r="N194" s="3"/>
+      <c r="O194" s="4"/>
+      <c r="P194" s="10"/>
+      <c r="Q194" s="3" t="s">
+        <v>1354</v>
+      </c>
+      <c r="R194" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S194" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T194" s="3">
+        <v>1</v>
+      </c>
+      <c r="U194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V194" s="3" t="s">
+        <v>1355</v>
+      </c>
+      <c r="W194" s="3" t="s">
+        <v>1356</v>
+      </c>
+      <c r="X194" s="3" t="s">
+        <v>1357</v>
+      </c>
+      <c r="Y194" s="3"/>
+      <c r="Z194" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA194" s="3"/>
+      <c r="AB194" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC194" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD194" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE194" s="3"/>
+      <c r="AF194" s="3"/>
+      <c r="AG194" s="3"/>
+      <c r="AH194" s="3"/>
+      <c r="AI194" s="3"/>
+      <c r="AJ194" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK194" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="195" spans="1:37">
+      <c r="A195" s="7">
+        <v>193</v>
+      </c>
+      <c r="B195" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C195" s="7">
+        <v>2026093524</v>
+      </c>
+      <c r="D195" s="7"/>
+      <c r="E195" s="7"/>
+      <c r="F195" s="7" t="s">
+        <v>1352</v>
+      </c>
+      <c r="G195" s="7" t="s">
+        <v>1353</v>
+      </c>
+      <c r="H195" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I195" s="7"/>
+      <c r="J195" s="7"/>
+      <c r="K195" s="7"/>
+      <c r="L195" s="7"/>
+      <c r="M195" s="8"/>
+      <c r="N195" s="7"/>
+      <c r="O195" s="8"/>
+      <c r="P195" s="8"/>
+      <c r="Q195" s="7" t="s">
+        <v>1354</v>
+      </c>
+      <c r="R195" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S195" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T195" s="7">
+        <v>1</v>
+      </c>
+      <c r="U195" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V195" s="7" t="s">
+        <v>1358</v>
+      </c>
+      <c r="W195" s="7" t="s">
+        <v>1348</v>
+      </c>
+      <c r="X195" s="7" t="s">
+        <v>1344</v>
+      </c>
+      <c r="Y195" s="7"/>
+      <c r="Z195" s="7">
+        <v>5</v>
+      </c>
+      <c r="AA195" s="7"/>
+      <c r="AB195" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC195" s="8" t="s">
+        <v>520</v>
+      </c>
+      <c r="AD195" s="7"/>
+      <c r="AE195" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF195" s="7"/>
+      <c r="AG195" s="7"/>
+      <c r="AH195" s="7"/>
+      <c r="AI195" s="7"/>
+      <c r="AJ195" s="7"/>
+      <c r="AK195" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09301523
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$195</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$203</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1359">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-29  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1393">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-30  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -4146,6 +4146,108 @@
   </si>
   <si>
     <t>2026-09-29 16:33:59</t>
+  </si>
+  <si>
+    <t>12596115093001</t>
+  </si>
+  <si>
+    <t>2026-09-30 11:13:39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台芝先生告知今日回裝發現SC滑鼠故障，需更換，請客服協助派工	</t>
+  </si>
+  <si>
+    <t>2026-09-30 11:14:34</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:40:00</t>
+  </si>
+  <si>
+    <t>2026-10-01 15:14:00</t>
+  </si>
+  <si>
+    <t>新北市民廣場</t>
+  </si>
+  <si>
+    <t>THILF05496</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:02:04</t>
+  </si>
+  <si>
+    <t>2026-09-30 12:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:00:00</t>
+  </si>
+  <si>
+    <t>板橋板億店</t>
+  </si>
+  <si>
+    <t>THILF02422</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:34:24</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:10:00</t>
+  </si>
+  <si>
+    <t>C894</t>
+  </si>
+  <si>
+    <t>中和遠東店</t>
+  </si>
+  <si>
+    <t>THILF0C894</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:47:58</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:22:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:50:25</t>
+  </si>
+  <si>
+    <t>2026-09-30 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:54:15</t>
+  </si>
+  <si>
+    <t>2026-09-30 14:04:45</t>
+  </si>
+  <si>
+    <t>13965115093001</t>
+  </si>
+  <si>
+    <t>2026-09-30 14:19:48</t>
+  </si>
+  <si>
+    <t>2026-09-30 14:21:28</t>
+  </si>
+  <si>
+    <t>2026-09-30 13:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-30 14:21:00</t>
+  </si>
+  <si>
+    <t>2026-10-01 18:21:00</t>
+  </si>
+  <si>
+    <t>+HUB重設後0800測試正常</t>
   </si>
 </sst>
 </file>
@@ -4559,7 +4661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK195"/>
+  <dimension ref="A1:AK203"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -21081,7 +21183,7 @@
       <c r="M195" s="8"/>
       <c r="N195" s="7"/>
       <c r="O195" s="8"/>
-      <c r="P195" s="8"/>
+      <c r="P195" s="9"/>
       <c r="Q195" s="7" t="s">
         <v>1354</v>
       </c>
@@ -21114,7 +21216,7 @@
       <c r="AB195" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC195" s="8" t="s">
+      <c r="AC195" s="9" t="s">
         <v>520</v>
       </c>
       <c r="AD195" s="7"/>
@@ -21127,6 +21229,664 @@
       <c r="AI195" s="7"/>
       <c r="AJ195" s="7"/>
       <c r="AK195" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="196" spans="1:37">
+      <c r="A196" s="3">
+        <v>194</v>
+      </c>
+      <c r="B196" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C196" s="3">
+        <v>2026093584</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>1359</v>
+      </c>
+      <c r="E196" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F196" s="3">
+        <v>2596</v>
+      </c>
+      <c r="G196" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H196" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I196" s="3" t="s">
+        <v>1360</v>
+      </c>
+      <c r="J196" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K196" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L196" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M196" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N196" s="3">
+        <v>2403</v>
+      </c>
+      <c r="O196" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="P196" s="10" t="s">
+        <v>1361</v>
+      </c>
+      <c r="Q196" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="R196" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S196" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T196" s="3">
+        <v>1</v>
+      </c>
+      <c r="U196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V196" s="3" t="s">
+        <v>1362</v>
+      </c>
+      <c r="W196" s="3" t="s">
+        <v>1363</v>
+      </c>
+      <c r="X196" s="3" t="s">
+        <v>1364</v>
+      </c>
+      <c r="Y196" s="3" t="s">
+        <v>1365</v>
+      </c>
+      <c r="Z196" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA196" s="3"/>
+      <c r="AB196" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC196" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD196" s="3"/>
+      <c r="AE196" s="3"/>
+      <c r="AF196" s="3"/>
+      <c r="AG196" s="3"/>
+      <c r="AH196" s="3"/>
+      <c r="AI196" s="3"/>
+      <c r="AJ196" s="3"/>
+      <c r="AK196" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="197" spans="1:37">
+      <c r="A197" s="7">
+        <v>195</v>
+      </c>
+      <c r="B197" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C197" s="7">
+        <v>2026093621</v>
+      </c>
+      <c r="D197" s="7"/>
+      <c r="E197" s="7"/>
+      <c r="F197" s="7">
+        <v>5496</v>
+      </c>
+      <c r="G197" s="7" t="s">
+        <v>1366</v>
+      </c>
+      <c r="H197" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I197" s="7"/>
+      <c r="J197" s="7"/>
+      <c r="K197" s="7"/>
+      <c r="L197" s="7"/>
+      <c r="M197" s="8"/>
+      <c r="N197" s="7"/>
+      <c r="O197" s="8"/>
+      <c r="P197" s="9"/>
+      <c r="Q197" s="7" t="s">
+        <v>1367</v>
+      </c>
+      <c r="R197" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S197" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T197" s="7">
+        <v>1</v>
+      </c>
+      <c r="U197" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V197" s="7" t="s">
+        <v>1368</v>
+      </c>
+      <c r="W197" s="7" t="s">
+        <v>1369</v>
+      </c>
+      <c r="X197" s="7" t="s">
+        <v>1370</v>
+      </c>
+      <c r="Y197" s="7"/>
+      <c r="Z197" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA197" s="7"/>
+      <c r="AB197" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC197" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD197" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE197" s="7"/>
+      <c r="AF197" s="7"/>
+      <c r="AG197" s="7"/>
+      <c r="AH197" s="7"/>
+      <c r="AI197" s="7"/>
+      <c r="AJ197" s="7"/>
+      <c r="AK197" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="198" spans="1:37">
+      <c r="A198" s="3">
+        <v>196</v>
+      </c>
+      <c r="B198" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C198" s="3">
+        <v>2026093622</v>
+      </c>
+      <c r="D198" s="3"/>
+      <c r="E198" s="3"/>
+      <c r="F198" s="3">
+        <v>2422</v>
+      </c>
+      <c r="G198" s="3" t="s">
+        <v>1371</v>
+      </c>
+      <c r="H198" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I198" s="3"/>
+      <c r="J198" s="3"/>
+      <c r="K198" s="3"/>
+      <c r="L198" s="3"/>
+      <c r="M198" s="4"/>
+      <c r="N198" s="3"/>
+      <c r="O198" s="4"/>
+      <c r="P198" s="10"/>
+      <c r="Q198" s="3" t="s">
+        <v>1372</v>
+      </c>
+      <c r="R198" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S198" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T198" s="3">
+        <v>1</v>
+      </c>
+      <c r="U198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V198" s="3" t="s">
+        <v>1373</v>
+      </c>
+      <c r="W198" s="3" t="s">
+        <v>1374</v>
+      </c>
+      <c r="X198" s="3" t="s">
+        <v>1363</v>
+      </c>
+      <c r="Y198" s="3"/>
+      <c r="Z198" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA198" s="3"/>
+      <c r="AB198" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC198" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD198" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE198" s="3"/>
+      <c r="AF198" s="3"/>
+      <c r="AG198" s="3"/>
+      <c r="AH198" s="3"/>
+      <c r="AI198" s="3"/>
+      <c r="AJ198" s="3"/>
+      <c r="AK198" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="199" spans="1:37">
+      <c r="A199" s="7">
+        <v>197</v>
+      </c>
+      <c r="B199" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C199" s="7">
+        <v>2026093624</v>
+      </c>
+      <c r="D199" s="7"/>
+      <c r="E199" s="7"/>
+      <c r="F199" s="7" t="s">
+        <v>1375</v>
+      </c>
+      <c r="G199" s="7" t="s">
+        <v>1376</v>
+      </c>
+      <c r="H199" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I199" s="7"/>
+      <c r="J199" s="7"/>
+      <c r="K199" s="7"/>
+      <c r="L199" s="7"/>
+      <c r="M199" s="8"/>
+      <c r="N199" s="7"/>
+      <c r="O199" s="8"/>
+      <c r="P199" s="9"/>
+      <c r="Q199" s="7" t="s">
+        <v>1377</v>
+      </c>
+      <c r="R199" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S199" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T199" s="7">
+        <v>1</v>
+      </c>
+      <c r="U199" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V199" s="7" t="s">
+        <v>1378</v>
+      </c>
+      <c r="W199" s="7" t="s">
+        <v>1379</v>
+      </c>
+      <c r="X199" s="7" t="s">
+        <v>1380</v>
+      </c>
+      <c r="Y199" s="7"/>
+      <c r="Z199" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA199" s="7"/>
+      <c r="AB199" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC199" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD199" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE199" s="7"/>
+      <c r="AF199" s="7"/>
+      <c r="AG199" s="7"/>
+      <c r="AH199" s="7"/>
+      <c r="AI199" s="7"/>
+      <c r="AJ199" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK199" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="200" spans="1:37">
+      <c r="A200" s="3">
+        <v>198</v>
+      </c>
+      <c r="B200" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C200" s="3">
+        <v>2026093680</v>
+      </c>
+      <c r="D200" s="3"/>
+      <c r="E200" s="3"/>
+      <c r="F200" s="3">
+        <v>2596</v>
+      </c>
+      <c r="G200" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H200" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I200" s="3"/>
+      <c r="J200" s="3"/>
+      <c r="K200" s="3"/>
+      <c r="L200" s="3"/>
+      <c r="M200" s="4"/>
+      <c r="N200" s="3"/>
+      <c r="O200" s="4"/>
+      <c r="P200" s="10"/>
+      <c r="Q200" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="R200" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S200" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T200" s="3">
+        <v>1</v>
+      </c>
+      <c r="U200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V200" s="3" t="s">
+        <v>1381</v>
+      </c>
+      <c r="W200" s="3" t="s">
+        <v>1382</v>
+      </c>
+      <c r="X200" s="3" t="s">
+        <v>1383</v>
+      </c>
+      <c r="Y200" s="3"/>
+      <c r="Z200" s="3">
+        <v>4</v>
+      </c>
+      <c r="AA200" s="3"/>
+      <c r="AB200" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC200" s="10" t="s">
+        <v>520</v>
+      </c>
+      <c r="AD200" s="3"/>
+      <c r="AE200" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF200" s="3"/>
+      <c r="AG200" s="3"/>
+      <c r="AH200" s="3"/>
+      <c r="AI200" s="3"/>
+      <c r="AJ200" s="3"/>
+      <c r="AK200" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="201" spans="1:37">
+      <c r="A201" s="7">
+        <v>199</v>
+      </c>
+      <c r="B201" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C201" s="7">
+        <v>2026093681</v>
+      </c>
+      <c r="D201" s="7"/>
+      <c r="E201" s="7"/>
+      <c r="F201" s="7">
+        <v>2596</v>
+      </c>
+      <c r="G201" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H201" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I201" s="7"/>
+      <c r="J201" s="7"/>
+      <c r="K201" s="7"/>
+      <c r="L201" s="7"/>
+      <c r="M201" s="8"/>
+      <c r="N201" s="7"/>
+      <c r="O201" s="8"/>
+      <c r="P201" s="9"/>
+      <c r="Q201" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="R201" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S201" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T201" s="7">
+        <v>1</v>
+      </c>
+      <c r="U201" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V201" s="7" t="s">
+        <v>1384</v>
+      </c>
+      <c r="W201" s="7" t="s">
+        <v>1382</v>
+      </c>
+      <c r="X201" s="7" t="s">
+        <v>1383</v>
+      </c>
+      <c r="Y201" s="7"/>
+      <c r="Z201" s="7">
+        <v>4</v>
+      </c>
+      <c r="AA201" s="7"/>
+      <c r="AB201" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC201" s="9" t="s">
+        <v>1350</v>
+      </c>
+      <c r="AD201" s="7"/>
+      <c r="AE201" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF201" s="7"/>
+      <c r="AG201" s="7"/>
+      <c r="AH201" s="7"/>
+      <c r="AI201" s="7"/>
+      <c r="AJ201" s="7"/>
+      <c r="AK201" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="202" spans="1:37">
+      <c r="A202" s="3">
+        <v>200</v>
+      </c>
+      <c r="B202" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C202" s="3">
+        <v>2026093686</v>
+      </c>
+      <c r="D202" s="3"/>
+      <c r="E202" s="3"/>
+      <c r="F202" s="3">
+        <v>2596</v>
+      </c>
+      <c r="G202" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H202" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I202" s="3"/>
+      <c r="J202" s="3"/>
+      <c r="K202" s="3"/>
+      <c r="L202" s="3"/>
+      <c r="M202" s="4"/>
+      <c r="N202" s="3"/>
+      <c r="O202" s="4"/>
+      <c r="P202" s="10"/>
+      <c r="Q202" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="R202" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S202" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T202" s="3">
+        <v>1</v>
+      </c>
+      <c r="U202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V202" s="3" t="s">
+        <v>1385</v>
+      </c>
+      <c r="W202" s="3" t="s">
+        <v>1364</v>
+      </c>
+      <c r="X202" s="3" t="s">
+        <v>1383</v>
+      </c>
+      <c r="Y202" s="3"/>
+      <c r="Z202" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA202" s="3"/>
+      <c r="AB202" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC202" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD202" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE202" s="3"/>
+      <c r="AF202" s="3"/>
+      <c r="AG202" s="3"/>
+      <c r="AH202" s="3"/>
+      <c r="AI202" s="3"/>
+      <c r="AJ202" s="3"/>
+      <c r="AK202" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="203" spans="1:37">
+      <c r="A203" s="7">
+        <v>201</v>
+      </c>
+      <c r="B203" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C203" s="7">
+        <v>2026093688</v>
+      </c>
+      <c r="D203" s="7" t="s">
+        <v>1386</v>
+      </c>
+      <c r="E203" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F203" s="7">
+        <v>3965</v>
+      </c>
+      <c r="G203" s="7" t="s">
+        <v>1270</v>
+      </c>
+      <c r="H203" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I203" s="7" t="s">
+        <v>1387</v>
+      </c>
+      <c r="J203" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K203" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L203" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="M203" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="N203" s="7">
+        <v>3404</v>
+      </c>
+      <c r="O203" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="P203" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="Q203" s="7" t="s">
+        <v>1271</v>
+      </c>
+      <c r="R203" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S203" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T203" s="7">
+        <v>1</v>
+      </c>
+      <c r="U203" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V203" s="7" t="s">
+        <v>1388</v>
+      </c>
+      <c r="W203" s="7" t="s">
+        <v>1389</v>
+      </c>
+      <c r="X203" s="7" t="s">
+        <v>1390</v>
+      </c>
+      <c r="Y203" s="7" t="s">
+        <v>1391</v>
+      </c>
+      <c r="Z203" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA203" s="7"/>
+      <c r="AB203" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC203" s="8" t="s">
+        <v>1392</v>
+      </c>
+      <c r="AD203" s="7"/>
+      <c r="AE203" s="7"/>
+      <c r="AF203" s="7"/>
+      <c r="AG203" s="7"/>
+      <c r="AH203" s="7"/>
+      <c r="AI203" s="7"/>
+      <c r="AJ203" s="7"/>
+      <c r="AK203" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>